<commit_message>
Update job tracker 2026-08-29 13:18 UTC
</commit_message>
<xml_diff>
--- a/data/job_matches.xlsx
+++ b/data/job_matches.xlsx
@@ -68,14 +68,14 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFF2CC"/>
-        <bgColor rgb="00FFF2CC"/>
+        <fgColor rgb="00FFC7CE"/>
+        <bgColor rgb="00FFC7CE"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFC7CE"/>
-        <bgColor rgb="00FFC7CE"/>
+        <fgColor rgb="00FFF2CC"/>
+        <bgColor rgb="00FFF2CC"/>
       </patternFill>
     </fill>
     <fill>
@@ -131,10 +131,10 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -517,7 +517,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M186"/>
+  <dimension ref="A1:M188"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -775,9 +775,9 @@
           <t>Not stated in JD</t>
         </is>
       </c>
-      <c r="K4" s="7" t="inlineStr">
-        <is>
-          <t>New this run (2026-08-28 22:31 UTC)</t>
+      <c r="K4" s="2" t="inlineStr">
+        <is>
+          <t>From previous run</t>
         </is>
       </c>
       <c r="L4" s="2" t="inlineStr">
@@ -1090,9 +1090,9 @@
           <t>Not stated in JD</t>
         </is>
       </c>
-      <c r="K9" s="7" t="inlineStr">
-        <is>
-          <t>New this run (2026-08-28 22:31 UTC)</t>
+      <c r="K9" s="2" t="inlineStr">
+        <is>
+          <t>From previous run</t>
         </is>
       </c>
       <c r="L9" s="2" t="inlineStr">
@@ -1886,10 +1886,10 @@
           <t>2026-08-26</t>
         </is>
       </c>
-      <c r="F22" s="8" t="n">
+      <c r="F22" s="7" t="n">
         <v>68</v>
       </c>
-      <c r="G22" s="9" t="inlineStr">
+      <c r="G22" s="8" t="inlineStr">
         <is>
           <t>Below threshold</t>
         </is>
@@ -1949,10 +1949,10 @@
           <t>2026-08-26</t>
         </is>
       </c>
-      <c r="F23" s="8" t="n">
+      <c r="F23" s="7" t="n">
         <v>68</v>
       </c>
-      <c r="G23" s="9" t="inlineStr">
+      <c r="G23" s="8" t="inlineStr">
         <is>
           <t>Below threshold</t>
         </is>
@@ -2012,10 +2012,10 @@
           <t>2026-08-26</t>
         </is>
       </c>
-      <c r="F24" s="8" t="n">
+      <c r="F24" s="7" t="n">
         <v>68</v>
       </c>
-      <c r="G24" s="9" t="inlineStr">
+      <c r="G24" s="8" t="inlineStr">
         <is>
           <t>Below threshold</t>
         </is>
@@ -2075,10 +2075,10 @@
           <t>2026-08-26</t>
         </is>
       </c>
-      <c r="F25" s="8" t="n">
+      <c r="F25" s="7" t="n">
         <v>68</v>
       </c>
-      <c r="G25" s="9" t="inlineStr">
+      <c r="G25" s="8" t="inlineStr">
         <is>
           <t>Below threshold</t>
         </is>
@@ -2138,10 +2138,10 @@
           <t>2026-08-27</t>
         </is>
       </c>
-      <c r="F26" s="8" t="n">
+      <c r="F26" s="7" t="n">
         <v>68</v>
       </c>
-      <c r="G26" s="9" t="inlineStr">
+      <c r="G26" s="8" t="inlineStr">
         <is>
           <t>Below threshold</t>
         </is>
@@ -2201,10 +2201,10 @@
           <t>2026-08-27</t>
         </is>
       </c>
-      <c r="F27" s="8" t="n">
+      <c r="F27" s="7" t="n">
         <v>68</v>
       </c>
-      <c r="G27" s="9" t="inlineStr">
+      <c r="G27" s="8" t="inlineStr">
         <is>
           <t>Below threshold</t>
         </is>
@@ -2264,10 +2264,10 @@
           <t>2026-08-27</t>
         </is>
       </c>
-      <c r="F28" s="8" t="n">
+      <c r="F28" s="7" t="n">
         <v>68</v>
       </c>
-      <c r="G28" s="9" t="inlineStr">
+      <c r="G28" s="8" t="inlineStr">
         <is>
           <t>Below threshold</t>
         </is>
@@ -2327,10 +2327,10 @@
           <t>2026-08-27</t>
         </is>
       </c>
-      <c r="F29" s="8" t="n">
+      <c r="F29" s="7" t="n">
         <v>68</v>
       </c>
-      <c r="G29" s="9" t="inlineStr">
+      <c r="G29" s="8" t="inlineStr">
         <is>
           <t>Below threshold</t>
         </is>
@@ -2390,10 +2390,10 @@
           <t>2026-08-27</t>
         </is>
       </c>
-      <c r="F30" s="8" t="n">
+      <c r="F30" s="7" t="n">
         <v>68</v>
       </c>
-      <c r="G30" s="9" t="inlineStr">
+      <c r="G30" s="8" t="inlineStr">
         <is>
           <t>Below threshold</t>
         </is>
@@ -2453,10 +2453,10 @@
           <t>2026-08-26</t>
         </is>
       </c>
-      <c r="F31" s="8" t="n">
+      <c r="F31" s="7" t="n">
         <v>65</v>
       </c>
-      <c r="G31" s="9" t="inlineStr">
+      <c r="G31" s="8" t="inlineStr">
         <is>
           <t>Below threshold</t>
         </is>
@@ -2516,10 +2516,10 @@
           <t>2026-08-26</t>
         </is>
       </c>
-      <c r="F32" s="8" t="n">
+      <c r="F32" s="7" t="n">
         <v>65</v>
       </c>
-      <c r="G32" s="9" t="inlineStr">
+      <c r="G32" s="8" t="inlineStr">
         <is>
           <t>Below threshold</t>
         </is>
@@ -2579,10 +2579,10 @@
           <t>2026-08-27</t>
         </is>
       </c>
-      <c r="F33" s="8" t="n">
+      <c r="F33" s="7" t="n">
         <v>65</v>
       </c>
-      <c r="G33" s="9" t="inlineStr">
+      <c r="G33" s="8" t="inlineStr">
         <is>
           <t>Below threshold</t>
         </is>
@@ -2642,10 +2642,10 @@
           <t>2026-08-28</t>
         </is>
       </c>
-      <c r="F34" s="8" t="n">
+      <c r="F34" s="7" t="n">
         <v>65</v>
       </c>
-      <c r="G34" s="9" t="inlineStr">
+      <c r="G34" s="8" t="inlineStr">
         <is>
           <t>Below threshold</t>
         </is>
@@ -2705,10 +2705,10 @@
           <t>2026-08-26</t>
         </is>
       </c>
-      <c r="F35" s="8" t="n">
+      <c r="F35" s="7" t="n">
         <v>60</v>
       </c>
-      <c r="G35" s="9" t="inlineStr">
+      <c r="G35" s="8" t="inlineStr">
         <is>
           <t>Below threshold</t>
         </is>
@@ -2768,10 +2768,10 @@
           <t>2026-08-26</t>
         </is>
       </c>
-      <c r="F36" s="8" t="n">
+      <c r="F36" s="7" t="n">
         <v>60</v>
       </c>
-      <c r="G36" s="9" t="inlineStr">
+      <c r="G36" s="8" t="inlineStr">
         <is>
           <t>Below threshold</t>
         </is>
@@ -2831,10 +2831,10 @@
           <t>2026-08-27</t>
         </is>
       </c>
-      <c r="F37" s="8" t="n">
+      <c r="F37" s="7" t="n">
         <v>60</v>
       </c>
-      <c r="G37" s="9" t="inlineStr">
+      <c r="G37" s="8" t="inlineStr">
         <is>
           <t>Below threshold</t>
         </is>
@@ -2894,10 +2894,10 @@
           <t>2026-08-26</t>
         </is>
       </c>
-      <c r="F38" s="8" t="n">
+      <c r="F38" s="7" t="n">
         <v>45</v>
       </c>
-      <c r="G38" s="9" t="inlineStr">
+      <c r="G38" s="8" t="inlineStr">
         <is>
           <t>Below threshold</t>
         </is>
@@ -2957,10 +2957,10 @@
           <t>2026-08-26</t>
         </is>
       </c>
-      <c r="F39" s="8" t="n">
+      <c r="F39" s="7" t="n">
         <v>45</v>
       </c>
-      <c r="G39" s="9" t="inlineStr">
+      <c r="G39" s="8" t="inlineStr">
         <is>
           <t>Below threshold</t>
         </is>
@@ -3020,10 +3020,10 @@
           <t>2026-08-27</t>
         </is>
       </c>
-      <c r="F40" s="8" t="n">
+      <c r="F40" s="7" t="n">
         <v>45</v>
       </c>
-      <c r="G40" s="9" t="inlineStr">
+      <c r="G40" s="8" t="inlineStr">
         <is>
           <t>Below threshold</t>
         </is>
@@ -3083,10 +3083,10 @@
           <t>2026-08-26</t>
         </is>
       </c>
-      <c r="F41" s="8" t="n">
+      <c r="F41" s="7" t="n">
         <v>45</v>
       </c>
-      <c r="G41" s="9" t="inlineStr">
+      <c r="G41" s="8" t="inlineStr">
         <is>
           <t>Below threshold</t>
         </is>
@@ -3146,10 +3146,10 @@
           <t>2026-08-26</t>
         </is>
       </c>
-      <c r="F42" s="8" t="n">
+      <c r="F42" s="7" t="n">
         <v>45</v>
       </c>
-      <c r="G42" s="9" t="inlineStr">
+      <c r="G42" s="8" t="inlineStr">
         <is>
           <t>Below threshold</t>
         </is>
@@ -3209,10 +3209,10 @@
           <t>2026-08-27</t>
         </is>
       </c>
-      <c r="F43" s="8" t="n">
+      <c r="F43" s="7" t="n">
         <v>45</v>
       </c>
-      <c r="G43" s="9" t="inlineStr">
+      <c r="G43" s="8" t="inlineStr">
         <is>
           <t>Below threshold</t>
         </is>
@@ -3272,10 +3272,10 @@
           <t>2026-08-26</t>
         </is>
       </c>
-      <c r="F44" s="8" t="n">
+      <c r="F44" s="7" t="n">
         <v>45</v>
       </c>
-      <c r="G44" s="9" t="inlineStr">
+      <c r="G44" s="8" t="inlineStr">
         <is>
           <t>Below threshold</t>
         </is>
@@ -3335,10 +3335,10 @@
           <t>2026-08-28</t>
         </is>
       </c>
-      <c r="F45" s="8" t="n">
+      <c r="F45" s="7" t="n">
         <v>45</v>
       </c>
-      <c r="G45" s="9" t="inlineStr">
+      <c r="G45" s="8" t="inlineStr">
         <is>
           <t>Below threshold</t>
         </is>
@@ -3358,9 +3358,9 @@
           <t>Not stated in JD</t>
         </is>
       </c>
-      <c r="K45" s="7" t="inlineStr">
-        <is>
-          <t>New this run (2026-08-28 22:31 UTC)</t>
+      <c r="K45" s="2" t="inlineStr">
+        <is>
+          <t>From previous run</t>
         </is>
       </c>
       <c r="L45" s="2" t="inlineStr">
@@ -3398,10 +3398,10 @@
           <t>2026-08-26</t>
         </is>
       </c>
-      <c r="F46" s="8" t="n">
+      <c r="F46" s="7" t="n">
         <v>42</v>
       </c>
-      <c r="G46" s="9" t="inlineStr">
+      <c r="G46" s="8" t="inlineStr">
         <is>
           <t>Below threshold</t>
         </is>
@@ -3461,10 +3461,10 @@
           <t>2026-08-27</t>
         </is>
       </c>
-      <c r="F47" s="8" t="n">
+      <c r="F47" s="7" t="n">
         <v>40</v>
       </c>
-      <c r="G47" s="9" t="inlineStr">
+      <c r="G47" s="8" t="inlineStr">
         <is>
           <t>Below threshold</t>
         </is>
@@ -3524,10 +3524,10 @@
           <t>2026-08-26</t>
         </is>
       </c>
-      <c r="F48" s="8" t="n">
+      <c r="F48" s="7" t="n">
         <v>40</v>
       </c>
-      <c r="G48" s="9" t="inlineStr">
+      <c r="G48" s="8" t="inlineStr">
         <is>
           <t>Below threshold</t>
         </is>
@@ -3587,10 +3587,10 @@
           <t>2026-08-26</t>
         </is>
       </c>
-      <c r="F49" s="8" t="n">
+      <c r="F49" s="7" t="n">
         <v>40</v>
       </c>
-      <c r="G49" s="9" t="inlineStr">
+      <c r="G49" s="8" t="inlineStr">
         <is>
           <t>Below threshold</t>
         </is>
@@ -3650,10 +3650,10 @@
           <t>2026-08-27</t>
         </is>
       </c>
-      <c r="F50" s="8" t="n">
+      <c r="F50" s="7" t="n">
         <v>40</v>
       </c>
-      <c r="G50" s="9" t="inlineStr">
+      <c r="G50" s="8" t="inlineStr">
         <is>
           <t>Below threshold</t>
         </is>
@@ -3713,10 +3713,10 @@
           <t>2026-08-27</t>
         </is>
       </c>
-      <c r="F51" s="8" t="n">
+      <c r="F51" s="7" t="n">
         <v>38</v>
       </c>
-      <c r="G51" s="9" t="inlineStr">
+      <c r="G51" s="8" t="inlineStr">
         <is>
           <t>Below threshold</t>
         </is>
@@ -3776,10 +3776,10 @@
           <t>2026-08-27</t>
         </is>
       </c>
-      <c r="F52" s="8" t="n">
+      <c r="F52" s="7" t="n">
         <v>35</v>
       </c>
-      <c r="G52" s="9" t="inlineStr">
+      <c r="G52" s="8" t="inlineStr">
         <is>
           <t>Below threshold</t>
         </is>
@@ -3839,10 +3839,10 @@
           <t>2026-08-26</t>
         </is>
       </c>
-      <c r="F53" s="8" t="n">
+      <c r="F53" s="7" t="n">
         <v>35</v>
       </c>
-      <c r="G53" s="9" t="inlineStr">
+      <c r="G53" s="8" t="inlineStr">
         <is>
           <t>Below threshold</t>
         </is>
@@ -3902,10 +3902,10 @@
           <t>2026-08-26</t>
         </is>
       </c>
-      <c r="F54" s="8" t="n">
+      <c r="F54" s="7" t="n">
         <v>35</v>
       </c>
-      <c r="G54" s="9" t="inlineStr">
+      <c r="G54" s="8" t="inlineStr">
         <is>
           <t>Below threshold</t>
         </is>
@@ -3965,10 +3965,10 @@
           <t>2026-08-26</t>
         </is>
       </c>
-      <c r="F55" s="8" t="n">
+      <c r="F55" s="7" t="n">
         <v>35</v>
       </c>
-      <c r="G55" s="9" t="inlineStr">
+      <c r="G55" s="8" t="inlineStr">
         <is>
           <t>Below threshold</t>
         </is>
@@ -4028,10 +4028,10 @@
           <t>2026-08-26</t>
         </is>
       </c>
-      <c r="F56" s="8" t="n">
+      <c r="F56" s="7" t="n">
         <v>35</v>
       </c>
-      <c r="G56" s="9" t="inlineStr">
+      <c r="G56" s="8" t="inlineStr">
         <is>
           <t>Below threshold</t>
         </is>
@@ -4091,10 +4091,10 @@
           <t>2026-08-26</t>
         </is>
       </c>
-      <c r="F57" s="8" t="n">
+      <c r="F57" s="7" t="n">
         <v>35</v>
       </c>
-      <c r="G57" s="9" t="inlineStr">
+      <c r="G57" s="8" t="inlineStr">
         <is>
           <t>Below threshold</t>
         </is>
@@ -4154,10 +4154,10 @@
           <t>2026-08-26</t>
         </is>
       </c>
-      <c r="F58" s="8" t="n">
+      <c r="F58" s="7" t="n">
         <v>35</v>
       </c>
-      <c r="G58" s="9" t="inlineStr">
+      <c r="G58" s="8" t="inlineStr">
         <is>
           <t>Below threshold</t>
         </is>
@@ -4217,10 +4217,10 @@
           <t>2026-08-26</t>
         </is>
       </c>
-      <c r="F59" s="8" t="n">
+      <c r="F59" s="7" t="n">
         <v>35</v>
       </c>
-      <c r="G59" s="9" t="inlineStr">
+      <c r="G59" s="8" t="inlineStr">
         <is>
           <t>Below threshold</t>
         </is>
@@ -4280,10 +4280,10 @@
           <t>2026-08-26</t>
         </is>
       </c>
-      <c r="F60" s="8" t="n">
+      <c r="F60" s="7" t="n">
         <v>35</v>
       </c>
-      <c r="G60" s="9" t="inlineStr">
+      <c r="G60" s="8" t="inlineStr">
         <is>
           <t>Below threshold</t>
         </is>
@@ -4343,10 +4343,10 @@
           <t>2026-08-26</t>
         </is>
       </c>
-      <c r="F61" s="8" t="n">
+      <c r="F61" s="7" t="n">
         <v>35</v>
       </c>
-      <c r="G61" s="9" t="inlineStr">
+      <c r="G61" s="8" t="inlineStr">
         <is>
           <t>Below threshold</t>
         </is>
@@ -4406,10 +4406,10 @@
           <t>2026-08-26</t>
         </is>
       </c>
-      <c r="F62" s="8" t="n">
+      <c r="F62" s="7" t="n">
         <v>35</v>
       </c>
-      <c r="G62" s="9" t="inlineStr">
+      <c r="G62" s="8" t="inlineStr">
         <is>
           <t>Below threshold</t>
         </is>
@@ -4469,10 +4469,10 @@
           <t>2026-08-26</t>
         </is>
       </c>
-      <c r="F63" s="8" t="n">
+      <c r="F63" s="7" t="n">
         <v>35</v>
       </c>
-      <c r="G63" s="9" t="inlineStr">
+      <c r="G63" s="8" t="inlineStr">
         <is>
           <t>Below threshold</t>
         </is>
@@ -4532,10 +4532,10 @@
           <t>2026-08-26</t>
         </is>
       </c>
-      <c r="F64" s="8" t="n">
+      <c r="F64" s="7" t="n">
         <v>35</v>
       </c>
-      <c r="G64" s="9" t="inlineStr">
+      <c r="G64" s="8" t="inlineStr">
         <is>
           <t>Below threshold</t>
         </is>
@@ -4595,10 +4595,10 @@
           <t>2026-08-26</t>
         </is>
       </c>
-      <c r="F65" s="8" t="n">
+      <c r="F65" s="7" t="n">
         <v>35</v>
       </c>
-      <c r="G65" s="9" t="inlineStr">
+      <c r="G65" s="8" t="inlineStr">
         <is>
           <t>Below threshold</t>
         </is>
@@ -4658,10 +4658,10 @@
           <t>2026-08-26</t>
         </is>
       </c>
-      <c r="F66" s="8" t="n">
+      <c r="F66" s="7" t="n">
         <v>35</v>
       </c>
-      <c r="G66" s="9" t="inlineStr">
+      <c r="G66" s="8" t="inlineStr">
         <is>
           <t>Below threshold</t>
         </is>
@@ -4721,10 +4721,10 @@
           <t>2026-08-26</t>
         </is>
       </c>
-      <c r="F67" s="8" t="n">
+      <c r="F67" s="7" t="n">
         <v>35</v>
       </c>
-      <c r="G67" s="9" t="inlineStr">
+      <c r="G67" s="8" t="inlineStr">
         <is>
           <t>Below threshold</t>
         </is>
@@ -4784,10 +4784,10 @@
           <t>2026-08-27</t>
         </is>
       </c>
-      <c r="F68" s="8" t="n">
+      <c r="F68" s="7" t="n">
         <v>35</v>
       </c>
-      <c r="G68" s="9" t="inlineStr">
+      <c r="G68" s="8" t="inlineStr">
         <is>
           <t>Below threshold</t>
         </is>
@@ -4847,10 +4847,10 @@
           <t>2026-08-27</t>
         </is>
       </c>
-      <c r="F69" s="8" t="n">
+      <c r="F69" s="7" t="n">
         <v>35</v>
       </c>
-      <c r="G69" s="9" t="inlineStr">
+      <c r="G69" s="8" t="inlineStr">
         <is>
           <t>Below threshold</t>
         </is>
@@ -4910,10 +4910,10 @@
           <t>2026-08-27</t>
         </is>
       </c>
-      <c r="F70" s="8" t="n">
+      <c r="F70" s="7" t="n">
         <v>35</v>
       </c>
-      <c r="G70" s="9" t="inlineStr">
+      <c r="G70" s="8" t="inlineStr">
         <is>
           <t>Below threshold</t>
         </is>
@@ -4973,10 +4973,10 @@
           <t>2026-08-27</t>
         </is>
       </c>
-      <c r="F71" s="8" t="n">
+      <c r="F71" s="7" t="n">
         <v>35</v>
       </c>
-      <c r="G71" s="9" t="inlineStr">
+      <c r="G71" s="8" t="inlineStr">
         <is>
           <t>Below threshold</t>
         </is>
@@ -5036,10 +5036,10 @@
           <t>2026-08-28</t>
         </is>
       </c>
-      <c r="F72" s="8" t="n">
+      <c r="F72" s="7" t="n">
         <v>35</v>
       </c>
-      <c r="G72" s="9" t="inlineStr">
+      <c r="G72" s="8" t="inlineStr">
         <is>
           <t>Below threshold</t>
         </is>
@@ -5059,9 +5059,9 @@
           <t>Not stated in JD</t>
         </is>
       </c>
-      <c r="K72" s="7" t="inlineStr">
-        <is>
-          <t>New this run (2026-08-28 22:31 UTC)</t>
+      <c r="K72" s="2" t="inlineStr">
+        <is>
+          <t>From previous run</t>
         </is>
       </c>
       <c r="L72" s="2" t="inlineStr">
@@ -5099,10 +5099,10 @@
           <t>2026-08-26</t>
         </is>
       </c>
-      <c r="F73" s="8" t="n">
+      <c r="F73" s="7" t="n">
         <v>30</v>
       </c>
-      <c r="G73" s="9" t="inlineStr">
+      <c r="G73" s="8" t="inlineStr">
         <is>
           <t>Below threshold</t>
         </is>
@@ -5162,10 +5162,10 @@
           <t>2026-08-26</t>
         </is>
       </c>
-      <c r="F74" s="8" t="n">
+      <c r="F74" s="7" t="n">
         <v>30</v>
       </c>
-      <c r="G74" s="9" t="inlineStr">
+      <c r="G74" s="8" t="inlineStr">
         <is>
           <t>Below threshold</t>
         </is>
@@ -5225,10 +5225,10 @@
           <t>2026-08-26</t>
         </is>
       </c>
-      <c r="F75" s="8" t="n">
+      <c r="F75" s="7" t="n">
         <v>30</v>
       </c>
-      <c r="G75" s="9" t="inlineStr">
+      <c r="G75" s="8" t="inlineStr">
         <is>
           <t>Below threshold</t>
         </is>
@@ -5288,10 +5288,10 @@
           <t>2026-08-26</t>
         </is>
       </c>
-      <c r="F76" s="8" t="n">
+      <c r="F76" s="7" t="n">
         <v>30</v>
       </c>
-      <c r="G76" s="9" t="inlineStr">
+      <c r="G76" s="8" t="inlineStr">
         <is>
           <t>Below threshold</t>
         </is>
@@ -5351,10 +5351,10 @@
           <t>2026-08-26</t>
         </is>
       </c>
-      <c r="F77" s="8" t="n">
+      <c r="F77" s="7" t="n">
         <v>30</v>
       </c>
-      <c r="G77" s="9" t="inlineStr">
+      <c r="G77" s="8" t="inlineStr">
         <is>
           <t>Below threshold</t>
         </is>
@@ -5414,10 +5414,10 @@
           <t>2026-08-26</t>
         </is>
       </c>
-      <c r="F78" s="8" t="n">
+      <c r="F78" s="7" t="n">
         <v>30</v>
       </c>
-      <c r="G78" s="9" t="inlineStr">
+      <c r="G78" s="8" t="inlineStr">
         <is>
           <t>Below threshold</t>
         </is>
@@ -5477,10 +5477,10 @@
           <t>2026-08-26</t>
         </is>
       </c>
-      <c r="F79" s="8" t="n">
+      <c r="F79" s="7" t="n">
         <v>30</v>
       </c>
-      <c r="G79" s="9" t="inlineStr">
+      <c r="G79" s="8" t="inlineStr">
         <is>
           <t>Below threshold</t>
         </is>
@@ -5540,10 +5540,10 @@
           <t>2026-08-26</t>
         </is>
       </c>
-      <c r="F80" s="8" t="n">
+      <c r="F80" s="7" t="n">
         <v>30</v>
       </c>
-      <c r="G80" s="9" t="inlineStr">
+      <c r="G80" s="8" t="inlineStr">
         <is>
           <t>Below threshold</t>
         </is>
@@ -5603,10 +5603,10 @@
           <t>2026-08-26</t>
         </is>
       </c>
-      <c r="F81" s="8" t="n">
+      <c r="F81" s="7" t="n">
         <v>30</v>
       </c>
-      <c r="G81" s="9" t="inlineStr">
+      <c r="G81" s="8" t="inlineStr">
         <is>
           <t>Below threshold</t>
         </is>
@@ -5666,10 +5666,10 @@
           <t>2026-08-26</t>
         </is>
       </c>
-      <c r="F82" s="8" t="n">
+      <c r="F82" s="7" t="n">
         <v>30</v>
       </c>
-      <c r="G82" s="9" t="inlineStr">
+      <c r="G82" s="8" t="inlineStr">
         <is>
           <t>Below threshold</t>
         </is>
@@ -5729,10 +5729,10 @@
           <t>2026-08-26</t>
         </is>
       </c>
-      <c r="F83" s="8" t="n">
+      <c r="F83" s="7" t="n">
         <v>30</v>
       </c>
-      <c r="G83" s="9" t="inlineStr">
+      <c r="G83" s="8" t="inlineStr">
         <is>
           <t>Below threshold</t>
         </is>
@@ -5792,10 +5792,10 @@
           <t>2026-08-26</t>
         </is>
       </c>
-      <c r="F84" s="8" t="n">
+      <c r="F84" s="7" t="n">
         <v>30</v>
       </c>
-      <c r="G84" s="9" t="inlineStr">
+      <c r="G84" s="8" t="inlineStr">
         <is>
           <t>Below threshold</t>
         </is>
@@ -5855,10 +5855,10 @@
           <t>2026-08-26</t>
         </is>
       </c>
-      <c r="F85" s="8" t="n">
+      <c r="F85" s="7" t="n">
         <v>30</v>
       </c>
-      <c r="G85" s="9" t="inlineStr">
+      <c r="G85" s="8" t="inlineStr">
         <is>
           <t>Below threshold</t>
         </is>
@@ -5918,10 +5918,10 @@
           <t>2026-08-27</t>
         </is>
       </c>
-      <c r="F86" s="8" t="n">
+      <c r="F86" s="7" t="n">
         <v>30</v>
       </c>
-      <c r="G86" s="9" t="inlineStr">
+      <c r="G86" s="8" t="inlineStr">
         <is>
           <t>Below threshold</t>
         </is>
@@ -5981,10 +5981,10 @@
           <t>2026-08-27</t>
         </is>
       </c>
-      <c r="F87" s="8" t="n">
+      <c r="F87" s="7" t="n">
         <v>30</v>
       </c>
-      <c r="G87" s="9" t="inlineStr">
+      <c r="G87" s="8" t="inlineStr">
         <is>
           <t>Below threshold</t>
         </is>
@@ -6044,10 +6044,10 @@
           <t>2026-08-27</t>
         </is>
       </c>
-      <c r="F88" s="8" t="n">
+      <c r="F88" s="7" t="n">
         <v>30</v>
       </c>
-      <c r="G88" s="9" t="inlineStr">
+      <c r="G88" s="8" t="inlineStr">
         <is>
           <t>Below threshold</t>
         </is>
@@ -6107,10 +6107,10 @@
           <t>2026-08-27</t>
         </is>
       </c>
-      <c r="F89" s="8" t="n">
+      <c r="F89" s="7" t="n">
         <v>30</v>
       </c>
-      <c r="G89" s="9" t="inlineStr">
+      <c r="G89" s="8" t="inlineStr">
         <is>
           <t>Below threshold</t>
         </is>
@@ -6170,10 +6170,10 @@
           <t>2026-08-27</t>
         </is>
       </c>
-      <c r="F90" s="8" t="n">
+      <c r="F90" s="7" t="n">
         <v>30</v>
       </c>
-      <c r="G90" s="9" t="inlineStr">
+      <c r="G90" s="8" t="inlineStr">
         <is>
           <t>Below threshold</t>
         </is>
@@ -6233,10 +6233,10 @@
           <t>2026-08-26</t>
         </is>
       </c>
-      <c r="F91" s="8" t="n">
+      <c r="F91" s="7" t="n">
         <v>25</v>
       </c>
-      <c r="G91" s="9" t="inlineStr">
+      <c r="G91" s="8" t="inlineStr">
         <is>
           <t>Below threshold</t>
         </is>
@@ -6296,10 +6296,10 @@
           <t>2026-08-26</t>
         </is>
       </c>
-      <c r="F92" s="8" t="n">
+      <c r="F92" s="7" t="n">
         <v>25</v>
       </c>
-      <c r="G92" s="9" t="inlineStr">
+      <c r="G92" s="8" t="inlineStr">
         <is>
           <t>Below threshold</t>
         </is>
@@ -6359,10 +6359,10 @@
           <t>2026-08-26</t>
         </is>
       </c>
-      <c r="F93" s="8" t="n">
+      <c r="F93" s="7" t="n">
         <v>25</v>
       </c>
-      <c r="G93" s="9" t="inlineStr">
+      <c r="G93" s="8" t="inlineStr">
         <is>
           <t>Below threshold</t>
         </is>
@@ -6422,10 +6422,10 @@
           <t>2026-08-26</t>
         </is>
       </c>
-      <c r="F94" s="8" t="n">
+      <c r="F94" s="7" t="n">
         <v>20</v>
       </c>
-      <c r="G94" s="9" t="inlineStr">
+      <c r="G94" s="8" t="inlineStr">
         <is>
           <t>Below threshold</t>
         </is>
@@ -6485,10 +6485,10 @@
           <t>2026-08-28</t>
         </is>
       </c>
-      <c r="F95" s="8" t="n">
+      <c r="F95" s="7" t="n">
         <v>20</v>
       </c>
-      <c r="G95" s="9" t="inlineStr">
+      <c r="G95" s="8" t="inlineStr">
         <is>
           <t>Below threshold</t>
         </is>
@@ -6548,10 +6548,10 @@
           <t>2026-08-26</t>
         </is>
       </c>
-      <c r="F96" s="8" t="n">
+      <c r="F96" s="7" t="n">
         <v>15</v>
       </c>
-      <c r="G96" s="9" t="inlineStr">
+      <c r="G96" s="8" t="inlineStr">
         <is>
           <t>Below threshold</t>
         </is>
@@ -6611,10 +6611,10 @@
           <t>2026-08-26</t>
         </is>
       </c>
-      <c r="F97" s="8" t="n">
+      <c r="F97" s="7" t="n">
         <v>15</v>
       </c>
-      <c r="G97" s="9" t="inlineStr">
+      <c r="G97" s="8" t="inlineStr">
         <is>
           <t>Below threshold</t>
         </is>
@@ -6674,10 +6674,10 @@
           <t>2026-08-26</t>
         </is>
       </c>
-      <c r="F98" s="8" t="n">
+      <c r="F98" s="7" t="n">
         <v>15</v>
       </c>
-      <c r="G98" s="9" t="inlineStr">
+      <c r="G98" s="8" t="inlineStr">
         <is>
           <t>Below threshold</t>
         </is>
@@ -6737,10 +6737,10 @@
           <t>2026-08-26</t>
         </is>
       </c>
-      <c r="F99" s="8" t="n">
+      <c r="F99" s="7" t="n">
         <v>12</v>
       </c>
-      <c r="G99" s="9" t="inlineStr">
+      <c r="G99" s="8" t="inlineStr">
         <is>
           <t>Below threshold</t>
         </is>
@@ -6800,10 +6800,10 @@
           <t>2026-08-26</t>
         </is>
       </c>
-      <c r="F100" s="8" t="n">
+      <c r="F100" s="7" t="n">
         <v>12</v>
       </c>
-      <c r="G100" s="9" t="inlineStr">
+      <c r="G100" s="8" t="inlineStr">
         <is>
           <t>Below threshold</t>
         </is>
@@ -6863,10 +6863,10 @@
           <t>2026-08-26</t>
         </is>
       </c>
-      <c r="F101" s="8" t="n">
+      <c r="F101" s="7" t="n">
         <v>10</v>
       </c>
-      <c r="G101" s="9" t="inlineStr">
+      <c r="G101" s="8" t="inlineStr">
         <is>
           <t>Below threshold</t>
         </is>
@@ -6926,10 +6926,10 @@
           <t>2026-08-26</t>
         </is>
       </c>
-      <c r="F102" s="8" t="n">
+      <c r="F102" s="7" t="n">
         <v>10</v>
       </c>
-      <c r="G102" s="9" t="inlineStr">
+      <c r="G102" s="8" t="inlineStr">
         <is>
           <t>Below threshold</t>
         </is>
@@ -6989,10 +6989,10 @@
           <t>2026-08-26</t>
         </is>
       </c>
-      <c r="F103" s="8" t="n">
+      <c r="F103" s="7" t="n">
         <v>10</v>
       </c>
-      <c r="G103" s="9" t="inlineStr">
+      <c r="G103" s="8" t="inlineStr">
         <is>
           <t>Below threshold</t>
         </is>
@@ -7052,10 +7052,10 @@
           <t>2026-08-26</t>
         </is>
       </c>
-      <c r="F104" s="8" t="n">
+      <c r="F104" s="7" t="n">
         <v>10</v>
       </c>
-      <c r="G104" s="9" t="inlineStr">
+      <c r="G104" s="8" t="inlineStr">
         <is>
           <t>Below threshold</t>
         </is>
@@ -7115,10 +7115,10 @@
           <t>2026-08-26</t>
         </is>
       </c>
-      <c r="F105" s="8" t="n">
+      <c r="F105" s="7" t="n">
         <v>10</v>
       </c>
-      <c r="G105" s="9" t="inlineStr">
+      <c r="G105" s="8" t="inlineStr">
         <is>
           <t>Below threshold</t>
         </is>
@@ -7178,10 +7178,10 @@
           <t>2026-08-26</t>
         </is>
       </c>
-      <c r="F106" s="8" t="n">
+      <c r="F106" s="7" t="n">
         <v>10</v>
       </c>
-      <c r="G106" s="9" t="inlineStr">
+      <c r="G106" s="8" t="inlineStr">
         <is>
           <t>Below threshold</t>
         </is>
@@ -7241,10 +7241,10 @@
           <t>2026-08-26</t>
         </is>
       </c>
-      <c r="F107" s="8" t="n">
+      <c r="F107" s="7" t="n">
         <v>10</v>
       </c>
-      <c r="G107" s="9" t="inlineStr">
+      <c r="G107" s="8" t="inlineStr">
         <is>
           <t>Below threshold</t>
         </is>
@@ -7304,10 +7304,10 @@
           <t>2026-08-26</t>
         </is>
       </c>
-      <c r="F108" s="8" t="n">
+      <c r="F108" s="7" t="n">
         <v>10</v>
       </c>
-      <c r="G108" s="9" t="inlineStr">
+      <c r="G108" s="8" t="inlineStr">
         <is>
           <t>Below threshold</t>
         </is>
@@ -7367,10 +7367,10 @@
           <t>2026-08-26</t>
         </is>
       </c>
-      <c r="F109" s="8" t="n">
+      <c r="F109" s="7" t="n">
         <v>10</v>
       </c>
-      <c r="G109" s="9" t="inlineStr">
+      <c r="G109" s="8" t="inlineStr">
         <is>
           <t>Below threshold</t>
         </is>
@@ -7430,10 +7430,10 @@
           <t>2026-08-26</t>
         </is>
       </c>
-      <c r="F110" s="8" t="n">
+      <c r="F110" s="7" t="n">
         <v>10</v>
       </c>
-      <c r="G110" s="9" t="inlineStr">
+      <c r="G110" s="8" t="inlineStr">
         <is>
           <t>Below threshold</t>
         </is>
@@ -7493,10 +7493,10 @@
           <t>2026-08-26</t>
         </is>
       </c>
-      <c r="F111" s="8" t="n">
+      <c r="F111" s="7" t="n">
         <v>10</v>
       </c>
-      <c r="G111" s="9" t="inlineStr">
+      <c r="G111" s="8" t="inlineStr">
         <is>
           <t>Below threshold</t>
         </is>
@@ -7556,10 +7556,10 @@
           <t>2026-08-26</t>
         </is>
       </c>
-      <c r="F112" s="8" t="n">
+      <c r="F112" s="7" t="n">
         <v>10</v>
       </c>
-      <c r="G112" s="9" t="inlineStr">
+      <c r="G112" s="8" t="inlineStr">
         <is>
           <t>Below threshold</t>
         </is>
@@ -7619,10 +7619,10 @@
           <t>2026-08-26</t>
         </is>
       </c>
-      <c r="F113" s="8" t="n">
+      <c r="F113" s="7" t="n">
         <v>10</v>
       </c>
-      <c r="G113" s="9" t="inlineStr">
+      <c r="G113" s="8" t="inlineStr">
         <is>
           <t>Below threshold</t>
         </is>
@@ -7682,10 +7682,10 @@
           <t>2026-08-26</t>
         </is>
       </c>
-      <c r="F114" s="8" t="n">
+      <c r="F114" s="7" t="n">
         <v>10</v>
       </c>
-      <c r="G114" s="9" t="inlineStr">
+      <c r="G114" s="8" t="inlineStr">
         <is>
           <t>Below threshold</t>
         </is>
@@ -7745,10 +7745,10 @@
           <t>2026-08-26</t>
         </is>
       </c>
-      <c r="F115" s="8" t="n">
+      <c r="F115" s="7" t="n">
         <v>10</v>
       </c>
-      <c r="G115" s="9" t="inlineStr">
+      <c r="G115" s="8" t="inlineStr">
         <is>
           <t>Below threshold</t>
         </is>
@@ -7808,10 +7808,10 @@
           <t>2026-08-26</t>
         </is>
       </c>
-      <c r="F116" s="8" t="n">
+      <c r="F116" s="7" t="n">
         <v>10</v>
       </c>
-      <c r="G116" s="9" t="inlineStr">
+      <c r="G116" s="8" t="inlineStr">
         <is>
           <t>Below threshold</t>
         </is>
@@ -7871,10 +7871,10 @@
           <t>2026-08-26</t>
         </is>
       </c>
-      <c r="F117" s="8" t="n">
+      <c r="F117" s="7" t="n">
         <v>10</v>
       </c>
-      <c r="G117" s="9" t="inlineStr">
+      <c r="G117" s="8" t="inlineStr">
         <is>
           <t>Below threshold</t>
         </is>
@@ -7934,10 +7934,10 @@
           <t>2026-08-26</t>
         </is>
       </c>
-      <c r="F118" s="8" t="n">
+      <c r="F118" s="7" t="n">
         <v>10</v>
       </c>
-      <c r="G118" s="9" t="inlineStr">
+      <c r="G118" s="8" t="inlineStr">
         <is>
           <t>Below threshold</t>
         </is>
@@ -7997,10 +7997,10 @@
           <t>2026-08-26</t>
         </is>
       </c>
-      <c r="F119" s="8" t="n">
+      <c r="F119" s="7" t="n">
         <v>10</v>
       </c>
-      <c r="G119" s="9" t="inlineStr">
+      <c r="G119" s="8" t="inlineStr">
         <is>
           <t>Below threshold</t>
         </is>
@@ -8060,10 +8060,10 @@
           <t>2026-08-26</t>
         </is>
       </c>
-      <c r="F120" s="8" t="n">
+      <c r="F120" s="7" t="n">
         <v>10</v>
       </c>
-      <c r="G120" s="9" t="inlineStr">
+      <c r="G120" s="8" t="inlineStr">
         <is>
           <t>Below threshold</t>
         </is>
@@ -8123,10 +8123,10 @@
           <t>2026-08-27</t>
         </is>
       </c>
-      <c r="F121" s="8" t="n">
+      <c r="F121" s="7" t="n">
         <v>10</v>
       </c>
-      <c r="G121" s="9" t="inlineStr">
+      <c r="G121" s="8" t="inlineStr">
         <is>
           <t>Below threshold</t>
         </is>
@@ -8186,10 +8186,10 @@
           <t>2026-08-26</t>
         </is>
       </c>
-      <c r="F122" s="8" t="n">
+      <c r="F122" s="7" t="n">
         <v>10</v>
       </c>
-      <c r="G122" s="9" t="inlineStr">
+      <c r="G122" s="8" t="inlineStr">
         <is>
           <t>Below threshold</t>
         </is>
@@ -8249,10 +8249,10 @@
           <t>2026-08-26</t>
         </is>
       </c>
-      <c r="F123" s="8" t="n">
+      <c r="F123" s="7" t="n">
         <v>10</v>
       </c>
-      <c r="G123" s="9" t="inlineStr">
+      <c r="G123" s="8" t="inlineStr">
         <is>
           <t>Below threshold</t>
         </is>
@@ -8312,10 +8312,10 @@
           <t>2026-08-26</t>
         </is>
       </c>
-      <c r="F124" s="8" t="n">
+      <c r="F124" s="7" t="n">
         <v>10</v>
       </c>
-      <c r="G124" s="9" t="inlineStr">
+      <c r="G124" s="8" t="inlineStr">
         <is>
           <t>Below threshold</t>
         </is>
@@ -8375,10 +8375,10 @@
           <t>2026-08-27</t>
         </is>
       </c>
-      <c r="F125" s="8" t="n">
+      <c r="F125" s="7" t="n">
         <v>10</v>
       </c>
-      <c r="G125" s="9" t="inlineStr">
+      <c r="G125" s="8" t="inlineStr">
         <is>
           <t>Below threshold</t>
         </is>
@@ -8438,10 +8438,10 @@
           <t>2026-08-27</t>
         </is>
       </c>
-      <c r="F126" s="8" t="n">
+      <c r="F126" s="7" t="n">
         <v>10</v>
       </c>
-      <c r="G126" s="9" t="inlineStr">
+      <c r="G126" s="8" t="inlineStr">
         <is>
           <t>Below threshold</t>
         </is>
@@ -8501,10 +8501,10 @@
           <t>2026-08-27</t>
         </is>
       </c>
-      <c r="F127" s="8" t="n">
+      <c r="F127" s="7" t="n">
         <v>10</v>
       </c>
-      <c r="G127" s="9" t="inlineStr">
+      <c r="G127" s="8" t="inlineStr">
         <is>
           <t>Below threshold</t>
         </is>
@@ -8564,10 +8564,10 @@
           <t>2026-08-27</t>
         </is>
       </c>
-      <c r="F128" s="8" t="n">
+      <c r="F128" s="7" t="n">
         <v>10</v>
       </c>
-      <c r="G128" s="9" t="inlineStr">
+      <c r="G128" s="8" t="inlineStr">
         <is>
           <t>Below threshold</t>
         </is>
@@ -8627,10 +8627,10 @@
           <t>2026-08-27</t>
         </is>
       </c>
-      <c r="F129" s="8" t="n">
+      <c r="F129" s="7" t="n">
         <v>10</v>
       </c>
-      <c r="G129" s="9" t="inlineStr">
+      <c r="G129" s="8" t="inlineStr">
         <is>
           <t>Below threshold</t>
         </is>
@@ -8690,10 +8690,10 @@
           <t>2026-08-27</t>
         </is>
       </c>
-      <c r="F130" s="8" t="n">
+      <c r="F130" s="7" t="n">
         <v>10</v>
       </c>
-      <c r="G130" s="9" t="inlineStr">
+      <c r="G130" s="8" t="inlineStr">
         <is>
           <t>Below threshold</t>
         </is>
@@ -8753,10 +8753,10 @@
           <t>2026-08-27</t>
         </is>
       </c>
-      <c r="F131" s="8" t="n">
+      <c r="F131" s="7" t="n">
         <v>10</v>
       </c>
-      <c r="G131" s="9" t="inlineStr">
+      <c r="G131" s="8" t="inlineStr">
         <is>
           <t>Below threshold</t>
         </is>
@@ -8816,10 +8816,10 @@
           <t>2026-08-28</t>
         </is>
       </c>
-      <c r="F132" s="8" t="n">
+      <c r="F132" s="7" t="n">
         <v>10</v>
       </c>
-      <c r="G132" s="9" t="inlineStr">
+      <c r="G132" s="8" t="inlineStr">
         <is>
           <t>Below threshold</t>
         </is>
@@ -8839,9 +8839,9 @@
           <t>Not stated in JD</t>
         </is>
       </c>
-      <c r="K132" s="7" t="inlineStr">
-        <is>
-          <t>New this run (2026-08-28 22:31 UTC)</t>
+      <c r="K132" s="2" t="inlineStr">
+        <is>
+          <t>From previous run</t>
         </is>
       </c>
       <c r="L132" s="2" t="inlineStr">
@@ -8879,10 +8879,10 @@
           <t>2026-08-28</t>
         </is>
       </c>
-      <c r="F133" s="8" t="n">
+      <c r="F133" s="7" t="n">
         <v>10</v>
       </c>
-      <c r="G133" s="9" t="inlineStr">
+      <c r="G133" s="8" t="inlineStr">
         <is>
           <t>Below threshold</t>
         </is>
@@ -8902,9 +8902,9 @@
           <t>Not stated in JD</t>
         </is>
       </c>
-      <c r="K133" s="7" t="inlineStr">
-        <is>
-          <t>New this run (2026-08-28 22:31 UTC)</t>
+      <c r="K133" s="2" t="inlineStr">
+        <is>
+          <t>From previous run</t>
         </is>
       </c>
       <c r="L133" s="2" t="inlineStr">
@@ -8942,10 +8942,10 @@
           <t>2026-08-26</t>
         </is>
       </c>
-      <c r="F134" s="8" t="n">
+      <c r="F134" s="7" t="n">
         <v>5</v>
       </c>
-      <c r="G134" s="9" t="inlineStr">
+      <c r="G134" s="8" t="inlineStr">
         <is>
           <t>Below threshold</t>
         </is>
@@ -9005,10 +9005,10 @@
           <t>2026-08-26</t>
         </is>
       </c>
-      <c r="F135" s="8" t="n">
+      <c r="F135" s="7" t="n">
         <v>5</v>
       </c>
-      <c r="G135" s="9" t="inlineStr">
+      <c r="G135" s="8" t="inlineStr">
         <is>
           <t>Below threshold</t>
         </is>
@@ -9068,10 +9068,10 @@
           <t>2026-08-26</t>
         </is>
       </c>
-      <c r="F136" s="8" t="n">
+      <c r="F136" s="7" t="n">
         <v>5</v>
       </c>
-      <c r="G136" s="9" t="inlineStr">
+      <c r="G136" s="8" t="inlineStr">
         <is>
           <t>Below threshold</t>
         </is>
@@ -9131,10 +9131,10 @@
           <t>2026-08-26</t>
         </is>
       </c>
-      <c r="F137" s="8" t="n">
+      <c r="F137" s="7" t="n">
         <v>5</v>
       </c>
-      <c r="G137" s="9" t="inlineStr">
+      <c r="G137" s="8" t="inlineStr">
         <is>
           <t>Below threshold</t>
         </is>
@@ -9194,10 +9194,10 @@
           <t>2026-08-26</t>
         </is>
       </c>
-      <c r="F138" s="8" t="n">
+      <c r="F138" s="7" t="n">
         <v>5</v>
       </c>
-      <c r="G138" s="9" t="inlineStr">
+      <c r="G138" s="8" t="inlineStr">
         <is>
           <t>Below threshold</t>
         </is>
@@ -9257,10 +9257,10 @@
           <t>2026-08-26</t>
         </is>
       </c>
-      <c r="F139" s="8" t="n">
+      <c r="F139" s="7" t="n">
         <v>5</v>
       </c>
-      <c r="G139" s="9" t="inlineStr">
+      <c r="G139" s="8" t="inlineStr">
         <is>
           <t>Below threshold</t>
         </is>
@@ -9320,10 +9320,10 @@
           <t>2026-08-26</t>
         </is>
       </c>
-      <c r="F140" s="8" t="n">
+      <c r="F140" s="7" t="n">
         <v>5</v>
       </c>
-      <c r="G140" s="9" t="inlineStr">
+      <c r="G140" s="8" t="inlineStr">
         <is>
           <t>Below threshold</t>
         </is>
@@ -9383,10 +9383,10 @@
           <t>2026-08-26</t>
         </is>
       </c>
-      <c r="F141" s="8" t="n">
+      <c r="F141" s="7" t="n">
         <v>5</v>
       </c>
-      <c r="G141" s="9" t="inlineStr">
+      <c r="G141" s="8" t="inlineStr">
         <is>
           <t>Below threshold</t>
         </is>
@@ -9446,10 +9446,10 @@
           <t>2026-08-26</t>
         </is>
       </c>
-      <c r="F142" s="8" t="n">
+      <c r="F142" s="7" t="n">
         <v>5</v>
       </c>
-      <c r="G142" s="9" t="inlineStr">
+      <c r="G142" s="8" t="inlineStr">
         <is>
           <t>Below threshold</t>
         </is>
@@ -9509,10 +9509,10 @@
           <t>2026-08-26</t>
         </is>
       </c>
-      <c r="F143" s="8" t="n">
+      <c r="F143" s="7" t="n">
         <v>5</v>
       </c>
-      <c r="G143" s="9" t="inlineStr">
+      <c r="G143" s="8" t="inlineStr">
         <is>
           <t>Below threshold</t>
         </is>
@@ -9572,10 +9572,10 @@
           <t>2026-08-26</t>
         </is>
       </c>
-      <c r="F144" s="8" t="n">
+      <c r="F144" s="7" t="n">
         <v>5</v>
       </c>
-      <c r="G144" s="9" t="inlineStr">
+      <c r="G144" s="8" t="inlineStr">
         <is>
           <t>Below threshold</t>
         </is>
@@ -9635,10 +9635,10 @@
           <t>2026-08-26</t>
         </is>
       </c>
-      <c r="F145" s="8" t="n">
+      <c r="F145" s="7" t="n">
         <v>5</v>
       </c>
-      <c r="G145" s="9" t="inlineStr">
+      <c r="G145" s="8" t="inlineStr">
         <is>
           <t>Below threshold</t>
         </is>
@@ -9698,10 +9698,10 @@
           <t>2026-08-26</t>
         </is>
       </c>
-      <c r="F146" s="8" t="n">
+      <c r="F146" s="7" t="n">
         <v>5</v>
       </c>
-      <c r="G146" s="9" t="inlineStr">
+      <c r="G146" s="8" t="inlineStr">
         <is>
           <t>Below threshold</t>
         </is>
@@ -9761,10 +9761,10 @@
           <t>2026-08-26</t>
         </is>
       </c>
-      <c r="F147" s="8" t="n">
+      <c r="F147" s="7" t="n">
         <v>5</v>
       </c>
-      <c r="G147" s="9" t="inlineStr">
+      <c r="G147" s="8" t="inlineStr">
         <is>
           <t>Below threshold</t>
         </is>
@@ -9824,10 +9824,10 @@
           <t>2026-08-26</t>
         </is>
       </c>
-      <c r="F148" s="8" t="n">
+      <c r="F148" s="7" t="n">
         <v>5</v>
       </c>
-      <c r="G148" s="9" t="inlineStr">
+      <c r="G148" s="8" t="inlineStr">
         <is>
           <t>Below threshold</t>
         </is>
@@ -9887,10 +9887,10 @@
           <t>2026-08-26</t>
         </is>
       </c>
-      <c r="F149" s="8" t="n">
+      <c r="F149" s="7" t="n">
         <v>5</v>
       </c>
-      <c r="G149" s="9" t="inlineStr">
+      <c r="G149" s="8" t="inlineStr">
         <is>
           <t>Below threshold</t>
         </is>
@@ -9950,10 +9950,10 @@
           <t>2026-08-26</t>
         </is>
       </c>
-      <c r="F150" s="8" t="n">
+      <c r="F150" s="7" t="n">
         <v>5</v>
       </c>
-      <c r="G150" s="9" t="inlineStr">
+      <c r="G150" s="8" t="inlineStr">
         <is>
           <t>Below threshold</t>
         </is>
@@ -10013,10 +10013,10 @@
           <t>2026-08-26</t>
         </is>
       </c>
-      <c r="F151" s="8" t="n">
+      <c r="F151" s="7" t="n">
         <v>5</v>
       </c>
-      <c r="G151" s="9" t="inlineStr">
+      <c r="G151" s="8" t="inlineStr">
         <is>
           <t>Below threshold</t>
         </is>
@@ -10076,10 +10076,10 @@
           <t>2026-08-26</t>
         </is>
       </c>
-      <c r="F152" s="8" t="n">
+      <c r="F152" s="7" t="n">
         <v>5</v>
       </c>
-      <c r="G152" s="9" t="inlineStr">
+      <c r="G152" s="8" t="inlineStr">
         <is>
           <t>Below threshold</t>
         </is>
@@ -10139,10 +10139,10 @@
           <t>2026-08-26</t>
         </is>
       </c>
-      <c r="F153" s="8" t="n">
+      <c r="F153" s="7" t="n">
         <v>5</v>
       </c>
-      <c r="G153" s="9" t="inlineStr">
+      <c r="G153" s="8" t="inlineStr">
         <is>
           <t>Below threshold</t>
         </is>
@@ -10202,10 +10202,10 @@
           <t>2026-08-26</t>
         </is>
       </c>
-      <c r="F154" s="8" t="n">
+      <c r="F154" s="7" t="n">
         <v>5</v>
       </c>
-      <c r="G154" s="9" t="inlineStr">
+      <c r="G154" s="8" t="inlineStr">
         <is>
           <t>Below threshold</t>
         </is>
@@ -10265,10 +10265,10 @@
           <t>2026-08-26</t>
         </is>
       </c>
-      <c r="F155" s="8" t="n">
+      <c r="F155" s="7" t="n">
         <v>5</v>
       </c>
-      <c r="G155" s="9" t="inlineStr">
+      <c r="G155" s="8" t="inlineStr">
         <is>
           <t>Below threshold</t>
         </is>
@@ -10328,10 +10328,10 @@
           <t>2026-08-26</t>
         </is>
       </c>
-      <c r="F156" s="8" t="n">
+      <c r="F156" s="7" t="n">
         <v>5</v>
       </c>
-      <c r="G156" s="9" t="inlineStr">
+      <c r="G156" s="8" t="inlineStr">
         <is>
           <t>Below threshold</t>
         </is>
@@ -10391,10 +10391,10 @@
           <t>2026-08-26</t>
         </is>
       </c>
-      <c r="F157" s="8" t="n">
+      <c r="F157" s="7" t="n">
         <v>5</v>
       </c>
-      <c r="G157" s="9" t="inlineStr">
+      <c r="G157" s="8" t="inlineStr">
         <is>
           <t>Below threshold</t>
         </is>
@@ -10454,10 +10454,10 @@
           <t>2026-08-26</t>
         </is>
       </c>
-      <c r="F158" s="8" t="n">
+      <c r="F158" s="7" t="n">
         <v>5</v>
       </c>
-      <c r="G158" s="9" t="inlineStr">
+      <c r="G158" s="8" t="inlineStr">
         <is>
           <t>Below threshold</t>
         </is>
@@ -10517,10 +10517,10 @@
           <t>2026-08-26</t>
         </is>
       </c>
-      <c r="F159" s="8" t="n">
+      <c r="F159" s="7" t="n">
         <v>5</v>
       </c>
-      <c r="G159" s="9" t="inlineStr">
+      <c r="G159" s="8" t="inlineStr">
         <is>
           <t>Below threshold</t>
         </is>
@@ -10580,10 +10580,10 @@
           <t>2026-08-27</t>
         </is>
       </c>
-      <c r="F160" s="8" t="n">
+      <c r="F160" s="7" t="n">
         <v>5</v>
       </c>
-      <c r="G160" s="9" t="inlineStr">
+      <c r="G160" s="8" t="inlineStr">
         <is>
           <t>Below threshold</t>
         </is>
@@ -10643,10 +10643,10 @@
           <t>2026-08-27</t>
         </is>
       </c>
-      <c r="F161" s="8" t="n">
+      <c r="F161" s="7" t="n">
         <v>5</v>
       </c>
-      <c r="G161" s="9" t="inlineStr">
+      <c r="G161" s="8" t="inlineStr">
         <is>
           <t>Below threshold</t>
         </is>
@@ -10706,10 +10706,10 @@
           <t>2026-08-27</t>
         </is>
       </c>
-      <c r="F162" s="8" t="n">
+      <c r="F162" s="7" t="n">
         <v>5</v>
       </c>
-      <c r="G162" s="9" t="inlineStr">
+      <c r="G162" s="8" t="inlineStr">
         <is>
           <t>Below threshold</t>
         </is>
@@ -10769,10 +10769,10 @@
           <t>2026-08-27</t>
         </is>
       </c>
-      <c r="F163" s="8" t="n">
+      <c r="F163" s="7" t="n">
         <v>5</v>
       </c>
-      <c r="G163" s="9" t="inlineStr">
+      <c r="G163" s="8" t="inlineStr">
         <is>
           <t>Below threshold</t>
         </is>
@@ -10832,10 +10832,10 @@
           <t>2026-08-28</t>
         </is>
       </c>
-      <c r="F164" s="8" t="n">
+      <c r="F164" s="7" t="n">
         <v>5</v>
       </c>
-      <c r="G164" s="9" t="inlineStr">
+      <c r="G164" s="8" t="inlineStr">
         <is>
           <t>Below threshold</t>
         </is>
@@ -10855,9 +10855,9 @@
           <t>Not stated in JD</t>
         </is>
       </c>
-      <c r="K164" s="7" t="inlineStr">
-        <is>
-          <t>New this run (2026-08-28 22:31 UTC)</t>
+      <c r="K164" s="2" t="inlineStr">
+        <is>
+          <t>From previous run</t>
         </is>
       </c>
       <c r="L164" s="2" t="inlineStr">
@@ -10895,10 +10895,10 @@
           <t>2026-08-28</t>
         </is>
       </c>
-      <c r="F165" s="8" t="n">
+      <c r="F165" s="7" t="n">
         <v>5</v>
       </c>
-      <c r="G165" s="9" t="inlineStr">
+      <c r="G165" s="8" t="inlineStr">
         <is>
           <t>Below threshold</t>
         </is>
@@ -10918,9 +10918,9 @@
           <t>Not stated in JD</t>
         </is>
       </c>
-      <c r="K165" s="7" t="inlineStr">
-        <is>
-          <t>New this run (2026-08-28 22:31 UTC)</t>
+      <c r="K165" s="2" t="inlineStr">
+        <is>
+          <t>From previous run</t>
         </is>
       </c>
       <c r="L165" s="2" t="inlineStr">
@@ -10958,10 +10958,10 @@
           <t>2026-08-28</t>
         </is>
       </c>
-      <c r="F166" s="8" t="n">
+      <c r="F166" s="7" t="n">
         <v>5</v>
       </c>
-      <c r="G166" s="9" t="inlineStr">
+      <c r="G166" s="8" t="inlineStr">
         <is>
           <t>Below threshold</t>
         </is>
@@ -10981,9 +10981,9 @@
           <t>Not stated in JD</t>
         </is>
       </c>
-      <c r="K166" s="7" t="inlineStr">
-        <is>
-          <t>New this run (2026-08-28 22:31 UTC)</t>
+      <c r="K166" s="2" t="inlineStr">
+        <is>
+          <t>From previous run</t>
         </is>
       </c>
       <c r="L166" s="2" t="inlineStr">
@@ -11021,10 +11021,10 @@
           <t>2026-08-28</t>
         </is>
       </c>
-      <c r="F167" s="8" t="n">
+      <c r="F167" s="7" t="n">
         <v>5</v>
       </c>
-      <c r="G167" s="9" t="inlineStr">
+      <c r="G167" s="8" t="inlineStr">
         <is>
           <t>Below threshold</t>
         </is>
@@ -11044,9 +11044,9 @@
           <t>Not stated in JD</t>
         </is>
       </c>
-      <c r="K167" s="7" t="inlineStr">
-        <is>
-          <t>New this run (2026-08-28 22:31 UTC)</t>
+      <c r="K167" s="2" t="inlineStr">
+        <is>
+          <t>From previous run</t>
         </is>
       </c>
       <c r="L167" s="2" t="inlineStr">
@@ -11066,12 +11066,12 @@
       </c>
       <c r="B168" s="3" t="inlineStr">
         <is>
-          <t>National Assistant Planner</t>
+          <t>BI Engineer</t>
         </is>
       </c>
       <c r="C168" s="3" t="inlineStr">
         <is>
-          <t>Al-Futtaim</t>
+          <t>JD.COM</t>
         </is>
       </c>
       <c r="D168" s="3" t="inlineStr">
@@ -11081,25 +11081,25 @@
       </c>
       <c r="E168" s="2" t="inlineStr">
         <is>
-          <t>2026-08-26</t>
-        </is>
-      </c>
-      <c r="F168" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="G168" s="9" t="inlineStr">
+          <t>2026-08-29</t>
+        </is>
+      </c>
+      <c r="F168" s="7" t="n">
+        <v>5</v>
+      </c>
+      <c r="G168" s="8" t="inlineStr">
         <is>
           <t>Below threshold</t>
         </is>
       </c>
       <c r="H168" s="3" t="inlineStr">
         <is>
-          <t>This is a non-technical retail merchandise planning role focused on financial forecasting, inventory management, and sales planning, which is entirely unrelated to the candidate's GenAI, LLM, and data science specialization.</t>
+          <t>This role is a BI Engineer position focused on supply chain, logistics, and retail operations rather than data science, AI, or Generative AI. It is entirely unrelated to the candidate's core expertise in LLMs, RAG, and agentic systems.</t>
         </is>
       </c>
       <c r="I168" s="3" t="inlineStr">
         <is>
-          <t>Not stated in JD</t>
+          <t>Yes - German required (see JD for exact level)</t>
         </is>
       </c>
       <c r="J168" s="3" t="inlineStr">
@@ -11107,9 +11107,9 @@
           <t>Not stated in JD</t>
         </is>
       </c>
-      <c r="K168" s="2" t="inlineStr">
-        <is>
-          <t>From previous run</t>
+      <c r="K168" s="9" t="inlineStr">
+        <is>
+          <t>New this run (2026-08-29 13:17 UTC)</t>
         </is>
       </c>
       <c r="L168" s="2" t="inlineStr">
@@ -11119,7 +11119,7 @@
       </c>
       <c r="M168" s="6" t="inlineStr">
         <is>
-          <t>https://ae.linkedin.com/jobs/view/national-assistant-planner-at-al-futtaim-4459335643?position=23&amp;pageNum=0&amp;refId=JBPPMgbgbAFzpV%2BDL5h2AA%3D%3D&amp;trackingId=udE1OmanEOJo5NqnDVVmsw%3D%3D</t>
+          <t>https://ae.linkedin.com/jobs/view/bi-engineer-at-jd-com-4414670937?position=6&amp;pageNum=0&amp;refId=WT017Qp%2F1VFpbzjZb903BA%3D%3D&amp;trackingId=uXRSjK39jDOlXpbtHq2yzQ%3D%3D</t>
         </is>
       </c>
     </row>
@@ -11129,35 +11129,35 @@
       </c>
       <c r="B169" s="3" t="inlineStr">
         <is>
-          <t>Forward Deployed AI Integrator (UAE National Only), Field Engineering</t>
+          <t>Power BI Developer</t>
         </is>
       </c>
       <c r="C169" s="3" t="inlineStr">
         <is>
-          <t>Amazon Web Services (AWS)</t>
+          <t>Danube Group</t>
         </is>
       </c>
       <c r="D169" s="3" t="inlineStr">
         <is>
-          <t>Dubai, Dubai, United Arab Emirates</t>
+          <t>Dubai, United Arab Emirates</t>
         </is>
       </c>
       <c r="E169" s="2" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
-        </is>
-      </c>
-      <c r="F169" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="G169" s="9" t="inlineStr">
+          <t>2026-08-29</t>
+        </is>
+      </c>
+      <c r="F169" s="7" t="n">
+        <v>5</v>
+      </c>
+      <c r="G169" s="8" t="inlineStr">
         <is>
           <t>Below threshold</t>
         </is>
       </c>
       <c r="H169" s="3" t="inlineStr">
         <is>
-          <t>Although the role involves AI tooling and Python, it is restricted to UAE Nationals only, making it impossible for the candidate to qualify. Additionally, the position leans heavily toward technical program management rather than hands-on Generative AI and LLM engineering.</t>
+          <t>This is a Power BI Developer role focused on dashboards, data visualization, DAX, and SQL, which is completely unrelated to the candidate's core specialization in Generative AI, LLMs, and agentic workflows.</t>
         </is>
       </c>
       <c r="I169" s="3" t="inlineStr">
@@ -11170,9 +11170,9 @@
           <t>Not stated in JD</t>
         </is>
       </c>
-      <c r="K169" s="2" t="inlineStr">
-        <is>
-          <t>From previous run</t>
+      <c r="K169" s="9" t="inlineStr">
+        <is>
+          <t>New this run (2026-08-29 13:17 UTC)</t>
         </is>
       </c>
       <c r="L169" s="2" t="inlineStr">
@@ -11182,7 +11182,7 @@
       </c>
       <c r="M169" s="6" t="inlineStr">
         <is>
-          <t>https://ae.linkedin.com/jobs/view/forward-deployed-ai-integrator-uae-national-only-field-engineering-at-amazon-web-services-aws-4459616402?position=14&amp;pageNum=0&amp;refId=JBPPMgbgbAFzpV%2BDL5h2AA%3D%3D&amp;trackingId=suYy8hgZkG37o3lG7FlDHQ%3D%3D</t>
+          <t>https://ae.linkedin.com/jobs/view/power-bi-developer-at-danube-group-4459465901?position=5&amp;pageNum=0&amp;refId=WT017Qp%2F1VFpbzjZb903BA%3D%3D&amp;trackingId=2u7KtmoSLaInXvl%2FCAGPzw%3D%3D</t>
         </is>
       </c>
     </row>
@@ -11192,12 +11192,12 @@
       </c>
       <c r="B170" s="3" t="inlineStr">
         <is>
-          <t>GIS Specialist / Developer</t>
+          <t>National Assistant Planner</t>
         </is>
       </c>
       <c r="C170" s="3" t="inlineStr">
         <is>
-          <t>AECOM</t>
+          <t>Al-Futtaim</t>
         </is>
       </c>
       <c r="D170" s="3" t="inlineStr">
@@ -11210,17 +11210,17 @@
           <t>2026-08-26</t>
         </is>
       </c>
-      <c r="F170" s="8" t="n">
+      <c r="F170" s="7" t="n">
         <v>0</v>
       </c>
-      <c r="G170" s="9" t="inlineStr">
+      <c r="G170" s="8" t="inlineStr">
         <is>
           <t>Below threshold</t>
         </is>
       </c>
       <c r="H170" s="3" t="inlineStr">
         <is>
-          <t>This is a GIS Specialist role focused on ArcGIS Enterprise administration, spatial analysis, and Python/ArcPy automation, which is completely unrelated to the candidate's core specialization in Generative AI, LLMs, and agentic systems.</t>
+          <t>This is a non-technical retail merchandise planning role focused on financial forecasting, inventory management, and sales planning, which is entirely unrelated to the candidate's GenAI, LLM, and data science specialization.</t>
         </is>
       </c>
       <c r="I170" s="3" t="inlineStr">
@@ -11245,7 +11245,7 @@
       </c>
       <c r="M170" s="6" t="inlineStr">
         <is>
-          <t>https://ae.linkedin.com/jobs/view/gis-specialist-developer-at-aecom-4456869023?position=15&amp;pageNum=0&amp;refId=JBPPMgbgbAFzpV%2BDL5h2AA%3D%3D&amp;trackingId=lGxG6%2FYECt2YwYGWf5hEZA%3D%3D</t>
+          <t>https://ae.linkedin.com/jobs/view/national-assistant-planner-at-al-futtaim-4459335643?position=23&amp;pageNum=0&amp;refId=JBPPMgbgbAFzpV%2BDL5h2AA%3D%3D&amp;trackingId=udE1OmanEOJo5NqnDVVmsw%3D%3D</t>
         </is>
       </c>
     </row>
@@ -11255,12 +11255,12 @@
       </c>
       <c r="B171" s="3" t="inlineStr">
         <is>
-          <t>Quant Desk Lead and Portfolio Manager</t>
+          <t>Forward Deployed AI Integrator (UAE National Only), Field Engineering</t>
         </is>
       </c>
       <c r="C171" s="3" t="inlineStr">
         <is>
-          <t>EMCD</t>
+          <t>Amazon Web Services (AWS)</t>
         </is>
       </c>
       <c r="D171" s="3" t="inlineStr">
@@ -11270,20 +11270,20 @@
       </c>
       <c r="E171" s="2" t="inlineStr">
         <is>
-          <t>2026-08-26</t>
-        </is>
-      </c>
-      <c r="F171" s="8" t="n">
+          <t>2026-08-27</t>
+        </is>
+      </c>
+      <c r="F171" s="7" t="n">
         <v>0</v>
       </c>
-      <c r="G171" s="9" t="inlineStr">
+      <c r="G171" s="8" t="inlineStr">
         <is>
           <t>Below threshold</t>
         </is>
       </c>
       <c r="H171" s="3" t="inlineStr">
         <is>
-          <t>This is a finance and quantitative trading role focused on running a systematic trading desk, portfolio management, and P&amp;L ownership, which is entirely unrelated to the candidate's core specialization in Generative AI, LLMs, and agentic systems.</t>
+          <t>Although the role involves AI tooling and Python, it is restricted to UAE Nationals only, making it impossible for the candidate to qualify. Additionally, the position leans heavily toward technical program management rather than hands-on Generative AI and LLM engineering.</t>
         </is>
       </c>
       <c r="I171" s="3" t="inlineStr">
@@ -11308,7 +11308,7 @@
       </c>
       <c r="M171" s="6" t="inlineStr">
         <is>
-          <t>https://ae.linkedin.com/jobs/view/quant-desk-lead-and-portfolio-manager-at-emcd-4457949555?position=13&amp;pageNum=0&amp;refId=JBPPMgbgbAFzpV%2BDL5h2AA%3D%3D&amp;trackingId=drHtrw6uBtEz5S2i%2BjBT5A%3D%3D</t>
+          <t>https://ae.linkedin.com/jobs/view/forward-deployed-ai-integrator-uae-national-only-field-engineering-at-amazon-web-services-aws-4459616402?position=14&amp;pageNum=0&amp;refId=JBPPMgbgbAFzpV%2BDL5h2AA%3D%3D&amp;trackingId=suYy8hgZkG37o3lG7FlDHQ%3D%3D</t>
         </is>
       </c>
     </row>
@@ -11318,17 +11318,17 @@
       </c>
       <c r="B172" s="3" t="inlineStr">
         <is>
-          <t>Join Norlys Energy Trading</t>
+          <t>GIS Specialist / Developer</t>
         </is>
       </c>
       <c r="C172" s="3" t="inlineStr">
         <is>
-          <t>Norlys Energy Trading A/S</t>
+          <t>AECOM</t>
         </is>
       </c>
       <c r="D172" s="3" t="inlineStr">
         <is>
-          <t>Aalborg, North Denmark Region, Denmark</t>
+          <t>Dubai, Dubai, United Arab Emirates</t>
         </is>
       </c>
       <c r="E172" s="2" t="inlineStr">
@@ -11336,17 +11336,17 @@
           <t>2026-08-26</t>
         </is>
       </c>
-      <c r="F172" s="8" t="n">
+      <c r="F172" s="7" t="n">
         <v>0</v>
       </c>
-      <c r="G172" s="9" t="inlineStr">
+      <c r="G172" s="8" t="inlineStr">
         <is>
           <t>Below threshold</t>
         </is>
       </c>
       <c r="H172" s="3" t="inlineStr">
         <is>
-          <t>This is an open, unsolicited job application for a general talent pool in energy trading, rather than a defined Data Science or Generative AI role. It completely lacks technical specifications, making it impossible to evaluate against the candidate's specialized GenAI and LLM expertise.</t>
+          <t>This is a GIS Specialist role focused on ArcGIS Enterprise administration, spatial analysis, and Python/ArcPy automation, which is completely unrelated to the candidate's core specialization in Generative AI, LLMs, and agentic systems.</t>
         </is>
       </c>
       <c r="I172" s="3" t="inlineStr">
@@ -11371,7 +11371,7 @@
       </c>
       <c r="M172" s="6" t="inlineStr">
         <is>
-          <t>https://dk.linkedin.com/jobs/view/join-norlys-energy-trading-at-norlys-energy-trading-a-s-4459158084?position=26&amp;pageNum=0&amp;refId=Pb2EWWHgR9a7i9BrLIIg7g%3D%3D&amp;trackingId=Z%2BOuDrbPap3omWro18MA2g%3D%3D</t>
+          <t>https://ae.linkedin.com/jobs/view/gis-specialist-developer-at-aecom-4456869023?position=15&amp;pageNum=0&amp;refId=JBPPMgbgbAFzpV%2BDL5h2AA%3D%3D&amp;trackingId=lGxG6%2FYECt2YwYGWf5hEZA%3D%3D</t>
         </is>
       </c>
     </row>
@@ -11381,17 +11381,17 @@
       </c>
       <c r="B173" s="3" t="inlineStr">
         <is>
-          <t>PhD scholarship in Modeling and Control of Parkinson’s Disease - DTU Electro</t>
+          <t>Quant Desk Lead and Portfolio Manager</t>
         </is>
       </c>
       <c r="C173" s="3" t="inlineStr">
         <is>
-          <t>DTU - Technical University of Denmark</t>
+          <t>EMCD</t>
         </is>
       </c>
       <c r="D173" s="3" t="inlineStr">
         <is>
-          <t>Kongens Lyngby, Capital Region of Denmark, Denmark</t>
+          <t>Dubai, Dubai, United Arab Emirates</t>
         </is>
       </c>
       <c r="E173" s="2" t="inlineStr">
@@ -11399,17 +11399,17 @@
           <t>2026-08-26</t>
         </is>
       </c>
-      <c r="F173" s="8" t="n">
+      <c r="F173" s="7" t="n">
         <v>0</v>
       </c>
-      <c r="G173" s="9" t="inlineStr">
+      <c r="G173" s="8" t="inlineStr">
         <is>
           <t>Below threshold</t>
         </is>
       </c>
       <c r="H173" s="3" t="inlineStr">
         <is>
-          <t>This is a PhD scholarship position in neuroengineering, control systems, and healthcare technology at DTU, which is completely unrelated to the candidate's specialization in Generative AI, LLMs, and agentic systems.</t>
+          <t>This is a finance and quantitative trading role focused on running a systematic trading desk, portfolio management, and P&amp;L ownership, which is entirely unrelated to the candidate's core specialization in Generative AI, LLMs, and agentic systems.</t>
         </is>
       </c>
       <c r="I173" s="3" t="inlineStr">
@@ -11419,7 +11419,7 @@
       </c>
       <c r="J173" s="3" t="inlineStr">
         <is>
-          <t>Possible - relocation support mentioned, visa not explicit</t>
+          <t>Not stated in JD</t>
         </is>
       </c>
       <c r="K173" s="2" t="inlineStr">
@@ -11434,7 +11434,7 @@
       </c>
       <c r="M173" s="6" t="inlineStr">
         <is>
-          <t>https://dk.linkedin.com/jobs/view/phd-scholarship-in-modeling-and-control-of-parkinson%E2%80%99s-disease-dtu-electro-at-dtu-technical-university-of-denmark-4459145557?position=20&amp;pageNum=0&amp;refId=Pb2EWWHgR9a7i9BrLIIg7g%3D%3D&amp;trackingId=mStwcLkWBAvzmreGSwO4Hw%3D%3D</t>
+          <t>https://ae.linkedin.com/jobs/view/quant-desk-lead-and-portfolio-manager-at-emcd-4457949555?position=13&amp;pageNum=0&amp;refId=JBPPMgbgbAFzpV%2BDL5h2AA%3D%3D&amp;trackingId=drHtrw6uBtEz5S2i%2BjBT5A%3D%3D</t>
         </is>
       </c>
     </row>
@@ -11444,17 +11444,17 @@
       </c>
       <c r="B174" s="3" t="inlineStr">
         <is>
-          <t>Analytikere med flair for databehandling til PET's kontraspionageindsats mod Rusland</t>
+          <t>Join Norlys Energy Trading</t>
         </is>
       </c>
       <c r="C174" s="3" t="inlineStr">
         <is>
-          <t>Politi</t>
+          <t>Norlys Energy Trading A/S</t>
         </is>
       </c>
       <c r="D174" s="3" t="inlineStr">
         <is>
-          <t>Copenhagen, Capital Region of Denmark, Denmark</t>
+          <t>Aalborg, North Denmark Region, Denmark</t>
         </is>
       </c>
       <c r="E174" s="2" t="inlineStr">
@@ -11462,17 +11462,17 @@
           <t>2026-08-26</t>
         </is>
       </c>
-      <c r="F174" s="8" t="n">
+      <c r="F174" s="7" t="n">
         <v>0</v>
       </c>
-      <c r="G174" s="9" t="inlineStr">
+      <c r="G174" s="8" t="inlineStr">
         <is>
           <t>Below threshold</t>
         </is>
       </c>
       <c r="H174" s="3" t="inlineStr">
         <is>
-          <t>This is a national security intelligence and counter-espionage analyst role at the Danish Security and Intelligence Service (PET), which is completely unrelated to data science, artificial intelligence, or the candidate's Generative AI and LLM specialization.</t>
+          <t>This is an open, unsolicited job application for a general talent pool in energy trading, rather than a defined Data Science or Generative AI role. It completely lacks technical specifications, making it impossible to evaluate against the candidate's specialized GenAI and LLM expertise.</t>
         </is>
       </c>
       <c r="I174" s="3" t="inlineStr">
@@ -11497,7 +11497,7 @@
       </c>
       <c r="M174" s="6" t="inlineStr">
         <is>
-          <t>https://dk.linkedin.com/jobs/view/analytikere-med-flair-for-databehandling-til-pet-s-kontraspionageindsats-mod-rusland-at-politi-4457943820?position=18&amp;pageNum=0&amp;refId=Pb2EWWHgR9a7i9BrLIIg7g%3D%3D&amp;trackingId=%2FGEw4KOC0oARqkQIDTGJ4Q%3D%3D</t>
+          <t>https://dk.linkedin.com/jobs/view/join-norlys-energy-trading-at-norlys-energy-trading-a-s-4459158084?position=26&amp;pageNum=0&amp;refId=Pb2EWWHgR9a7i9BrLIIg7g%3D%3D&amp;trackingId=Z%2BOuDrbPap3omWro18MA2g%3D%3D</t>
         </is>
       </c>
     </row>
@@ -11507,17 +11507,17 @@
       </c>
       <c r="B175" s="3" t="inlineStr">
         <is>
-          <t>PostDoc - Uncertainty-Aware Optimization in Inverse Problems for Next-Generation 3D Scanning</t>
+          <t>PhD scholarship in Modeling and Control of Parkinson’s Disease - DTU Electro</t>
         </is>
       </c>
       <c r="C175" s="3" t="inlineStr">
         <is>
-          <t>3Shape</t>
+          <t>DTU - Technical University of Denmark</t>
         </is>
       </c>
       <c r="D175" s="3" t="inlineStr">
         <is>
-          <t>Copenhagen, Capital Region of Denmark, Denmark</t>
+          <t>Kongens Lyngby, Capital Region of Denmark, Denmark</t>
         </is>
       </c>
       <c r="E175" s="2" t="inlineStr">
@@ -11525,17 +11525,17 @@
           <t>2026-08-26</t>
         </is>
       </c>
-      <c r="F175" s="8" t="n">
+      <c r="F175" s="7" t="n">
         <v>0</v>
       </c>
-      <c r="G175" s="9" t="inlineStr">
+      <c r="G175" s="8" t="inlineStr">
         <is>
           <t>Below threshold</t>
         </is>
       </c>
       <c r="H175" s="3" t="inlineStr">
         <is>
-          <t>This is a PostDoc position focused on mathematical optimization, numerical linear algebra, and uncertainty quantification for 3D scanning, which requires a PhD. It has no overlap with the candidate's specialization in GenAI, LLMs, and agentic systems.</t>
+          <t>This is a PhD scholarship position in neuroengineering, control systems, and healthcare technology at DTU, which is completely unrelated to the candidate's specialization in Generative AI, LLMs, and agentic systems.</t>
         </is>
       </c>
       <c r="I175" s="3" t="inlineStr">
@@ -11545,7 +11545,7 @@
       </c>
       <c r="J175" s="3" t="inlineStr">
         <is>
-          <t>Not stated in JD</t>
+          <t>Possible - relocation support mentioned, visa not explicit</t>
         </is>
       </c>
       <c r="K175" s="2" t="inlineStr">
@@ -11560,7 +11560,7 @@
       </c>
       <c r="M175" s="6" t="inlineStr">
         <is>
-          <t>https://dk.linkedin.com/jobs/view/postdoc-uncertainty-aware-optimization-in-inverse-problems-for-next-generation-3d-scanning-at-3shape-4459171806?position=15&amp;pageNum=0&amp;refId=Pb2EWWHgR9a7i9BrLIIg7g%3D%3D&amp;trackingId=bO0aSGZ%2FUAxThXN9yvOERg%3D%3D</t>
+          <t>https://dk.linkedin.com/jobs/view/phd-scholarship-in-modeling-and-control-of-parkinson%E2%80%99s-disease-dtu-electro-at-dtu-technical-university-of-denmark-4459145557?position=20&amp;pageNum=0&amp;refId=Pb2EWWHgR9a7i9BrLIIg7g%3D%3D&amp;trackingId=mStwcLkWBAvzmreGSwO4Hw%3D%3D</t>
         </is>
       </c>
     </row>
@@ -11570,17 +11570,17 @@
       </c>
       <c r="B176" s="3" t="inlineStr">
         <is>
-          <t>Scientist, Quantitative Clinical Pharmacology (PK/PD Modeling &amp; Simulation)</t>
+          <t>Analytikere med flair for databehandling til PET's kontraspionageindsats mod Rusland</t>
         </is>
       </c>
       <c r="C176" s="3" t="inlineStr">
         <is>
-          <t>Hemab Therapeutics</t>
+          <t>Politi</t>
         </is>
       </c>
       <c r="D176" s="3" t="inlineStr">
         <is>
-          <t>Copenhagen Metropolitan Area</t>
+          <t>Copenhagen, Capital Region of Denmark, Denmark</t>
         </is>
       </c>
       <c r="E176" s="2" t="inlineStr">
@@ -11588,17 +11588,17 @@
           <t>2026-08-26</t>
         </is>
       </c>
-      <c r="F176" s="8" t="n">
+      <c r="F176" s="7" t="n">
         <v>0</v>
       </c>
-      <c r="G176" s="9" t="inlineStr">
+      <c r="G176" s="8" t="inlineStr">
         <is>
           <t>Below threshold</t>
         </is>
       </c>
       <c r="H176" s="3" t="inlineStr">
         <is>
-          <t>This is a highly specialized biomedical role focusing on Pharmacokinetics/Pharmacodynamics (PK/PD) modeling and clinical pharmacology, requiring a Ph.D. and experience with tools like NONMEM or Monolix. It has zero overlap with the candidate's GenAI, LLM, and data science background.</t>
+          <t>This is a national security intelligence and counter-espionage analyst role at the Danish Security and Intelligence Service (PET), which is completely unrelated to data science, artificial intelligence, or the candidate's Generative AI and LLM specialization.</t>
         </is>
       </c>
       <c r="I176" s="3" t="inlineStr">
@@ -11623,7 +11623,7 @@
       </c>
       <c r="M176" s="6" t="inlineStr">
         <is>
-          <t>https://dk.linkedin.com/jobs/view/scientist-quantitative-clinical-pharmacology-pk-pd-modeling-simulation-at-hemab-therapeutics-4457218306?position=14&amp;pageNum=0&amp;refId=Pb2EWWHgR9a7i9BrLIIg7g%3D%3D&amp;trackingId=jhTyKvDAQ70R9PD5s0x2yA%3D%3D</t>
+          <t>https://dk.linkedin.com/jobs/view/analytikere-med-flair-for-databehandling-til-pet-s-kontraspionageindsats-mod-rusland-at-politi-4457943820?position=18&amp;pageNum=0&amp;refId=Pb2EWWHgR9a7i9BrLIIg7g%3D%3D&amp;trackingId=%2FGEw4KOC0oARqkQIDTGJ4Q%3D%3D</t>
         </is>
       </c>
     </row>
@@ -11633,17 +11633,17 @@
       </c>
       <c r="B177" s="3" t="inlineStr">
         <is>
-          <t>Senior Payload Data Operator</t>
+          <t>PostDoc - Uncertainty-Aware Optimization in Inverse Problems for Next-Generation 3D Scanning</t>
         </is>
       </c>
       <c r="C177" s="3" t="inlineStr">
         <is>
-          <t>FADA</t>
+          <t>3Shape</t>
         </is>
       </c>
       <c r="D177" s="3" t="inlineStr">
         <is>
-          <t>United Arab Emirates</t>
+          <t>Copenhagen, Capital Region of Denmark, Denmark</t>
         </is>
       </c>
       <c r="E177" s="2" t="inlineStr">
@@ -11651,17 +11651,17 @@
           <t>2026-08-26</t>
         </is>
       </c>
-      <c r="F177" s="8" t="n">
+      <c r="F177" s="7" t="n">
         <v>0</v>
       </c>
-      <c r="G177" s="9" t="inlineStr">
+      <c r="G177" s="8" t="inlineStr">
         <is>
           <t>Below threshold</t>
         </is>
       </c>
       <c r="H177" s="3" t="inlineStr">
         <is>
-          <t>This is a satellite payload data engineering role focused on aerospace, remote sensing, and image processing (EO/SAR), which is completely unrelated to the candidate's specialization in GenAI, LLMs, and agentic systems.</t>
+          <t>This is a PostDoc position focused on mathematical optimization, numerical linear algebra, and uncertainty quantification for 3D scanning, which requires a PhD. It has no overlap with the candidate's specialization in GenAI, LLMs, and agentic systems.</t>
         </is>
       </c>
       <c r="I177" s="3" t="inlineStr">
@@ -11686,7 +11686,7 @@
       </c>
       <c r="M177" s="6" t="inlineStr">
         <is>
-          <t>https://ae.linkedin.com/jobs/view/senior-payload-data-operator-at-fada-4448986926?position=20&amp;pageNum=0&amp;refId=W92GFmCMxOQHlXfyvp17MQ%3D%3D&amp;trackingId=xdfP2za0I45WGIW%2FRJb%2BgA%3D%3D</t>
+          <t>https://dk.linkedin.com/jobs/view/postdoc-uncertainty-aware-optimization-in-inverse-problems-for-next-generation-3d-scanning-at-3shape-4459171806?position=15&amp;pageNum=0&amp;refId=Pb2EWWHgR9a7i9BrLIIg7g%3D%3D&amp;trackingId=bO0aSGZ%2FUAxThXN9yvOERg%3D%3D</t>
         </is>
       </c>
     </row>
@@ -11696,35 +11696,35 @@
       </c>
       <c r="B178" s="3" t="inlineStr">
         <is>
-          <t>Arabic Speech And Natural Language Processing Specialist</t>
+          <t>Scientist, Quantitative Clinical Pharmacology (PK/PD Modeling &amp; Simulation)</t>
         </is>
       </c>
       <c r="C178" s="3" t="inlineStr">
         <is>
-          <t>Birbal AI</t>
+          <t>Hemab Therapeutics</t>
         </is>
       </c>
       <c r="D178" s="3" t="inlineStr">
         <is>
-          <t>Abu Dhabi Emirate, United Arab Emirates</t>
+          <t>Copenhagen Metropolitan Area</t>
         </is>
       </c>
       <c r="E178" s="2" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
-        </is>
-      </c>
-      <c r="F178" s="8" t="n">
+          <t>2026-08-26</t>
+        </is>
+      </c>
+      <c r="F178" s="7" t="n">
         <v>0</v>
       </c>
-      <c r="G178" s="9" t="inlineStr">
+      <c r="G178" s="8" t="inlineStr">
         <is>
           <t>Below threshold</t>
         </is>
       </c>
       <c r="H178" s="3" t="inlineStr">
         <is>
-          <t>The role requires specialized expertise in Arabic speech technology (ASR, TTS, audio DSP) and native command of Gulf Arabic dialects, which does not match the candidate's core background in GenAI, LLMs, and RAG for English-language banking and HR use cases.</t>
+          <t>This is a highly specialized biomedical role focusing on Pharmacokinetics/Pharmacodynamics (PK/PD) modeling and clinical pharmacology, requiring a Ph.D. and experience with tools like NONMEM or Monolix. It has zero overlap with the candidate's GenAI, LLM, and data science background.</t>
         </is>
       </c>
       <c r="I178" s="3" t="inlineStr">
@@ -11749,7 +11749,7 @@
       </c>
       <c r="M178" s="6" t="inlineStr">
         <is>
-          <t>https://ae.linkedin.com/jobs/view/arabic-speech-and-natural-language-processing-specialist-at-birbal-ai-4457738899?position=14&amp;pageNum=0&amp;refId=W92GFmCMxOQHlXfyvp17MQ%3D%3D&amp;trackingId=ztG06Ly%2FIZ3fxm%2Fhvl626A%3D%3D</t>
+          <t>https://dk.linkedin.com/jobs/view/scientist-quantitative-clinical-pharmacology-pk-pd-modeling-simulation-at-hemab-therapeutics-4457218306?position=14&amp;pageNum=0&amp;refId=Pb2EWWHgR9a7i9BrLIIg7g%3D%3D&amp;trackingId=jhTyKvDAQ70R9PD5s0x2yA%3D%3D</t>
         </is>
       </c>
     </row>
@@ -11759,12 +11759,12 @@
       </c>
       <c r="B179" s="3" t="inlineStr">
         <is>
-          <t>Member of Technical Staff - Medical Research (Remote)</t>
+          <t>Senior Payload Data Operator</t>
         </is>
       </c>
       <c r="C179" s="3" t="inlineStr">
         <is>
-          <t>Hire Feed</t>
+          <t>FADA</t>
         </is>
       </c>
       <c r="D179" s="3" t="inlineStr">
@@ -11774,20 +11774,20 @@
       </c>
       <c r="E179" s="2" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
-        </is>
-      </c>
-      <c r="F179" s="8" t="n">
+          <t>2026-08-26</t>
+        </is>
+      </c>
+      <c r="F179" s="7" t="n">
         <v>0</v>
       </c>
-      <c r="G179" s="9" t="inlineStr">
+      <c r="G179" s="8" t="inlineStr">
         <is>
           <t>Below threshold</t>
         </is>
       </c>
       <c r="H179" s="3" t="inlineStr">
         <is>
-          <t>This role is completely unrelated to the candidate's specialization in Generative AI, LLMs, and agentic workflows, focusing instead on medical imaging, computational biology, and clinical research requiring a PhD.</t>
+          <t>This is a satellite payload data engineering role focused on aerospace, remote sensing, and image processing (EO/SAR), which is completely unrelated to the candidate's specialization in GenAI, LLMs, and agentic systems.</t>
         </is>
       </c>
       <c r="I179" s="3" t="inlineStr">
@@ -11812,7 +11812,7 @@
       </c>
       <c r="M179" s="6" t="inlineStr">
         <is>
-          <t>https://ae.linkedin.com/jobs/view/member-of-technical-staff-medical-research-remote-at-hire-feed-4459638503?position=3&amp;pageNum=0&amp;refId=W92GFmCMxOQHlXfyvp17MQ%3D%3D&amp;trackingId=b91zxKPZNgdFnMmW%2FlYbHA%3D%3D</t>
+          <t>https://ae.linkedin.com/jobs/view/senior-payload-data-operator-at-fada-4448986926?position=20&amp;pageNum=0&amp;refId=W92GFmCMxOQHlXfyvp17MQ%3D%3D&amp;trackingId=xdfP2za0I45WGIW%2FRJb%2BgA%3D%3D</t>
         </is>
       </c>
     </row>
@@ -11822,17 +11822,17 @@
       </c>
       <c r="B180" s="3" t="inlineStr">
         <is>
-          <t>AI Image Specialist</t>
+          <t>Arabic Speech And Natural Language Processing Specialist</t>
         </is>
       </c>
       <c r="C180" s="3" t="inlineStr">
         <is>
-          <t>Puffy</t>
+          <t>Birbal AI</t>
         </is>
       </c>
       <c r="D180" s="3" t="inlineStr">
         <is>
-          <t>Dubai, United Arab Emirates</t>
+          <t>Abu Dhabi Emirate, United Arab Emirates</t>
         </is>
       </c>
       <c r="E180" s="2" t="inlineStr">
@@ -11840,17 +11840,17 @@
           <t>2026-08-27</t>
         </is>
       </c>
-      <c r="F180" s="8" t="n">
+      <c r="F180" s="7" t="n">
         <v>0</v>
       </c>
-      <c r="G180" s="9" t="inlineStr">
+      <c r="G180" s="8" t="inlineStr">
         <is>
           <t>Below threshold</t>
         </is>
       </c>
       <c r="H180" s="3" t="inlineStr">
         <is>
-          <t>This is an AI Image Specialist role focused on generative visual design and creative production (Midjourney, DALL-E, image synthesis), which is completely unrelated to the candidate's core specialization in LLMs, RAG, LangChain, and agentic AI pipelines for data science and enterprise applications.</t>
+          <t>The role requires specialized expertise in Arabic speech technology (ASR, TTS, audio DSP) and native command of Gulf Arabic dialects, which does not match the candidate's core background in GenAI, LLMs, and RAG for English-language banking and HR use cases.</t>
         </is>
       </c>
       <c r="I180" s="3" t="inlineStr">
@@ -11860,7 +11860,7 @@
       </c>
       <c r="J180" s="3" t="inlineStr">
         <is>
-          <t>Yes - explicitly stated in JD</t>
+          <t>Not stated in JD</t>
         </is>
       </c>
       <c r="K180" s="2" t="inlineStr">
@@ -11875,7 +11875,7 @@
       </c>
       <c r="M180" s="6" t="inlineStr">
         <is>
-          <t>https://ae.linkedin.com/jobs/view/ai-image-specialist-at-puffy-4457756193?position=10&amp;pageNum=0&amp;refId=50H6yCrEXIuhgr6eqEojNg%3D%3D&amp;trackingId=9EIvgvUNu%2BE37717JffiJA%3D%3D</t>
+          <t>https://ae.linkedin.com/jobs/view/arabic-speech-and-natural-language-processing-specialist-at-birbal-ai-4457738899?position=14&amp;pageNum=0&amp;refId=W92GFmCMxOQHlXfyvp17MQ%3D%3D&amp;trackingId=ztG06Ly%2FIZ3fxm%2Fhvl626A%3D%3D</t>
         </is>
       </c>
     </row>
@@ -11885,35 +11885,35 @@
       </c>
       <c r="B181" s="3" t="inlineStr">
         <is>
-          <t>Market Operations &amp; Analytics Specialist — Institutional</t>
+          <t>Member of Technical Staff - Medical Research (Remote)</t>
         </is>
       </c>
       <c r="C181" s="3" t="inlineStr">
         <is>
-          <t>Confidential</t>
+          <t>Hire Feed</t>
         </is>
       </c>
       <c r="D181" s="3" t="inlineStr">
         <is>
-          <t>Dubai, United Arab Emirates</t>
+          <t>United Arab Emirates</t>
         </is>
       </c>
       <c r="E181" s="2" t="inlineStr">
         <is>
-          <t>2026-08-28</t>
-        </is>
-      </c>
-      <c r="F181" s="8" t="n">
+          <t>2026-08-27</t>
+        </is>
+      </c>
+      <c r="F181" s="7" t="n">
         <v>0</v>
       </c>
-      <c r="G181" s="9" t="inlineStr">
+      <c r="G181" s="8" t="inlineStr">
         <is>
           <t>Below threshold</t>
         </is>
       </c>
       <c r="H181" s="3" t="inlineStr">
         <is>
-          <t>This role is completely unrelated to data science, artificial intelligence, LLMs, or generative AI, focusing entirely on cryptocurrency exchange operations, institutional client management, and trading analytics instead.</t>
+          <t>This role is completely unrelated to the candidate's specialization in Generative AI, LLMs, and agentic workflows, focusing instead on medical imaging, computational biology, and clinical research requiring a PhD.</t>
         </is>
       </c>
       <c r="I181" s="3" t="inlineStr">
@@ -11938,7 +11938,7 @@
       </c>
       <c r="M181" s="6" t="inlineStr">
         <is>
-          <t>https://ae.linkedin.com/jobs/view/market-operations-analytics-specialist-%E2%80%94-institutional-at-confidential-4453037100?position=10&amp;pageNum=0&amp;refId=zJBbvwb5H0wsbJ5fs9ZTVw%3D%3D&amp;trackingId=ENnWCvoEQXOg1fXKuxlBug%3D%3D</t>
+          <t>https://ae.linkedin.com/jobs/view/member-of-technical-staff-medical-research-remote-at-hire-feed-4459638503?position=3&amp;pageNum=0&amp;refId=W92GFmCMxOQHlXfyvp17MQ%3D%3D&amp;trackingId=b91zxKPZNgdFnMmW%2FlYbHA%3D%3D</t>
         </is>
       </c>
     </row>
@@ -11948,17 +11948,17 @@
       </c>
       <c r="B182" s="3" t="inlineStr">
         <is>
-          <t>Quantitative Developer, Systematic Equities</t>
+          <t>AI Image Specialist</t>
         </is>
       </c>
       <c r="C182" s="3" t="inlineStr">
         <is>
-          <t>Millennium</t>
+          <t>Puffy</t>
         </is>
       </c>
       <c r="D182" s="3" t="inlineStr">
         <is>
-          <t>Dubai, Dubai, United Arab Emirates</t>
+          <t>Dubai, United Arab Emirates</t>
         </is>
       </c>
       <c r="E182" s="2" t="inlineStr">
@@ -11966,17 +11966,17 @@
           <t>2026-08-27</t>
         </is>
       </c>
-      <c r="F182" s="8" t="n">
+      <c r="F182" s="7" t="n">
         <v>0</v>
       </c>
-      <c r="G182" s="9" t="inlineStr">
+      <c r="G182" s="8" t="inlineStr">
         <is>
           <t>Below threshold</t>
         </is>
       </c>
       <c r="H182" s="3" t="inlineStr">
         <is>
-          <t>This role is a quantitative software engineering position focused on low-latency trading infrastructure, C++/C# development, and execution systems for a hedge fund, which is entirely unrelated to the candidate's specialization in GenAI, LLMs, and agentic architectures.</t>
+          <t>This is an AI Image Specialist role focused on generative visual design and creative production (Midjourney, DALL-E, image synthesis), which is completely unrelated to the candidate's core specialization in LLMs, RAG, LangChain, and agentic AI pipelines for data science and enterprise applications.</t>
         </is>
       </c>
       <c r="I182" s="3" t="inlineStr">
@@ -11986,7 +11986,7 @@
       </c>
       <c r="J182" s="3" t="inlineStr">
         <is>
-          <t>Not stated in JD</t>
+          <t>Yes - explicitly stated in JD</t>
         </is>
       </c>
       <c r="K182" s="2" t="inlineStr">
@@ -12001,7 +12001,7 @@
       </c>
       <c r="M182" s="6" t="inlineStr">
         <is>
-          <t>https://ae.linkedin.com/jobs/view/quantitative-developer-systematic-equities-at-millennium-4290849018?position=6&amp;pageNum=0&amp;refId=zJBbvwb5H0wsbJ5fs9ZTVw%3D%3D&amp;trackingId=8TTWkyG2j%2F7MELtLSQ5VCA%3D%3D</t>
+          <t>https://ae.linkedin.com/jobs/view/ai-image-specialist-at-puffy-4457756193?position=10&amp;pageNum=0&amp;refId=50H6yCrEXIuhgr6eqEojNg%3D%3D&amp;trackingId=9EIvgvUNu%2BE37717JffiJA%3D%3D</t>
         </is>
       </c>
     </row>
@@ -12011,17 +12011,17 @@
       </c>
       <c r="B183" s="3" t="inlineStr">
         <is>
-          <t>Senior Specialist - Portfolio Management</t>
+          <t>Market Operations &amp; Analytics Specialist — Institutional</t>
         </is>
       </c>
       <c r="C183" s="3" t="inlineStr">
         <is>
-          <t>MENA Careers</t>
+          <t>Confidential</t>
         </is>
       </c>
       <c r="D183" s="3" t="inlineStr">
         <is>
-          <t>Dubai, Dubai, United Arab Emirates</t>
+          <t>Dubai, United Arab Emirates</t>
         </is>
       </c>
       <c r="E183" s="2" t="inlineStr">
@@ -12029,17 +12029,17 @@
           <t>2026-08-28</t>
         </is>
       </c>
-      <c r="F183" s="8" t="n">
+      <c r="F183" s="7" t="n">
         <v>0</v>
       </c>
-      <c r="G183" s="9" t="inlineStr">
+      <c r="G183" s="8" t="inlineStr">
         <is>
           <t>Below threshold</t>
         </is>
       </c>
       <c r="H183" s="3" t="inlineStr">
         <is>
-          <t>This is a non-AI banking role focused on portfolio management, loan optimization, and regulatory capital compliance in Dubai requiring UAE nationality, which completely misaligns with the candidate's GenAI, LLM, and data science specialization.</t>
+          <t>This role is completely unrelated to data science, artificial intelligence, LLMs, or generative AI, focusing entirely on cryptocurrency exchange operations, institutional client management, and trading analytics instead.</t>
         </is>
       </c>
       <c r="I183" s="3" t="inlineStr">
@@ -12052,9 +12052,9 @@
           <t>Not stated in JD</t>
         </is>
       </c>
-      <c r="K183" s="7" t="inlineStr">
-        <is>
-          <t>New this run (2026-08-28 22:31 UTC)</t>
+      <c r="K183" s="2" t="inlineStr">
+        <is>
+          <t>From previous run</t>
         </is>
       </c>
       <c r="L183" s="2" t="inlineStr">
@@ -12064,7 +12064,7 @@
       </c>
       <c r="M183" s="6" t="inlineStr">
         <is>
-          <t>https://ae.linkedin.com/jobs/view/senior-specialist-portfolio-management-at-mena-careers-4458066015?position=12&amp;pageNum=0&amp;refId=umynRMWB8laV9lcrAC5yvg%3D%3D&amp;trackingId=kbnf5IoX2jxOWD9%2Fe1UaKg%3D%3D</t>
+          <t>https://ae.linkedin.com/jobs/view/market-operations-analytics-specialist-%E2%80%94-institutional-at-confidential-4453037100?position=10&amp;pageNum=0&amp;refId=zJBbvwb5H0wsbJ5fs9ZTVw%3D%3D&amp;trackingId=ENnWCvoEQXOg1fXKuxlBug%3D%3D</t>
         </is>
       </c>
     </row>
@@ -12074,12 +12074,12 @@
       </c>
       <c r="B184" s="3" t="inlineStr">
         <is>
-          <t>Manager Logistics Performance</t>
+          <t>Quantitative Developer, Systematic Equities</t>
         </is>
       </c>
       <c r="C184" s="3" t="inlineStr">
         <is>
-          <t>talabat</t>
+          <t>Millennium</t>
         </is>
       </c>
       <c r="D184" s="3" t="inlineStr">
@@ -12089,25 +12089,25 @@
       </c>
       <c r="E184" s="2" t="inlineStr">
         <is>
-          <t>2026-08-28</t>
-        </is>
-      </c>
-      <c r="F184" s="8" t="n">
+          <t>2026-08-27</t>
+        </is>
+      </c>
+      <c r="F184" s="7" t="n">
         <v>0</v>
       </c>
-      <c r="G184" s="9" t="inlineStr">
+      <c r="G184" s="8" t="inlineStr">
         <is>
           <t>Below threshold</t>
         </is>
       </c>
       <c r="H184" s="3" t="inlineStr">
         <is>
-          <t>This is a commercial operations, logistics, and P&amp;L management role completely unrelated to data science, artificial intelligence, or Large Language Models. It requires background in marketplace operations, logistics, or quick-commerce rather than GenAI engineering.</t>
+          <t>This role is a quantitative software engineering position focused on low-latency trading infrastructure, C++/C# development, and execution systems for a hedge fund, which is entirely unrelated to the candidate's specialization in GenAI, LLMs, and agentic architectures.</t>
         </is>
       </c>
       <c r="I184" s="3" t="inlineStr">
         <is>
-          <t>Yes - German required (see JD for exact level)</t>
+          <t>Not stated in JD</t>
         </is>
       </c>
       <c r="J184" s="3" t="inlineStr">
@@ -12115,9 +12115,9 @@
           <t>Not stated in JD</t>
         </is>
       </c>
-      <c r="K184" s="7" t="inlineStr">
-        <is>
-          <t>New this run (2026-08-28 22:31 UTC)</t>
+      <c r="K184" s="2" t="inlineStr">
+        <is>
+          <t>From previous run</t>
         </is>
       </c>
       <c r="L184" s="2" t="inlineStr">
@@ -12127,7 +12127,7 @@
       </c>
       <c r="M184" s="6" t="inlineStr">
         <is>
-          <t>https://ae.linkedin.com/jobs/view/manager-logistics-performance-at-talabat-4440740657?position=7&amp;pageNum=0&amp;refId=umynRMWB8laV9lcrAC5yvg%3D%3D&amp;trackingId=lMQWp6LAUNLwXpGhMCpl2Q%3D%3D</t>
+          <t>https://ae.linkedin.com/jobs/view/quantitative-developer-systematic-equities-at-millennium-4290849018?position=6&amp;pageNum=0&amp;refId=zJBbvwb5H0wsbJ5fs9ZTVw%3D%3D&amp;trackingId=8TTWkyG2j%2F7MELtLSQ5VCA%3D%3D</t>
         </is>
       </c>
     </row>
@@ -12137,121 +12137,247 @@
       </c>
       <c r="B185" s="3" t="inlineStr">
         <is>
+          <t>Senior Specialist - Portfolio Management</t>
+        </is>
+      </c>
+      <c r="C185" s="3" t="inlineStr">
+        <is>
+          <t>MENA Careers</t>
+        </is>
+      </c>
+      <c r="D185" s="3" t="inlineStr">
+        <is>
+          <t>Dubai, Dubai, United Arab Emirates</t>
+        </is>
+      </c>
+      <c r="E185" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="F185" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="G185" s="8" t="inlineStr">
+        <is>
+          <t>Below threshold</t>
+        </is>
+      </c>
+      <c r="H185" s="3" t="inlineStr">
+        <is>
+          <t>This is a non-AI banking role focused on portfolio management, loan optimization, and regulatory capital compliance in Dubai requiring UAE nationality, which completely misaligns with the candidate's GenAI, LLM, and data science specialization.</t>
+        </is>
+      </c>
+      <c r="I185" s="3" t="inlineStr">
+        <is>
+          <t>Not stated in JD</t>
+        </is>
+      </c>
+      <c r="J185" s="3" t="inlineStr">
+        <is>
+          <t>Not stated in JD</t>
+        </is>
+      </c>
+      <c r="K185" s="2" t="inlineStr">
+        <is>
+          <t>From previous run</t>
+        </is>
+      </c>
+      <c r="L185" s="2" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="M185" s="6" t="inlineStr">
+        <is>
+          <t>https://ae.linkedin.com/jobs/view/senior-specialist-portfolio-management-at-mena-careers-4458066015?position=12&amp;pageNum=0&amp;refId=umynRMWB8laV9lcrAC5yvg%3D%3D&amp;trackingId=kbnf5IoX2jxOWD9%2Fe1UaKg%3D%3D</t>
+        </is>
+      </c>
+    </row>
+    <row r="186" ht="55" customHeight="1">
+      <c r="A186" s="2" t="n">
+        <v>185</v>
+      </c>
+      <c r="B186" s="3" t="inlineStr">
+        <is>
+          <t>Manager Logistics Performance</t>
+        </is>
+      </c>
+      <c r="C186" s="3" t="inlineStr">
+        <is>
+          <t>talabat</t>
+        </is>
+      </c>
+      <c r="D186" s="3" t="inlineStr">
+        <is>
+          <t>Dubai, Dubai, United Arab Emirates</t>
+        </is>
+      </c>
+      <c r="E186" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="F186" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="G186" s="8" t="inlineStr">
+        <is>
+          <t>Below threshold</t>
+        </is>
+      </c>
+      <c r="H186" s="3" t="inlineStr">
+        <is>
+          <t>This is a commercial operations, logistics, and P&amp;L management role completely unrelated to data science, artificial intelligence, or Large Language Models. It requires background in marketplace operations, logistics, or quick-commerce rather than GenAI engineering.</t>
+        </is>
+      </c>
+      <c r="I186" s="3" t="inlineStr">
+        <is>
+          <t>Yes - German required (see JD for exact level)</t>
+        </is>
+      </c>
+      <c r="J186" s="3" t="inlineStr">
+        <is>
+          <t>Not stated in JD</t>
+        </is>
+      </c>
+      <c r="K186" s="2" t="inlineStr">
+        <is>
+          <t>From previous run</t>
+        </is>
+      </c>
+      <c r="L186" s="2" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="M186" s="6" t="inlineStr">
+        <is>
+          <t>https://ae.linkedin.com/jobs/view/manager-logistics-performance-at-talabat-4440740657?position=7&amp;pageNum=0&amp;refId=umynRMWB8laV9lcrAC5yvg%3D%3D&amp;trackingId=lMQWp6LAUNLwXpGhMCpl2Q%3D%3D</t>
+        </is>
+      </c>
+    </row>
+    <row r="187" ht="55" customHeight="1">
+      <c r="A187" s="2" t="n">
+        <v>186</v>
+      </c>
+      <c r="B187" s="3" t="inlineStr">
+        <is>
           <t>Perception Engineer</t>
         </is>
       </c>
-      <c r="C185" s="3" t="inlineStr">
+      <c r="C187" s="3" t="inlineStr">
         <is>
           <t>Careernet</t>
         </is>
       </c>
-      <c r="D185" s="3" t="inlineStr">
+      <c r="D187" s="3" t="inlineStr">
         <is>
           <t>Ajman, Ajman Emirate, United Arab Emirates</t>
         </is>
       </c>
-      <c r="E185" s="2" t="inlineStr">
+      <c r="E187" s="2" t="inlineStr">
         <is>
           <t>2026-08-28</t>
         </is>
       </c>
-      <c r="F185" s="8" t="n">
+      <c r="F187" s="7" t="n">
         <v>0</v>
       </c>
-      <c r="G185" s="9" t="inlineStr">
-        <is>
-          <t>Below threshold</t>
-        </is>
-      </c>
-      <c r="H185" s="3" t="inlineStr">
+      <c r="G187" s="8" t="inlineStr">
+        <is>
+          <t>Below threshold</t>
+        </is>
+      </c>
+      <c r="H187" s="3" t="inlineStr">
         <is>
           <t>This is a hardware-focused Perception Engineer role centering on 2D/3D computer vision, camera calibration, point clouds, and robotics. It is completely unrelated to the candidate's specialization in GenAI, LLMs, RAG, and agentic AI.</t>
         </is>
       </c>
-      <c r="I185" s="3" t="inlineStr">
-        <is>
-          <t>Not stated in JD</t>
-        </is>
-      </c>
-      <c r="J185" s="3" t="inlineStr">
-        <is>
-          <t>Not stated in JD</t>
-        </is>
-      </c>
-      <c r="K185" s="7" t="inlineStr">
-        <is>
-          <t>New this run (2026-08-28 22:31 UTC)</t>
-        </is>
-      </c>
-      <c r="L185" s="2" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="M185" s="6" t="inlineStr">
+      <c r="I187" s="3" t="inlineStr">
+        <is>
+          <t>Not stated in JD</t>
+        </is>
+      </c>
+      <c r="J187" s="3" t="inlineStr">
+        <is>
+          <t>Not stated in JD</t>
+        </is>
+      </c>
+      <c r="K187" s="2" t="inlineStr">
+        <is>
+          <t>From previous run</t>
+        </is>
+      </c>
+      <c r="L187" s="2" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="M187" s="6" t="inlineStr">
         <is>
           <t>https://ae.linkedin.com/jobs/view/perception-engineer-at-careernet-4458403150?position=10&amp;pageNum=0&amp;refId=umynRMWB8laV9lcrAC5yvg%3D%3D&amp;trackingId=8I7i%2FeIdinpIC7lB70K7fg%3D%3D</t>
         </is>
       </c>
     </row>
-    <row r="186" ht="55" customHeight="1">
-      <c r="A186" s="10" t="n">
-        <v>185</v>
-      </c>
-      <c r="B186" s="11" t="inlineStr">
+    <row r="188" ht="55" customHeight="1">
+      <c r="A188" s="10" t="n">
+        <v>187</v>
+      </c>
+      <c r="B188" s="11" t="inlineStr">
         <is>
           <t>Data Scientist</t>
         </is>
       </c>
-      <c r="C186" s="11" t="inlineStr">
+      <c r="C188" s="11" t="inlineStr">
         <is>
           <t>Magno IT Recruitment</t>
         </is>
       </c>
-      <c r="D186" s="11" t="inlineStr">
+      <c r="D188" s="11" t="inlineStr">
         <is>
           <t>Amsterdam, North Holland, Netherlands</t>
         </is>
       </c>
-      <c r="E186" s="10" t="inlineStr">
+      <c r="E188" s="10" t="inlineStr">
         <is>
           <t>2026-08-26</t>
         </is>
       </c>
-      <c r="F186" s="10" t="n">
+      <c r="F188" s="10" t="n">
         <v>92</v>
       </c>
-      <c r="G186" s="12" t="inlineStr">
+      <c r="G188" s="12" t="inlineStr">
         <is>
           <t>APPLY</t>
         </is>
       </c>
-      <c r="H186" s="11" t="inlineStr">
+      <c r="H188" s="11" t="inlineStr">
         <is>
           <t>This Senior AI Engineer role is an exceptional technical match, focusing directly on LLMs, RAG, agentic AI applications, and semantic search which align precisely with the candidate's core specialization. The seniority level (Senior) fits the candidate's 10+ years of experience very well.</t>
         </is>
       </c>
-      <c r="I186" s="11" t="inlineStr">
-        <is>
-          <t>Not stated in JD</t>
-        </is>
-      </c>
-      <c r="J186" s="11" t="inlineStr">
-        <is>
-          <t>Not stated in JD</t>
-        </is>
-      </c>
-      <c r="K186" s="10" t="inlineStr">
-        <is>
-          <t>From previous run</t>
-        </is>
-      </c>
-      <c r="L186" s="10" t="inlineStr">
+      <c r="I188" s="11" t="inlineStr">
+        <is>
+          <t>Not stated in JD</t>
+        </is>
+      </c>
+      <c r="J188" s="11" t="inlineStr">
+        <is>
+          <t>Not stated in JD</t>
+        </is>
+      </c>
+      <c r="K188" s="10" t="inlineStr">
+        <is>
+          <t>From previous run</t>
+        </is>
+      </c>
+      <c r="L188" s="10" t="inlineStr">
         <is>
           <t>Closed</t>
         </is>
       </c>
-      <c r="M186" s="13" t="inlineStr">
+      <c r="M188" s="13" t="inlineStr">
         <is>
           <t>https://nl.linkedin.com/jobs/view/data-scientist-at-magno-it-recruitment-4448992517?position=9&amp;pageNum=0&amp;refId=AM27LUOGtvYOeETm648UMw%3D%3D&amp;trackingId=26%2BZzuSXNPWrglox%2BL4Wqg%3D%3D</t>
         </is>
@@ -12444,6 +12570,8 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M184" r:id="rId183"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M185" r:id="rId184"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M186" r:id="rId185"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M187" r:id="rId186"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M188" r:id="rId187"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update job tracker 2026-08-29 19:28 UTC
</commit_message>
<xml_diff>
--- a/data/job_matches.xlsx
+++ b/data/job_matches.xlsx
@@ -517,7 +517,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M188"/>
+  <dimension ref="A1:M190"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -8924,26 +8924,26 @@
       </c>
       <c r="B134" s="3" t="inlineStr">
         <is>
-          <t>Graphene Photonics Data Analyst (f/m/d)</t>
+          <t>Postdoctoral Researcher in AI for Testing and Threat Detection : Computer Science and Engineeing (CSE)-College of Engineering</t>
         </is>
       </c>
       <c r="C134" s="3" t="inlineStr">
         <is>
-          <t>Black Semiconductor</t>
+          <t>American University of Sharjah</t>
         </is>
       </c>
       <c r="D134" s="3" t="inlineStr">
         <is>
-          <t>Aachen, North Rhine-Westphalia, Germany</t>
+          <t>Sharjah, Sharjah Emirate, United Arab Emirates</t>
         </is>
       </c>
       <c r="E134" s="2" t="inlineStr">
         <is>
-          <t>2026-08-26</t>
+          <t>2026-08-29</t>
         </is>
       </c>
       <c r="F134" s="7" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="G134" s="8" t="inlineStr">
         <is>
@@ -8952,7 +8952,7 @@
       </c>
       <c r="H134" s="3" t="inlineStr">
         <is>
-          <t>This role is entirely focused on semiconductor hardware, graphene photonics, and physical data analysis, with zero relevance to the candidate's core specialization in Generative AI, LLMs, and agentic workflows.</t>
+          <t>This is a Postdoctoral Researcher role in an academic setting focused on reinforcement learning, formal verification, and threat detection, requiring a recent PhD, which completely mismatches the candidate's industry-focused Lead Data Scientist profile and 10+ years of corporate GenAI/RAG experience.</t>
         </is>
       </c>
       <c r="I134" s="3" t="inlineStr">
@@ -8965,9 +8965,9 @@
           <t>Not stated in JD</t>
         </is>
       </c>
-      <c r="K134" s="2" t="inlineStr">
-        <is>
-          <t>From previous run</t>
+      <c r="K134" s="9" t="inlineStr">
+        <is>
+          <t>New this run (2026-08-29 19:27 UTC)</t>
         </is>
       </c>
       <c r="L134" s="2" t="inlineStr">
@@ -8977,7 +8977,7 @@
       </c>
       <c r="M134" s="6" t="inlineStr">
         <is>
-          <t>https://de.linkedin.com/jobs/view/graphene-photonics-data-analyst-f-m-d-at-black-semiconductor-4459334621?position=26&amp;pageNum=0&amp;refId=T%2F0KkBXL%2Fl%2B5Iv5tUGTY7Q%3D%3D&amp;trackingId=KgQ01De6ChDgIN8UxnUvXg%3D%3D</t>
+          <t>https://ae.linkedin.com/jobs/view/postdoctoral-researcher-in-ai-for-testing-and-threat-detection-computer-science-and-engineeing-cse-college-of-engineering-at-american-university-of-sharjah-4423527619?position=2&amp;pageNum=0&amp;refId=ObYT%2FC%2FLT0LzMJUTwHqKZQ%3D%3D&amp;trackingId=FMQzyAWSKj5TyGLquO63tw%3D%3D</t>
         </is>
       </c>
     </row>
@@ -8987,26 +8987,26 @@
       </c>
       <c r="B135" s="3" t="inlineStr">
         <is>
-          <t>Financial Planning and Analysis Manager</t>
+          <t>Fitch Learning | Data Science Trainer, Associate Director - Dubai, UAE</t>
         </is>
       </c>
       <c r="C135" s="3" t="inlineStr">
         <is>
-          <t>Confidential Jobs</t>
+          <t>Fitch Ratings</t>
         </is>
       </c>
       <c r="D135" s="3" t="inlineStr">
         <is>
-          <t>Dubai, United Arab Emirates</t>
+          <t>Dubai, Dubai, United Arab Emirates</t>
         </is>
       </c>
       <c r="E135" s="2" t="inlineStr">
         <is>
-          <t>2026-08-26</t>
+          <t>2026-08-29</t>
         </is>
       </c>
       <c r="F135" s="7" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="G135" s="8" t="inlineStr">
         <is>
@@ -9015,7 +9015,7 @@
       </c>
       <c r="H135" s="3" t="inlineStr">
         <is>
-          <t>This Financial Planning and Analysis Manager role is entirely unrelated to data science, machine learning, or software engineering, focusing instead on corporate finance, budgeting, construction economics, and IFRS 15 accounting. There is a massive domain and seniority mismatch for an AI/GenAI Lead Data Scientist.</t>
+          <t>This role is for a Data Science Trainer focusing on teaching professional learners, which is a significant mismatch for a hands-on technical Lead Data Scientist specializing in GenAI engineering and agentic workflows.</t>
         </is>
       </c>
       <c r="I135" s="3" t="inlineStr">
@@ -9028,9 +9028,9 @@
           <t>Not stated in JD</t>
         </is>
       </c>
-      <c r="K135" s="2" t="inlineStr">
-        <is>
-          <t>From previous run</t>
+      <c r="K135" s="9" t="inlineStr">
+        <is>
+          <t>New this run (2026-08-29 19:27 UTC)</t>
         </is>
       </c>
       <c r="L135" s="2" t="inlineStr">
@@ -9040,7 +9040,7 @@
       </c>
       <c r="M135" s="6" t="inlineStr">
         <is>
-          <t>https://ae.linkedin.com/jobs/view/financial-planning-and-analysis-manager-at-confidential-jobs-4452594332?position=29&amp;pageNum=0&amp;refId=JBPPMgbgbAFzpV%2BDL5h2AA%3D%3D&amp;trackingId=KEfZVTEknZKckxH1vstrzQ%3D%3D</t>
+          <t>https://ae.linkedin.com/jobs/view/fitch-learning-data-science-trainer-associate-director-dubai-uae-at-fitch-ratings-4413826649?position=3&amp;pageNum=0&amp;refId=ObYT%2FC%2FLT0LzMJUTwHqKZQ%3D%3D&amp;trackingId=%2B6ZDB6n4%2BzrdaJhgz1Rx5A%3D%3D</t>
         </is>
       </c>
     </row>
@@ -9050,17 +9050,17 @@
       </c>
       <c r="B136" s="3" t="inlineStr">
         <is>
-          <t>Data QA Engineer</t>
+          <t>Graphene Photonics Data Analyst (f/m/d)</t>
         </is>
       </c>
       <c r="C136" s="3" t="inlineStr">
         <is>
-          <t>ClearGrid</t>
+          <t>Black Semiconductor</t>
         </is>
       </c>
       <c r="D136" s="3" t="inlineStr">
         <is>
-          <t>Dubai, Dubai, United Arab Emirates</t>
+          <t>Aachen, North Rhine-Westphalia, Germany</t>
         </is>
       </c>
       <c r="E136" s="2" t="inlineStr">
@@ -9078,7 +9078,7 @@
       </c>
       <c r="H136" s="3" t="inlineStr">
         <is>
-          <t>This role is a Data QA Engineer focused entirely on data quality, dbt testing, and warehouse reconciliation in a fintech/collections environment, lacking any Generative AI, LLM, or agentic specialization. Furthermore, the seniority requirement (2+ years) is well below the candidate's 10+ years as a Lead Data Scientist.</t>
+          <t>This role is entirely focused on semiconductor hardware, graphene photonics, and physical data analysis, with zero relevance to the candidate's core specialization in Generative AI, LLMs, and agentic workflows.</t>
         </is>
       </c>
       <c r="I136" s="3" t="inlineStr">
@@ -9103,7 +9103,7 @@
       </c>
       <c r="M136" s="6" t="inlineStr">
         <is>
-          <t>https://ae.linkedin.com/jobs/view/data-qa-engineer-at-cleargrid-4457980735?position=25&amp;pageNum=0&amp;refId=JBPPMgbgbAFzpV%2BDL5h2AA%3D%3D&amp;trackingId=RbMMQ6DAm%2FMomlqBLUM2IQ%3D%3D</t>
+          <t>https://de.linkedin.com/jobs/view/graphene-photonics-data-analyst-f-m-d-at-black-semiconductor-4459334621?position=26&amp;pageNum=0&amp;refId=T%2F0KkBXL%2Fl%2B5Iv5tUGTY7Q%3D%3D&amp;trackingId=KgQ01De6ChDgIN8UxnUvXg%3D%3D</t>
         </is>
       </c>
     </row>
@@ -9113,17 +9113,17 @@
       </c>
       <c r="B137" s="3" t="inlineStr">
         <is>
-          <t>OTR Planning Manager, Hub Delivery UAE , Hub Delivery</t>
+          <t>Financial Planning and Analysis Manager</t>
         </is>
       </c>
       <c r="C137" s="3" t="inlineStr">
         <is>
-          <t>Amazon</t>
+          <t>Confidential Jobs</t>
         </is>
       </c>
       <c r="D137" s="3" t="inlineStr">
         <is>
-          <t>Dubai, Dubai, United Arab Emirates</t>
+          <t>Dubai, United Arab Emirates</t>
         </is>
       </c>
       <c r="E137" s="2" t="inlineStr">
@@ -9141,7 +9141,7 @@
       </c>
       <c r="H137" s="3" t="inlineStr">
         <is>
-          <t>This operations and logistics management role is entirely unrelated to data science, machine learning, and Generative AI, focusing instead on supply chain planning and fleet management. Therefore, it is a very poor match for the candidate's core specialization.</t>
+          <t>This Financial Planning and Analysis Manager role is entirely unrelated to data science, machine learning, or software engineering, focusing instead on corporate finance, budgeting, construction economics, and IFRS 15 accounting. There is a massive domain and seniority mismatch for an AI/GenAI Lead Data Scientist.</t>
         </is>
       </c>
       <c r="I137" s="3" t="inlineStr">
@@ -9166,7 +9166,7 @@
       </c>
       <c r="M137" s="6" t="inlineStr">
         <is>
-          <t>https://ae.linkedin.com/jobs/view/otr-planning-manager-hub-delivery-uae-hub-delivery-at-amazon-4459184678?position=21&amp;pageNum=0&amp;refId=JBPPMgbgbAFzpV%2BDL5h2AA%3D%3D&amp;trackingId=bqoXqft%2BGFtLz05C2kL0FA%3D%3D</t>
+          <t>https://ae.linkedin.com/jobs/view/financial-planning-and-analysis-manager-at-confidential-jobs-4452594332?position=29&amp;pageNum=0&amp;refId=JBPPMgbgbAFzpV%2BDL5h2AA%3D%3D&amp;trackingId=KEfZVTEknZKckxH1vstrzQ%3D%3D</t>
         </is>
       </c>
     </row>
@@ -9176,12 +9176,12 @@
       </c>
       <c r="B138" s="3" t="inlineStr">
         <is>
-          <t>Senior Compensation Analyst</t>
+          <t>Data QA Engineer</t>
         </is>
       </c>
       <c r="C138" s="3" t="inlineStr">
         <is>
-          <t>Cartier</t>
+          <t>ClearGrid</t>
         </is>
       </c>
       <c r="D138" s="3" t="inlineStr">
@@ -9204,7 +9204,7 @@
       </c>
       <c r="H138" s="3" t="inlineStr">
         <is>
-          <t>This is a non-technical role focused strictly on compensation analysis, financial modeling, and advanced Excel simulation design within HR, which has no overlap with the candidate's core GenAI, LLM, or data science specialization.</t>
+          <t>This role is a Data QA Engineer focused entirely on data quality, dbt testing, and warehouse reconciliation in a fintech/collections environment, lacking any Generative AI, LLM, or agentic specialization. Furthermore, the seniority requirement (2+ years) is well below the candidate's 10+ years as a Lead Data Scientist.</t>
         </is>
       </c>
       <c r="I138" s="3" t="inlineStr">
@@ -9229,7 +9229,7 @@
       </c>
       <c r="M138" s="6" t="inlineStr">
         <is>
-          <t>https://ae.linkedin.com/jobs/view/senior-compensation-analyst-at-cartier-4448528069?position=20&amp;pageNum=0&amp;refId=JBPPMgbgbAFzpV%2BDL5h2AA%3D%3D&amp;trackingId=uU%2BxMpwsg7Xv71%2Fjk83xeg%3D%3D</t>
+          <t>https://ae.linkedin.com/jobs/view/data-qa-engineer-at-cleargrid-4457980735?position=25&amp;pageNum=0&amp;refId=JBPPMgbgbAFzpV%2BDL5h2AA%3D%3D&amp;trackingId=RbMMQ6DAm%2FMomlqBLUM2IQ%3D%3D</t>
         </is>
       </c>
     </row>
@@ -9239,12 +9239,12 @@
       </c>
       <c r="B139" s="3" t="inlineStr">
         <is>
-          <t>AI &amp; Data - BrightStar program - Part-Time For Students | UAE Nationals Only - Dubai</t>
+          <t>OTR Planning Manager, Hub Delivery UAE , Hub Delivery</t>
         </is>
       </c>
       <c r="C139" s="3" t="inlineStr">
         <is>
-          <t>Deloitte</t>
+          <t>Amazon</t>
         </is>
       </c>
       <c r="D139" s="3" t="inlineStr">
@@ -9267,7 +9267,7 @@
       </c>
       <c r="H139" s="3" t="inlineStr">
         <is>
-          <t>This student internship/part-time program is an extreme seniority mismatch for a Lead Data Scientist with 10+ years of experience. Furthermore, the role is strictly restricted to UAE Nationals and unrelated to the candidate's specialized GenAI and agentic AI expertise.</t>
+          <t>This operations and logistics management role is entirely unrelated to data science, machine learning, and Generative AI, focusing instead on supply chain planning and fleet management. Therefore, it is a very poor match for the candidate's core specialization.</t>
         </is>
       </c>
       <c r="I139" s="3" t="inlineStr">
@@ -9292,7 +9292,7 @@
       </c>
       <c r="M139" s="6" t="inlineStr">
         <is>
-          <t>https://ae.linkedin.com/jobs/view/ai-data-brightstar-program-part-time-for-students-uae-nationals-only-dubai-at-deloitte-4459165278?position=18&amp;pageNum=0&amp;refId=JBPPMgbgbAFzpV%2BDL5h2AA%3D%3D&amp;trackingId=rkeXlOzDBapH9BYwLoMUoA%3D%3D</t>
+          <t>https://ae.linkedin.com/jobs/view/otr-planning-manager-hub-delivery-uae-hub-delivery-at-amazon-4459184678?position=21&amp;pageNum=0&amp;refId=JBPPMgbgbAFzpV%2BDL5h2AA%3D%3D&amp;trackingId=bqoXqft%2BGFtLz05C2kL0FA%3D%3D</t>
         </is>
       </c>
     </row>
@@ -9302,12 +9302,12 @@
       </c>
       <c r="B140" s="3" t="inlineStr">
         <is>
-          <t>Junior Market Analyst - UAE National</t>
+          <t>Senior Compensation Analyst</t>
         </is>
       </c>
       <c r="C140" s="3" t="inlineStr">
         <is>
-          <t>Richemont</t>
+          <t>Cartier</t>
         </is>
       </c>
       <c r="D140" s="3" t="inlineStr">
@@ -9330,7 +9330,7 @@
       </c>
       <c r="H140" s="3" t="inlineStr">
         <is>
-          <t>This role is a junior market research and business development position focused on luxury retail intelligence in the MEIAT region, which is completely unrelated to data science, artificial intelligence, or the candidate's GenAI and LLM specialization.</t>
+          <t>This is a non-technical role focused strictly on compensation analysis, financial modeling, and advanced Excel simulation design within HR, which has no overlap with the candidate's core GenAI, LLM, or data science specialization.</t>
         </is>
       </c>
       <c r="I140" s="3" t="inlineStr">
@@ -9355,7 +9355,7 @@
       </c>
       <c r="M140" s="6" t="inlineStr">
         <is>
-          <t>https://ae.linkedin.com/jobs/view/junior-market-analyst-uae-national-at-richemont-4448527067?position=22&amp;pageNum=0&amp;refId=JBPPMgbgbAFzpV%2BDL5h2AA%3D%3D&amp;trackingId=fabWFpBqiTWxCuIFUXVosg%3D%3D</t>
+          <t>https://ae.linkedin.com/jobs/view/senior-compensation-analyst-at-cartier-4448528069?position=20&amp;pageNum=0&amp;refId=JBPPMgbgbAFzpV%2BDL5h2AA%3D%3D&amp;trackingId=uU%2BxMpwsg7Xv71%2Fjk83xeg%3D%3D</t>
         </is>
       </c>
     </row>
@@ -9365,12 +9365,12 @@
       </c>
       <c r="B141" s="3" t="inlineStr">
         <is>
-          <t>Data Analyst - (Advanced Excel expertise)</t>
+          <t>AI &amp; Data - BrightStar program - Part-Time For Students | UAE Nationals Only - Dubai</t>
         </is>
       </c>
       <c r="C141" s="3" t="inlineStr">
         <is>
-          <t>BigTapp Analytics</t>
+          <t>Deloitte</t>
         </is>
       </c>
       <c r="D141" s="3" t="inlineStr">
@@ -9393,7 +9393,7 @@
       </c>
       <c r="H141" s="3" t="inlineStr">
         <is>
-          <t>This is a Data Analyst role focused entirely on Advanced Excel, corporate tax data quality, and data validation, with no connection to the candidate's GenAI, LLM, or agentic AI specialization.</t>
+          <t>This student internship/part-time program is an extreme seniority mismatch for a Lead Data Scientist with 10+ years of experience. Furthermore, the role is strictly restricted to UAE Nationals and unrelated to the candidate's specialized GenAI and agentic AI expertise.</t>
         </is>
       </c>
       <c r="I141" s="3" t="inlineStr">
@@ -9418,7 +9418,7 @@
       </c>
       <c r="M141" s="6" t="inlineStr">
         <is>
-          <t>https://ae.linkedin.com/jobs/view/data-analyst-advanced-excel-expertise-at-bigtapp-analytics-4459194093?position=16&amp;pageNum=0&amp;refId=JBPPMgbgbAFzpV%2BDL5h2AA%3D%3D&amp;trackingId=vJ8ubhhJtvsWirwhmdkH%2BA%3D%3D</t>
+          <t>https://ae.linkedin.com/jobs/view/ai-data-brightstar-program-part-time-for-students-uae-nationals-only-dubai-at-deloitte-4459165278?position=18&amp;pageNum=0&amp;refId=JBPPMgbgbAFzpV%2BDL5h2AA%3D%3D&amp;trackingId=rkeXlOzDBapH9BYwLoMUoA%3D%3D</t>
         </is>
       </c>
     </row>
@@ -9428,17 +9428,17 @@
       </c>
       <c r="B142" s="3" t="inlineStr">
         <is>
-          <t>Junior Data Analyst</t>
+          <t>Junior Market Analyst - UAE National</t>
         </is>
       </c>
       <c r="C142" s="3" t="inlineStr">
         <is>
-          <t>Arabian Private Holdings</t>
+          <t>Richemont</t>
         </is>
       </c>
       <c r="D142" s="3" t="inlineStr">
         <is>
-          <t>Sharjah, Sharjah Emirate, United Arab Emirates</t>
+          <t>Dubai, Dubai, United Arab Emirates</t>
         </is>
       </c>
       <c r="E142" s="2" t="inlineStr">
@@ -9456,7 +9456,7 @@
       </c>
       <c r="H142" s="3" t="inlineStr">
         <is>
-          <t>This is a junior data analyst role focused on operational data interpretation, basic SQL/Excel database maintenance, and corporate strategy support, completely unrelated to the candidate's GenAI, LLMs, and agentic AI specialization. Additionally, there is a severe seniority mismatch as the role is strictly junior while the candidate is a Lead Data Scientist with 10+ years of experience.</t>
+          <t>This role is a junior market research and business development position focused on luxury retail intelligence in the MEIAT region, which is completely unrelated to data science, artificial intelligence, or the candidate's GenAI and LLM specialization.</t>
         </is>
       </c>
       <c r="I142" s="3" t="inlineStr">
@@ -9481,7 +9481,7 @@
       </c>
       <c r="M142" s="6" t="inlineStr">
         <is>
-          <t>https://ae.linkedin.com/jobs/view/junior-data-analyst-at-arabian-private-holdings-4457918646?position=11&amp;pageNum=0&amp;refId=JBPPMgbgbAFzpV%2BDL5h2AA%3D%3D&amp;trackingId=n3OKFNsTAywRSCMqHYFmlg%3D%3D</t>
+          <t>https://ae.linkedin.com/jobs/view/junior-market-analyst-uae-national-at-richemont-4448527067?position=22&amp;pageNum=0&amp;refId=JBPPMgbgbAFzpV%2BDL5h2AA%3D%3D&amp;trackingId=fabWFpBqiTWxCuIFUXVosg%3D%3D</t>
         </is>
       </c>
     </row>
@@ -9491,17 +9491,17 @@
       </c>
       <c r="B143" s="3" t="inlineStr">
         <is>
-          <t>Data Analyst – Social Support Operations - UAE National</t>
+          <t>Data Analyst - (Advanced Excel expertise)</t>
         </is>
       </c>
       <c r="C143" s="3" t="inlineStr">
         <is>
-          <t>Ministry of Community Empowerment</t>
+          <t>BigTapp Analytics</t>
         </is>
       </c>
       <c r="D143" s="3" t="inlineStr">
         <is>
-          <t>Dubai, United Arab Emirates</t>
+          <t>Dubai, Dubai, United Arab Emirates</t>
         </is>
       </c>
       <c r="E143" s="2" t="inlineStr">
@@ -9519,7 +9519,7 @@
       </c>
       <c r="H143" s="3" t="inlineStr">
         <is>
-          <t>This role is a data analyst position focused on BI, Power BI dashboards, SQL, and social support operations, which is completely unrelated to the candidate's core GenAI, LLMs, and agentic AI specialization. Additionally, it specifies a nationality requirement.</t>
+          <t>This is a Data Analyst role focused entirely on Advanced Excel, corporate tax data quality, and data validation, with no connection to the candidate's GenAI, LLM, or agentic AI specialization.</t>
         </is>
       </c>
       <c r="I143" s="3" t="inlineStr">
@@ -9544,7 +9544,7 @@
       </c>
       <c r="M143" s="6" t="inlineStr">
         <is>
-          <t>https://ae.linkedin.com/jobs/view/data-analyst-%E2%80%93-social-support-operations-uae-national-at-ministry-of-community-empowerment-4459118725?position=4&amp;pageNum=0&amp;refId=JBPPMgbgbAFzpV%2BDL5h2AA%3D%3D&amp;trackingId=q%2FHUZ0XJHF5eY2WSwIWmAg%3D%3D</t>
+          <t>https://ae.linkedin.com/jobs/view/data-analyst-advanced-excel-expertise-at-bigtapp-analytics-4459194093?position=16&amp;pageNum=0&amp;refId=JBPPMgbgbAFzpV%2BDL5h2AA%3D%3D&amp;trackingId=vJ8ubhhJtvsWirwhmdkH%2BA%3D%3D</t>
         </is>
       </c>
     </row>
@@ -9554,17 +9554,17 @@
       </c>
       <c r="B144" s="3" t="inlineStr">
         <is>
-          <t>Graduate - Data Scientist إماراتيين (خلاصة القيد)</t>
+          <t>Junior Data Analyst</t>
         </is>
       </c>
       <c r="C144" s="3" t="inlineStr">
         <is>
-          <t>AECOM</t>
+          <t>Arabian Private Holdings</t>
         </is>
       </c>
       <c r="D144" s="3" t="inlineStr">
         <is>
-          <t>Dubai, Dubai, United Arab Emirates</t>
+          <t>Sharjah, Sharjah Emirate, United Arab Emirates</t>
         </is>
       </c>
       <c r="E144" s="2" t="inlineStr">
@@ -9582,7 +9582,7 @@
       </c>
       <c r="H144" s="3" t="inlineStr">
         <is>
-          <t>This is a graduate/entry-level program designed specifically for recent graduates (2024-2026) and UAE Nationals, representing a severe seniority and eligibility mismatch for a Lead Data Scientist with 10+ years of experience. Furthermore, the role focuses on construction digital tools, cost management, and general data analytics rather than the candidate's core GenAI, LLMs, and agentic AI specialization.</t>
+          <t>This is a junior data analyst role focused on operational data interpretation, basic SQL/Excel database maintenance, and corporate strategy support, completely unrelated to the candidate's GenAI, LLMs, and agentic AI specialization. Additionally, there is a severe seniority mismatch as the role is strictly junior while the candidate is a Lead Data Scientist with 10+ years of experience.</t>
         </is>
       </c>
       <c r="I144" s="3" t="inlineStr">
@@ -9607,7 +9607,7 @@
       </c>
       <c r="M144" s="6" t="inlineStr">
         <is>
-          <t>https://ae.linkedin.com/jobs/view/graduate-data-scientist-%D8%A5%D9%85%D8%A7%D8%B1%D8%A7%D8%AA%D9%8A%D9%8A%D9%86-%D8%AE%D9%84%D8%A7%D8%B5%D8%A9-%D8%A7%D9%84%D9%82%D9%8A%D8%AF-at-aecom-4457915285?position=1&amp;pageNum=0&amp;refId=JBPPMgbgbAFzpV%2BDL5h2AA%3D%3D&amp;trackingId=deUfOEFHstE7TEtandLeTg%3D%3D</t>
+          <t>https://ae.linkedin.com/jobs/view/junior-data-analyst-at-arabian-private-holdings-4457918646?position=11&amp;pageNum=0&amp;refId=JBPPMgbgbAFzpV%2BDL5h2AA%3D%3D&amp;trackingId=n3OKFNsTAywRSCMqHYFmlg%3D%3D</t>
         </is>
       </c>
     </row>
@@ -9617,17 +9617,17 @@
       </c>
       <c r="B145" s="3" t="inlineStr">
         <is>
-          <t>Quantitative Researcher, Quantitative Strategies</t>
+          <t>Data Analyst – Social Support Operations - UAE National</t>
         </is>
       </c>
       <c r="C145" s="3" t="inlineStr">
         <is>
-          <t>Millennium</t>
+          <t>Ministry of Community Empowerment</t>
         </is>
       </c>
       <c r="D145" s="3" t="inlineStr">
         <is>
-          <t>Dubai, Dubai, United Arab Emirates</t>
+          <t>Dubai, United Arab Emirates</t>
         </is>
       </c>
       <c r="E145" s="2" t="inlineStr">
@@ -9645,7 +9645,7 @@
       </c>
       <c r="H145" s="3" t="inlineStr">
         <is>
-          <t>This role focuses entirely on quantitative finance, statistical modeling, and systematic equity trading in Asian markets, which has no overlap with the candidate's core specialization in Generative AI, LLMs, and agentic systems. Additionally, the domain requires specific desk quant trading experience that is absent from the candidate's profile.</t>
+          <t>This role is a data analyst position focused on BI, Power BI dashboards, SQL, and social support operations, which is completely unrelated to the candidate's core GenAI, LLMs, and agentic AI specialization. Additionally, it specifies a nationality requirement.</t>
         </is>
       </c>
       <c r="I145" s="3" t="inlineStr">
@@ -9670,7 +9670,7 @@
       </c>
       <c r="M145" s="6" t="inlineStr">
         <is>
-          <t>https://ae.linkedin.com/jobs/view/quantitative-researcher-quantitative-strategies-at-millennium-4439427782?position=2&amp;pageNum=0&amp;refId=JBPPMgbgbAFzpV%2BDL5h2AA%3D%3D&amp;trackingId=uptfSAbwEngBw3yrsrQehg%3D%3D</t>
+          <t>https://ae.linkedin.com/jobs/view/data-analyst-%E2%80%93-social-support-operations-uae-national-at-ministry-of-community-empowerment-4459118725?position=4&amp;pageNum=0&amp;refId=JBPPMgbgbAFzpV%2BDL5h2AA%3D%3D&amp;trackingId=q%2FHUZ0XJHF5eY2WSwIWmAg%3D%3D</t>
         </is>
       </c>
     </row>
@@ -9680,12 +9680,12 @@
       </c>
       <c r="B146" s="3" t="inlineStr">
         <is>
-          <t>Analyst I - Advisory</t>
+          <t>Graduate - Data Scientist إماراتيين (خلاصة القيد)</t>
         </is>
       </c>
       <c r="C146" s="3" t="inlineStr">
         <is>
-          <t>Marsh Risk</t>
+          <t>AECOM</t>
         </is>
       </c>
       <c r="D146" s="3" t="inlineStr">
@@ -9708,7 +9708,7 @@
       </c>
       <c r="H146" s="3" t="inlineStr">
         <is>
-          <t>This is a fresh-graduate/entry-level role for recent graduates that focuses heavily on risk engineering and basic internal digitalization using Excel and Microsoft tools, which is far below the candidate's 10+ years of experience as a Lead Data Scientist specializing in advanced GenAI and agentic systems.</t>
+          <t>This is a graduate/entry-level program designed specifically for recent graduates (2024-2026) and UAE Nationals, representing a severe seniority and eligibility mismatch for a Lead Data Scientist with 10+ years of experience. Furthermore, the role focuses on construction digital tools, cost management, and general data analytics rather than the candidate's core GenAI, LLMs, and agentic AI specialization.</t>
         </is>
       </c>
       <c r="I146" s="3" t="inlineStr">
@@ -9733,7 +9733,7 @@
       </c>
       <c r="M146" s="6" t="inlineStr">
         <is>
-          <t>https://ae.linkedin.com/jobs/view/analyst-i-advisory-at-marsh-risk-4459165267?position=3&amp;pageNum=0&amp;refId=JBPPMgbgbAFzpV%2BDL5h2AA%3D%3D&amp;trackingId=NpomdoqDoXrgLAw8%2BZjEQA%3D%3D</t>
+          <t>https://ae.linkedin.com/jobs/view/graduate-data-scientist-%D8%A5%D9%85%D8%A7%D8%B1%D8%A7%D8%AA%D9%8A%D9%8A%D9%86-%D8%AE%D9%84%D8%A7%D8%B5%D8%A9-%D8%A7%D9%84%D9%82%D9%8A%D8%AF-at-aecom-4457915285?position=1&amp;pageNum=0&amp;refId=JBPPMgbgbAFzpV%2BDL5h2AA%3D%3D&amp;trackingId=deUfOEFHstE7TEtandLeTg%3D%3D</t>
         </is>
       </c>
     </row>
@@ -9743,17 +9743,17 @@
       </c>
       <c r="B147" s="3" t="inlineStr">
         <is>
-          <t>Demand Planner (f/m/x)</t>
+          <t>Quantitative Researcher, Quantitative Strategies</t>
         </is>
       </c>
       <c r="C147" s="3" t="inlineStr">
         <is>
-          <t>HelloFresh</t>
+          <t>Millennium</t>
         </is>
       </c>
       <c r="D147" s="3" t="inlineStr">
         <is>
-          <t>Amsterdam, North Holland, Netherlands</t>
+          <t>Dubai, Dubai, United Arab Emirates</t>
         </is>
       </c>
       <c r="E147" s="2" t="inlineStr">
@@ -9771,7 +9771,7 @@
       </c>
       <c r="H147" s="3" t="inlineStr">
         <is>
-          <t>This is a supply chain demand planning role requiring 2-3 years of experience in business forecasting, which is completely unrelated to the candidate's specialization in Generative AI, LLMs, and agentic systems. Furthermore, there is a severe seniority mismatch as the candidate is a Lead Data Scientist with 10+ years of experience.</t>
+          <t>This role focuses entirely on quantitative finance, statistical modeling, and systematic equity trading in Asian markets, which has no overlap with the candidate's core specialization in Generative AI, LLMs, and agentic systems. Additionally, the domain requires specific desk quant trading experience that is absent from the candidate's profile.</t>
         </is>
       </c>
       <c r="I147" s="3" t="inlineStr">
@@ -9796,7 +9796,7 @@
       </c>
       <c r="M147" s="6" t="inlineStr">
         <is>
-          <t>https://nl.linkedin.com/jobs/view/demand-planner-f-m-x-at-hellofresh-4459621163?position=29&amp;pageNum=0&amp;refId=AM27LUOGtvYOeETm648UMw%3D%3D&amp;trackingId=ScTLY%2B93hMGSjD1GtPlxQw%3D%3D</t>
+          <t>https://ae.linkedin.com/jobs/view/quantitative-researcher-quantitative-strategies-at-millennium-4439427782?position=2&amp;pageNum=0&amp;refId=JBPPMgbgbAFzpV%2BDL5h2AA%3D%3D&amp;trackingId=uptfSAbwEngBw3yrsrQehg%3D%3D</t>
         </is>
       </c>
     </row>
@@ -9806,17 +9806,17 @@
       </c>
       <c r="B148" s="3" t="inlineStr">
         <is>
-          <t>Traineeship Data Analytics</t>
+          <t>Analyst I - Advisory</t>
         </is>
       </c>
       <c r="C148" s="3" t="inlineStr">
         <is>
-          <t>Breinstein</t>
+          <t>Marsh Risk</t>
         </is>
       </c>
       <c r="D148" s="3" t="inlineStr">
         <is>
-          <t>Groningen, Netherlands</t>
+          <t>Dubai, Dubai, United Arab Emirates</t>
         </is>
       </c>
       <c r="E148" s="2" t="inlineStr">
@@ -9834,7 +9834,7 @@
       </c>
       <c r="H148" s="3" t="inlineStr">
         <is>
-          <t>This is a junior/graduate-level traineeship requiring Dutch language proficiency, which represents a severe mismatch with the candidate's 10+ years of senior experience and Generative AI/LLM specialization.</t>
+          <t>This is a fresh-graduate/entry-level role for recent graduates that focuses heavily on risk engineering and basic internal digitalization using Excel and Microsoft tools, which is far below the candidate's 10+ years of experience as a Lead Data Scientist specializing in advanced GenAI and agentic systems.</t>
         </is>
       </c>
       <c r="I148" s="3" t="inlineStr">
@@ -9859,7 +9859,7 @@
       </c>
       <c r="M148" s="6" t="inlineStr">
         <is>
-          <t>https://nl.linkedin.com/jobs/view/traineeship-data-analytics-at-breinstein-4457240429?position=18&amp;pageNum=0&amp;refId=AM27LUOGtvYOeETm648UMw%3D%3D&amp;trackingId=09Fo%2Bt8pd71ON%2B4bzhNIXw%3D%3D</t>
+          <t>https://ae.linkedin.com/jobs/view/analyst-i-advisory-at-marsh-risk-4459165267?position=3&amp;pageNum=0&amp;refId=JBPPMgbgbAFzpV%2BDL5h2AA%3D%3D&amp;trackingId=NpomdoqDoXrgLAw8%2BZjEQA%3D%3D</t>
         </is>
       </c>
     </row>
@@ -9869,17 +9869,17 @@
       </c>
       <c r="B149" s="3" t="inlineStr">
         <is>
-          <t>Økonom til finansielle data om pensionssektoren og investeringsfonde i Nationalbanken</t>
+          <t>Demand Planner (f/m/x)</t>
         </is>
       </c>
       <c r="C149" s="3" t="inlineStr">
         <is>
-          <t>Altandetlige.dk</t>
+          <t>HelloFresh</t>
         </is>
       </c>
       <c r="D149" s="3" t="inlineStr">
         <is>
-          <t>Copenhagen, Capital Region of Denmark, Denmark</t>
+          <t>Amsterdam, North Holland, Netherlands</t>
         </is>
       </c>
       <c r="E149" s="2" t="inlineStr">
@@ -9897,7 +9897,7 @@
       </c>
       <c r="H149" s="3" t="inlineStr">
         <is>
-          <t>This is a non-technical economics and financial statistics role at Denmark's central bank focusing on pension funds and investment data, which is completely unrelated to the candidate's specialization in Generative AI, LLMs, and agentic systems.</t>
+          <t>This is a supply chain demand planning role requiring 2-3 years of experience in business forecasting, which is completely unrelated to the candidate's specialization in Generative AI, LLMs, and agentic systems. Furthermore, there is a severe seniority mismatch as the candidate is a Lead Data Scientist with 10+ years of experience.</t>
         </is>
       </c>
       <c r="I149" s="3" t="inlineStr">
@@ -9922,7 +9922,7 @@
       </c>
       <c r="M149" s="6" t="inlineStr">
         <is>
-          <t>https://dk.linkedin.com/jobs/view/%C3%B8konom-til-finansielle-data-om-pensionssektoren-og-investeringsfonde-i-nationalbanken-at-altandetlige-dk-4459168468?position=25&amp;pageNum=0&amp;refId=Pb2EWWHgR9a7i9BrLIIg7g%3D%3D&amp;trackingId=%2BEekg%2B%2FvA%2BH0hxU4LsvJ5w%3D%3D</t>
+          <t>https://nl.linkedin.com/jobs/view/demand-planner-f-m-x-at-hellofresh-4459621163?position=29&amp;pageNum=0&amp;refId=AM27LUOGtvYOeETm648UMw%3D%3D&amp;trackingId=ScTLY%2B93hMGSjD1GtPlxQw%3D%3D</t>
         </is>
       </c>
     </row>
@@ -9932,17 +9932,17 @@
       </c>
       <c r="B150" s="3" t="inlineStr">
         <is>
-          <t>Lead Trading Strategist</t>
+          <t>Traineeship Data Analytics</t>
         </is>
       </c>
       <c r="C150" s="3" t="inlineStr">
         <is>
-          <t>Ørsted</t>
+          <t>Breinstein</t>
         </is>
       </c>
       <c r="D150" s="3" t="inlineStr">
         <is>
-          <t>Gentofte, Capital Region of Denmark, Denmark</t>
+          <t>Groningen, Netherlands</t>
         </is>
       </c>
       <c r="E150" s="2" t="inlineStr">
@@ -9960,7 +9960,7 @@
       </c>
       <c r="H150" s="3" t="inlineStr">
         <is>
-          <t>This is a quantitative energy trading and fundamental market analysis role requiring deep domain expertise in European power markets and commodities trading, which is completely unrelated to the candidate's core GenAI, LLM, and data science specialization.</t>
+          <t>This is a junior/graduate-level traineeship requiring Dutch language proficiency, which represents a severe mismatch with the candidate's 10+ years of senior experience and Generative AI/LLM specialization.</t>
         </is>
       </c>
       <c r="I150" s="3" t="inlineStr">
@@ -9985,7 +9985,7 @@
       </c>
       <c r="M150" s="6" t="inlineStr">
         <is>
-          <t>https://dk.linkedin.com/jobs/view/lead-trading-strategist-at-%C3%B8rsted-4439179684?position=21&amp;pageNum=0&amp;refId=Pb2EWWHgR9a7i9BrLIIg7g%3D%3D&amp;trackingId=LxVb1rg9c7QiaOEs5%2BY%2FTw%3D%3D</t>
+          <t>https://nl.linkedin.com/jobs/view/traineeship-data-analytics-at-breinstein-4457240429?position=18&amp;pageNum=0&amp;refId=AM27LUOGtvYOeETm648UMw%3D%3D&amp;trackingId=09Fo%2Bt8pd71ON%2B4bzhNIXw%3D%3D</t>
         </is>
       </c>
     </row>
@@ -9995,12 +9995,12 @@
       </c>
       <c r="B151" s="3" t="inlineStr">
         <is>
-          <t>Analytikere med flair for databehandling til PET's kontraspionageindsats mod Rusland</t>
+          <t>Økonom til finansielle data om pensionssektoren og investeringsfonde i Nationalbanken</t>
         </is>
       </c>
       <c r="C151" s="3" t="inlineStr">
         <is>
-          <t>Politiets Efterretningstjeneste (PET)</t>
+          <t>Altandetlige.dk</t>
         </is>
       </c>
       <c r="D151" s="3" t="inlineStr">
@@ -10023,7 +10023,7 @@
       </c>
       <c r="H151" s="3" t="inlineStr">
         <is>
-          <t>This is a national security intelligence and counter-espionage analyst role entirely unrelated to data science, artificial intelligence, LLMs, or software engineering. It focuses on intelligence operations and telecommunications data processing rather than the candidate's core Generative AI specialization.</t>
+          <t>This is a non-technical economics and financial statistics role at Denmark's central bank focusing on pension funds and investment data, which is completely unrelated to the candidate's specialization in Generative AI, LLMs, and agentic systems.</t>
         </is>
       </c>
       <c r="I151" s="3" t="inlineStr">
@@ -10048,7 +10048,7 @@
       </c>
       <c r="M151" s="6" t="inlineStr">
         <is>
-          <t>https://dk.linkedin.com/jobs/view/analytikere-med-flair-for-databehandling-til-pet-s-kontraspionageindsats-mod-rusland-at-politiets-efterretningstjeneste-pet-4457295379?position=17&amp;pageNum=0&amp;refId=Pb2EWWHgR9a7i9BrLIIg7g%3D%3D&amp;trackingId=jfzRay2PLGqzZJAC5yISBA%3D%3D</t>
+          <t>https://dk.linkedin.com/jobs/view/%C3%B8konom-til-finansielle-data-om-pensionssektoren-og-investeringsfonde-i-nationalbanken-at-altandetlige-dk-4459168468?position=25&amp;pageNum=0&amp;refId=Pb2EWWHgR9a7i9BrLIIg7g%3D%3D&amp;trackingId=%2BEekg%2B%2FvA%2BH0hxU4LsvJ5w%3D%3D</t>
         </is>
       </c>
     </row>
@@ -10058,17 +10058,17 @@
       </c>
       <c r="B152" s="3" t="inlineStr">
         <is>
-          <t>BI Specialist - turn healthcare data into better care decisions</t>
+          <t>Lead Trading Strategist</t>
         </is>
       </c>
       <c r="C152" s="3" t="inlineStr">
         <is>
-          <t>Systematic</t>
+          <t>Ørsted</t>
         </is>
       </c>
       <c r="D152" s="3" t="inlineStr">
         <is>
-          <t>Aarhus, Central Denmark Region, Denmark</t>
+          <t>Gentofte, Capital Region of Denmark, Denmark</t>
         </is>
       </c>
       <c r="E152" s="2" t="inlineStr">
@@ -10086,7 +10086,7 @@
       </c>
       <c r="H152" s="3" t="inlineStr">
         <is>
-          <t>This role is for a BI Specialist focusing on healthcare data systems, SQL, T-SQL, DAX, and client communication, which is completely unrelated to the candidate's core specialization in Generative AI, LLMs, and agentic AI systems. Additionally, it requires proficiency in Danish.</t>
+          <t>This is a quantitative energy trading and fundamental market analysis role requiring deep domain expertise in European power markets and commodities trading, which is completely unrelated to the candidate's core GenAI, LLM, and data science specialization.</t>
         </is>
       </c>
       <c r="I152" s="3" t="inlineStr">
@@ -10111,7 +10111,7 @@
       </c>
       <c r="M152" s="6" t="inlineStr">
         <is>
-          <t>https://dk.linkedin.com/jobs/view/bi-specialist-turn-healthcare-data-into-better-care-decisions-at-systematic-4449000390?position=13&amp;pageNum=0&amp;refId=Pb2EWWHgR9a7i9BrLIIg7g%3D%3D&amp;trackingId=C4YvYCcgfvLE1Lup1m630A%3D%3D</t>
+          <t>https://dk.linkedin.com/jobs/view/lead-trading-strategist-at-%C3%B8rsted-4439179684?position=21&amp;pageNum=0&amp;refId=Pb2EWWHgR9a7i9BrLIIg7g%3D%3D&amp;trackingId=LxVb1rg9c7QiaOEs5%2BY%2FTw%3D%3D</t>
         </is>
       </c>
     </row>
@@ -10121,17 +10121,17 @@
       </c>
       <c r="B153" s="3" t="inlineStr">
         <is>
-          <t>Demand Planner (f/m/x)</t>
+          <t>Analytikere med flair for databehandling til PET's kontraspionageindsats mod Rusland</t>
         </is>
       </c>
       <c r="C153" s="3" t="inlineStr">
         <is>
-          <t>HelloFresh</t>
+          <t>Politiets Efterretningstjeneste (PET)</t>
         </is>
       </c>
       <c r="D153" s="3" t="inlineStr">
         <is>
-          <t>Copenhagen Municipality, Capital Region of Denmark, Denmark</t>
+          <t>Copenhagen, Capital Region of Denmark, Denmark</t>
         </is>
       </c>
       <c r="E153" s="2" t="inlineStr">
@@ -10149,7 +10149,7 @@
       </c>
       <c r="H153" s="3" t="inlineStr">
         <is>
-          <t>This is a non-AI supply chain demand planning role focused on SQL, logistics, and forecasting metrics like MAPE, which is completely unrelated to the candidate's core GenAI, LLM, and agentic AI specialization.</t>
+          <t>This is a national security intelligence and counter-espionage analyst role entirely unrelated to data science, artificial intelligence, LLMs, or software engineering. It focuses on intelligence operations and telecommunications data processing rather than the candidate's core Generative AI specialization.</t>
         </is>
       </c>
       <c r="I153" s="3" t="inlineStr">
@@ -10174,7 +10174,7 @@
       </c>
       <c r="M153" s="6" t="inlineStr">
         <is>
-          <t>https://dk.linkedin.com/jobs/view/demand-planner-f-m-x-at-hellofresh-4459625132?position=6&amp;pageNum=0&amp;refId=Pb2EWWHgR9a7i9BrLIIg7g%3D%3D&amp;trackingId=%2FDvrjQmxzWwgXh6GBB3pqA%3D%3D</t>
+          <t>https://dk.linkedin.com/jobs/view/analytikere-med-flair-for-databehandling-til-pet-s-kontraspionageindsats-mod-rusland-at-politiets-efterretningstjeneste-pet-4457295379?position=17&amp;pageNum=0&amp;refId=Pb2EWWHgR9a7i9BrLIIg7g%3D%3D&amp;trackingId=jfzRay2PLGqzZJAC5yISBA%3D%3D</t>
         </is>
       </c>
     </row>
@@ -10184,17 +10184,17 @@
       </c>
       <c r="B154" s="3" t="inlineStr">
         <is>
-          <t>Senior Analyst - Market Intelligence (Trade &amp; Commodities)</t>
+          <t>BI Specialist - turn healthcare data into better care decisions</t>
         </is>
       </c>
       <c r="C154" s="3" t="inlineStr">
         <is>
-          <t>Robert Walters</t>
+          <t>Systematic</t>
         </is>
       </c>
       <c r="D154" s="3" t="inlineStr">
         <is>
-          <t>Abu Dhabi, Abu Dhabi Emirate, United Arab Emirates</t>
+          <t>Aarhus, Central Denmark Region, Denmark</t>
         </is>
       </c>
       <c r="E154" s="2" t="inlineStr">
@@ -10212,7 +10212,7 @@
       </c>
       <c r="H154" s="3" t="inlineStr">
         <is>
-          <t>This is a non-technical role focusing on market intelligence, trade flows, and supply chain analysis requiring Arabic fluency, which has no overlap with the candidate's core GenAI, LLMs, and agentic AI specialization.</t>
+          <t>This role is for a BI Specialist focusing on healthcare data systems, SQL, T-SQL, DAX, and client communication, which is completely unrelated to the candidate's core specialization in Generative AI, LLMs, and agentic AI systems. Additionally, it requires proficiency in Danish.</t>
         </is>
       </c>
       <c r="I154" s="3" t="inlineStr">
@@ -10237,7 +10237,7 @@
       </c>
       <c r="M154" s="6" t="inlineStr">
         <is>
-          <t>https://ae.linkedin.com/jobs/view/senior-analyst-market-intelligence-trade-commodities-at-robert-walters-4457222382?position=30&amp;pageNum=0&amp;refId=W92GFmCMxOQHlXfyvp17MQ%3D%3D&amp;trackingId=JK2lIzdStMxW3Rb1o%2FxSgQ%3D%3D</t>
+          <t>https://dk.linkedin.com/jobs/view/bi-specialist-turn-healthcare-data-into-better-care-decisions-at-systematic-4449000390?position=13&amp;pageNum=0&amp;refId=Pb2EWWHgR9a7i9BrLIIg7g%3D%3D&amp;trackingId=C4YvYCcgfvLE1Lup1m630A%3D%3D</t>
         </is>
       </c>
     </row>
@@ -10247,17 +10247,17 @@
       </c>
       <c r="B155" s="3" t="inlineStr">
         <is>
-          <t>AI &amp; Data - BrightStar program - Part-Time For Students | UAE Nationals Only - Dubai</t>
+          <t>Demand Planner (f/m/x)</t>
         </is>
       </c>
       <c r="C155" s="3" t="inlineStr">
         <is>
-          <t>Deloitte</t>
+          <t>HelloFresh</t>
         </is>
       </c>
       <c r="D155" s="3" t="inlineStr">
         <is>
-          <t>Abu Dhabi, Abu Dhabi Emirate, United Arab Emirates</t>
+          <t>Copenhagen Municipality, Capital Region of Denmark, Denmark</t>
         </is>
       </c>
       <c r="E155" s="2" t="inlineStr">
@@ -10275,7 +10275,7 @@
       </c>
       <c r="H155" s="3" t="inlineStr">
         <is>
-          <t>This is a student/internship program ('Part-Time For Students') restricted to UAE Nationals only, representing a severe seniority and eligibility mismatch for a Lead Data Scientist with 10 years of experience.</t>
+          <t>This is a non-AI supply chain demand planning role focused on SQL, logistics, and forecasting metrics like MAPE, which is completely unrelated to the candidate's core GenAI, LLM, and agentic AI specialization.</t>
         </is>
       </c>
       <c r="I155" s="3" t="inlineStr">
@@ -10300,7 +10300,7 @@
       </c>
       <c r="M155" s="6" t="inlineStr">
         <is>
-          <t>https://ae.linkedin.com/jobs/view/ai-data-brightstar-program-part-time-for-students-uae-nationals-only-dubai-at-deloitte-4459166169?position=29&amp;pageNum=0&amp;refId=W92GFmCMxOQHlXfyvp17MQ%3D%3D&amp;trackingId=eJo5yKx6Zm7GgBBf0abvaA%3D%3D</t>
+          <t>https://dk.linkedin.com/jobs/view/demand-planner-f-m-x-at-hellofresh-4459625132?position=6&amp;pageNum=0&amp;refId=Pb2EWWHgR9a7i9BrLIIg7g%3D%3D&amp;trackingId=%2FDvrjQmxzWwgXh6GBB3pqA%3D%3D</t>
         </is>
       </c>
     </row>
@@ -10310,17 +10310,17 @@
       </c>
       <c r="B156" s="3" t="inlineStr">
         <is>
-          <t>SAS Analyst</t>
+          <t>Senior Analyst - Market Intelligence (Trade &amp; Commodities)</t>
         </is>
       </c>
       <c r="C156" s="3" t="inlineStr">
         <is>
-          <t>One75mb HRM Pvt Ltd.</t>
+          <t>Robert Walters</t>
         </is>
       </c>
       <c r="D156" s="3" t="inlineStr">
         <is>
-          <t>Abu Dhabi Emirate, United Arab Emirates</t>
+          <t>Abu Dhabi, Abu Dhabi Emirate, United Arab Emirates</t>
         </is>
       </c>
       <c r="E156" s="2" t="inlineStr">
@@ -10338,7 +10338,7 @@
       </c>
       <c r="H156" s="3" t="inlineStr">
         <is>
-          <t>This role is a SAS Anti-Money Laundering (AML) Developer position focused on SAS Viya, SAS programming, and compliance systems. It has no connection to Generative AI, LLMs, RAG, or agentic systems, making it an entirely irrelevant fit for a GenAI specialist.</t>
+          <t>This is a non-technical role focusing on market intelligence, trade flows, and supply chain analysis requiring Arabic fluency, which has no overlap with the candidate's core GenAI, LLMs, and agentic AI specialization.</t>
         </is>
       </c>
       <c r="I156" s="3" t="inlineStr">
@@ -10363,7 +10363,7 @@
       </c>
       <c r="M156" s="6" t="inlineStr">
         <is>
-          <t>https://ae.linkedin.com/jobs/view/sas-analyst-at-one75mb-hrm-pvt-ltd-4459306494?position=19&amp;pageNum=0&amp;refId=W92GFmCMxOQHlXfyvp17MQ%3D%3D&amp;trackingId=NfyeO5P7KUMAsO5xQjjwEA%3D%3D</t>
+          <t>https://ae.linkedin.com/jobs/view/senior-analyst-market-intelligence-trade-commodities-at-robert-walters-4457222382?position=30&amp;pageNum=0&amp;refId=W92GFmCMxOQHlXfyvp17MQ%3D%3D&amp;trackingId=JK2lIzdStMxW3Rb1o%2FxSgQ%3D%3D</t>
         </is>
       </c>
     </row>
@@ -10373,12 +10373,12 @@
       </c>
       <c r="B157" s="3" t="inlineStr">
         <is>
-          <t>Finance Information Systems Analyst</t>
+          <t>AI &amp; Data - BrightStar program - Part-Time For Students | UAE Nationals Only - Dubai</t>
         </is>
       </c>
       <c r="C157" s="3" t="inlineStr">
         <is>
-          <t>United Arab Emirates University, Department of Family Medicine</t>
+          <t>Deloitte</t>
         </is>
       </c>
       <c r="D157" s="3" t="inlineStr">
@@ -10401,7 +10401,7 @@
       </c>
       <c r="H157" s="3" t="inlineStr">
         <is>
-          <t>This role is for a Finance Information Systems Analyst focusing on Oracle SQL, financial reporting, and system maintenance, which is completely unrelated to the candidate's core expertise in Generative AI, LLMs, and agentic workflows.</t>
+          <t>This is a student/internship program ('Part-Time For Students') restricted to UAE Nationals only, representing a severe seniority and eligibility mismatch for a Lead Data Scientist with 10 years of experience.</t>
         </is>
       </c>
       <c r="I157" s="3" t="inlineStr">
@@ -10426,7 +10426,7 @@
       </c>
       <c r="M157" s="6" t="inlineStr">
         <is>
-          <t>https://ae.linkedin.com/jobs/view/finance-information-systems-analyst-at-united-arab-emirates-university-department-of-family-medicine-4458309884?position=18&amp;pageNum=0&amp;refId=W92GFmCMxOQHlXfyvp17MQ%3D%3D&amp;trackingId=ZkLRAbbB1OpTP3DQTi%2FB4Q%3D%3D</t>
+          <t>https://ae.linkedin.com/jobs/view/ai-data-brightstar-program-part-time-for-students-uae-nationals-only-dubai-at-deloitte-4459166169?position=29&amp;pageNum=0&amp;refId=W92GFmCMxOQHlXfyvp17MQ%3D%3D&amp;trackingId=eJo5yKx6Zm7GgBBf0abvaA%3D%3D</t>
         </is>
       </c>
     </row>
@@ -10436,17 +10436,17 @@
       </c>
       <c r="B158" s="3" t="inlineStr">
         <is>
-          <t>Analyst I - Advisory</t>
+          <t>SAS Analyst</t>
         </is>
       </c>
       <c r="C158" s="3" t="inlineStr">
         <is>
-          <t>Marsh Risk</t>
+          <t>One75mb HRM Pvt Ltd.</t>
         </is>
       </c>
       <c r="D158" s="3" t="inlineStr">
         <is>
-          <t>Abu Dhabi, Abu Dhabi Emirate, United Arab Emirates</t>
+          <t>Abu Dhabi Emirate, United Arab Emirates</t>
         </is>
       </c>
       <c r="E158" s="2" t="inlineStr">
@@ -10464,7 +10464,7 @@
       </c>
       <c r="H158" s="3" t="inlineStr">
         <is>
-          <t>This is a graduate/entry-level risk engineering and data analyst role located in the UAE restricted to UAE Nationals, representing a severe mismatch in both seniority and specialization for a Lead Data Scientist with 10+ years of experience in GenAI.</t>
+          <t>This role is a SAS Anti-Money Laundering (AML) Developer position focused on SAS Viya, SAS programming, and compliance systems. It has no connection to Generative AI, LLMs, RAG, or agentic systems, making it an entirely irrelevant fit for a GenAI specialist.</t>
         </is>
       </c>
       <c r="I158" s="3" t="inlineStr">
@@ -10489,7 +10489,7 @@
       </c>
       <c r="M158" s="6" t="inlineStr">
         <is>
-          <t>https://ae.linkedin.com/jobs/view/analyst-i-advisory-at-marsh-risk-4459170127?position=6&amp;pageNum=0&amp;refId=W92GFmCMxOQHlXfyvp17MQ%3D%3D&amp;trackingId=hO0QLO%2FIAeXdRsG2PtQkTA%3D%3D</t>
+          <t>https://ae.linkedin.com/jobs/view/sas-analyst-at-one75mb-hrm-pvt-ltd-4459306494?position=19&amp;pageNum=0&amp;refId=W92GFmCMxOQHlXfyvp17MQ%3D%3D&amp;trackingId=NfyeO5P7KUMAsO5xQjjwEA%3D%3D</t>
         </is>
       </c>
     </row>
@@ -10499,12 +10499,12 @@
       </c>
       <c r="B159" s="3" t="inlineStr">
         <is>
-          <t>Senior Economist / Economic Researcher</t>
+          <t>Finance Information Systems Analyst</t>
         </is>
       </c>
       <c r="C159" s="3" t="inlineStr">
         <is>
-          <t>Robert Walters</t>
+          <t>United Arab Emirates University, Department of Family Medicine</t>
         </is>
       </c>
       <c r="D159" s="3" t="inlineStr">
@@ -10527,7 +10527,7 @@
       </c>
       <c r="H159" s="3" t="inlineStr">
         <is>
-          <t>This role is for a Senior Economist focusing on macroeconomic research, policy analysis, and economic forecasting, which is completely unrelated to the candidate's specialization in Generative AI, LLMs, and data science.</t>
+          <t>This role is for a Finance Information Systems Analyst focusing on Oracle SQL, financial reporting, and system maintenance, which is completely unrelated to the candidate's core expertise in Generative AI, LLMs, and agentic workflows.</t>
         </is>
       </c>
       <c r="I159" s="3" t="inlineStr">
@@ -10552,7 +10552,7 @@
       </c>
       <c r="M159" s="6" t="inlineStr">
         <is>
-          <t>https://ae.linkedin.com/jobs/view/senior-economist-economic-researcher-at-robert-walters-4457234594?position=21&amp;pageNum=0&amp;refId=W92GFmCMxOQHlXfyvp17MQ%3D%3D&amp;trackingId=hNkG3K%2BgFb1grR8QDMiBxA%3D%3D</t>
+          <t>https://ae.linkedin.com/jobs/view/finance-information-systems-analyst-at-united-arab-emirates-university-department-of-family-medicine-4458309884?position=18&amp;pageNum=0&amp;refId=W92GFmCMxOQHlXfyvp17MQ%3D%3D&amp;trackingId=ZkLRAbbB1OpTP3DQTi%2FB4Q%3D%3D</t>
         </is>
       </c>
     </row>
@@ -10562,22 +10562,22 @@
       </c>
       <c r="B160" s="3" t="inlineStr">
         <is>
-          <t>Data Engineer</t>
+          <t>Analyst I - Advisory</t>
         </is>
       </c>
       <c r="C160" s="3" t="inlineStr">
         <is>
-          <t>ChipSoft Nederland</t>
+          <t>Marsh Risk</t>
         </is>
       </c>
       <c r="D160" s="3" t="inlineStr">
         <is>
-          <t>Amsterdam, North Holland, Netherlands</t>
+          <t>Abu Dhabi, Abu Dhabi Emirate, United Arab Emirates</t>
         </is>
       </c>
       <c r="E160" s="2" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-08-26</t>
         </is>
       </c>
       <c r="F160" s="7" t="n">
@@ -10590,7 +10590,7 @@
       </c>
       <c r="H160" s="3" t="inlineStr">
         <is>
-          <t>This is a Data Engineer role focused on ELT, SQL, data warehousing, and clickstream data, which is entirely unrelated to the candidate's core specialization in Generative AI, LLMs, and agentic systems.</t>
+          <t>This is a graduate/entry-level risk engineering and data analyst role located in the UAE restricted to UAE Nationals, representing a severe mismatch in both seniority and specialization for a Lead Data Scientist with 10+ years of experience in GenAI.</t>
         </is>
       </c>
       <c r="I160" s="3" t="inlineStr">
@@ -10615,7 +10615,7 @@
       </c>
       <c r="M160" s="6" t="inlineStr">
         <is>
-          <t>https://nl.linkedin.com/jobs/view/data-engineer-at-chipsoft-nederland-4448895866?position=29&amp;pageNum=0&amp;refId=oiBIn1Czflg0JjZjH5z0Lg%3D%3D&amp;trackingId=CakhxR8nCpksAoEXyMZPHQ%3D%3D</t>
+          <t>https://ae.linkedin.com/jobs/view/analyst-i-advisory-at-marsh-risk-4459170127?position=6&amp;pageNum=0&amp;refId=W92GFmCMxOQHlXfyvp17MQ%3D%3D&amp;trackingId=hO0QLO%2FIAeXdRsG2PtQkTA%3D%3D</t>
         </is>
       </c>
     </row>
@@ -10625,22 +10625,22 @@
       </c>
       <c r="B161" s="3" t="inlineStr">
         <is>
-          <t>Quantitative Developer - Pricing Data</t>
+          <t>Senior Economist / Economic Researcher</t>
         </is>
       </c>
       <c r="C161" s="3" t="inlineStr">
         <is>
-          <t>Optiver</t>
+          <t>Robert Walters</t>
         </is>
       </c>
       <c r="D161" s="3" t="inlineStr">
         <is>
-          <t>Amsterdam, North Holland, Netherlands</t>
+          <t>Abu Dhabi, Abu Dhabi Emirate, United Arab Emirates</t>
         </is>
       </c>
       <c r="E161" s="2" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-08-26</t>
         </is>
       </c>
       <c r="F161" s="7" t="n">
@@ -10653,7 +10653,7 @@
       </c>
       <c r="H161" s="3" t="inlineStr">
         <is>
-          <t>This Quantitative Developer role focuses entirely on financial pricing data systems, market data pipelines, and low-latency/historical trading infrastructure in C++/Python, which is completely unrelated to the candidate's specialization in Generative AI, LLMs, and agentic workflows.</t>
+          <t>This role is for a Senior Economist focusing on macroeconomic research, policy analysis, and economic forecasting, which is completely unrelated to the candidate's specialization in Generative AI, LLMs, and data science.</t>
         </is>
       </c>
       <c r="I161" s="3" t="inlineStr">
@@ -10663,7 +10663,7 @@
       </c>
       <c r="J161" s="3" t="inlineStr">
         <is>
-          <t>Yes - explicitly stated in JD</t>
+          <t>Not stated in JD</t>
         </is>
       </c>
       <c r="K161" s="2" t="inlineStr">
@@ -10678,7 +10678,7 @@
       </c>
       <c r="M161" s="6" t="inlineStr">
         <is>
-          <t>https://nl.linkedin.com/jobs/view/quantitative-developer-pricing-data-at-optiver-4437686371?position=21&amp;pageNum=0&amp;refId=oiBIn1Czflg0JjZjH5z0Lg%3D%3D&amp;trackingId=bm7u%2BG7QRNRgNoiTgqdkzg%3D%3D</t>
+          <t>https://ae.linkedin.com/jobs/view/senior-economist-economic-researcher-at-robert-walters-4457234594?position=21&amp;pageNum=0&amp;refId=W92GFmCMxOQHlXfyvp17MQ%3D%3D&amp;trackingId=hNkG3K%2BgFb1grR8QDMiBxA%3D%3D</t>
         </is>
       </c>
     </row>
@@ -10688,17 +10688,17 @@
       </c>
       <c r="B162" s="3" t="inlineStr">
         <is>
-          <t>Data Analyst — Operational Analysis (Python, Power BI, Modelling) for NATO with security clearance</t>
+          <t>Data Engineer</t>
         </is>
       </c>
       <c r="C162" s="3" t="inlineStr">
         <is>
-          <t>WLG</t>
+          <t>ChipSoft Nederland</t>
         </is>
       </c>
       <c r="D162" s="3" t="inlineStr">
         <is>
-          <t>The Hague, South Holland, Netherlands</t>
+          <t>Amsterdam, North Holland, Netherlands</t>
         </is>
       </c>
       <c r="E162" s="2" t="inlineStr">
@@ -10716,7 +10716,7 @@
       </c>
       <c r="H162" s="3" t="inlineStr">
         <is>
-          <t>This is an unrelated junior Data Analyst role focused on operational analysis, dashboards, and spreadsheets rather than Generative AI or advanced data science. Given the candidate's 10+ years of experience as a Lead Data Scientist specializing in LLMs and agentic AI, this position represents a severe mismatch in both domain and seniority.</t>
+          <t>This is a Data Engineer role focused on ELT, SQL, data warehousing, and clickstream data, which is entirely unrelated to the candidate's core specialization in Generative AI, LLMs, and agentic systems.</t>
         </is>
       </c>
       <c r="I162" s="3" t="inlineStr">
@@ -10741,7 +10741,7 @@
       </c>
       <c r="M162" s="6" t="inlineStr">
         <is>
-          <t>https://nl.linkedin.com/jobs/view/data-analyst-%E2%80%94-operational-analysis-python-power-bi-modelling-for-nato-with-security-clearance-at-wlg-4458620413?position=26&amp;pageNum=0&amp;refId=oiBIn1Czflg0JjZjH5z0Lg%3D%3D&amp;trackingId=NK7DxxVQL3iwGI1saGNrZg%3D%3D</t>
+          <t>https://nl.linkedin.com/jobs/view/data-engineer-at-chipsoft-nederland-4448895866?position=29&amp;pageNum=0&amp;refId=oiBIn1Czflg0JjZjH5z0Lg%3D%3D&amp;trackingId=CakhxR8nCpksAoEXyMZPHQ%3D%3D</t>
         </is>
       </c>
     </row>
@@ -10751,17 +10751,17 @@
       </c>
       <c r="B163" s="3" t="inlineStr">
         <is>
-          <t>Hadoop / Big Data Engineer</t>
+          <t>Quantitative Developer - Pricing Data</t>
         </is>
       </c>
       <c r="C163" s="3" t="inlineStr">
         <is>
-          <t>HTC Global Services</t>
+          <t>Optiver</t>
         </is>
       </c>
       <c r="D163" s="3" t="inlineStr">
         <is>
-          <t>Dubai, United Arab Emirates</t>
+          <t>Amsterdam, North Holland, Netherlands</t>
         </is>
       </c>
       <c r="E163" s="2" t="inlineStr">
@@ -10779,7 +10779,7 @@
       </c>
       <c r="H163" s="3" t="inlineStr">
         <is>
-          <t>This is a classical data engineering and Hadoop role focusing on infrastructure, Spark, Hive, and data pipelines, which is entirely unrelated to the candidate's core specialization in Generative AI, LLMs, and agentic workflows.</t>
+          <t>This Quantitative Developer role focuses entirely on financial pricing data systems, market data pipelines, and low-latency/historical trading infrastructure in C++/Python, which is completely unrelated to the candidate's specialization in Generative AI, LLMs, and agentic workflows.</t>
         </is>
       </c>
       <c r="I163" s="3" t="inlineStr">
@@ -10789,7 +10789,7 @@
       </c>
       <c r="J163" s="3" t="inlineStr">
         <is>
-          <t>Not stated in JD</t>
+          <t>Yes - explicitly stated in JD</t>
         </is>
       </c>
       <c r="K163" s="2" t="inlineStr">
@@ -10804,7 +10804,7 @@
       </c>
       <c r="M163" s="6" t="inlineStr">
         <is>
-          <t>https://ae.linkedin.com/jobs/view/hadoop-big-data-engineer-at-htc-global-services-4460123484?position=9&amp;pageNum=0&amp;refId=zJBbvwb5H0wsbJ5fs9ZTVw%3D%3D&amp;trackingId=SQM7VXeym81F4YKdSlXxkg%3D%3D</t>
+          <t>https://nl.linkedin.com/jobs/view/quantitative-developer-pricing-data-at-optiver-4437686371?position=21&amp;pageNum=0&amp;refId=oiBIn1Czflg0JjZjH5z0Lg%3D%3D&amp;trackingId=bm7u%2BG7QRNRgNoiTgqdkzg%3D%3D</t>
         </is>
       </c>
     </row>
@@ -10814,22 +10814,22 @@
       </c>
       <c r="B164" s="3" t="inlineStr">
         <is>
-          <t>Business Analyst - Dubai (UAE Nationals only)</t>
+          <t>Data Analyst — Operational Analysis (Python, Power BI, Modelling) for NATO with security clearance</t>
         </is>
       </c>
       <c r="C164" s="3" t="inlineStr">
         <is>
-          <t>Efficio</t>
+          <t>WLG</t>
         </is>
       </c>
       <c r="D164" s="3" t="inlineStr">
         <is>
-          <t>Dubai, Dubai, United Arab Emirates</t>
+          <t>The Hague, South Holland, Netherlands</t>
         </is>
       </c>
       <c r="E164" s="2" t="inlineStr">
         <is>
-          <t>2026-08-28</t>
+          <t>2026-08-27</t>
         </is>
       </c>
       <c r="F164" s="7" t="n">
@@ -10842,7 +10842,7 @@
       </c>
       <c r="H164" s="3" t="inlineStr">
         <is>
-          <t>This role is a Business Analyst position focused on procurement and supply chain consulting, completely unrelated to data science, artificial intelligence, or the candidate's core GenAI/LLM specialization. Furthermore, the role explicitly requires being a UAE National.</t>
+          <t>This is an unrelated junior Data Analyst role focused on operational analysis, dashboards, and spreadsheets rather than Generative AI or advanced data science. Given the candidate's 10+ years of experience as a Lead Data Scientist specializing in LLMs and agentic AI, this position represents a severe mismatch in both domain and seniority.</t>
         </is>
       </c>
       <c r="I164" s="3" t="inlineStr">
@@ -10867,7 +10867,7 @@
       </c>
       <c r="M164" s="6" t="inlineStr">
         <is>
-          <t>https://ae.linkedin.com/jobs/view/business-analyst-dubai-uae-nationals-only-at-efficio-4291615037?position=11&amp;pageNum=0&amp;refId=umynRMWB8laV9lcrAC5yvg%3D%3D&amp;trackingId=97gwiNAcH3ASkR2fVgtg7A%3D%3D</t>
+          <t>https://nl.linkedin.com/jobs/view/data-analyst-%E2%80%94-operational-analysis-python-power-bi-modelling-for-nato-with-security-clearance-at-wlg-4458620413?position=26&amp;pageNum=0&amp;refId=oiBIn1Czflg0JjZjH5z0Lg%3D%3D&amp;trackingId=NK7DxxVQL3iwGI1saGNrZg%3D%3D</t>
         </is>
       </c>
     </row>
@@ -10877,22 +10877,22 @@
       </c>
       <c r="B165" s="3" t="inlineStr">
         <is>
-          <t>Oliver Wyman - Government and Public Institutions (GPI) and Financial Services (FS) Researcher - Dubai</t>
+          <t>Hadoop / Big Data Engineer</t>
         </is>
       </c>
       <c r="C165" s="3" t="inlineStr">
         <is>
-          <t>Oliver Wyman</t>
+          <t>HTC Global Services</t>
         </is>
       </c>
       <c r="D165" s="3" t="inlineStr">
         <is>
-          <t>Dubai, Dubai, United Arab Emirates</t>
+          <t>Dubai, United Arab Emirates</t>
         </is>
       </c>
       <c r="E165" s="2" t="inlineStr">
         <is>
-          <t>2026-08-28</t>
+          <t>2026-08-27</t>
         </is>
       </c>
       <c r="F165" s="7" t="n">
@@ -10905,7 +10905,7 @@
       </c>
       <c r="H165" s="3" t="inlineStr">
         <is>
-          <t>This is a non-technical management consulting research role focusing on market data, databases like Factiva, and slide preparation in Excel/PowerPoint. It has no connection to the candidate's core specialization in Generative AI, LLMs, LangChain, or data science modeling.</t>
+          <t>This is a classical data engineering and Hadoop role focusing on infrastructure, Spark, Hive, and data pipelines, which is entirely unrelated to the candidate's core specialization in Generative AI, LLMs, and agentic workflows.</t>
         </is>
       </c>
       <c r="I165" s="3" t="inlineStr">
@@ -10930,7 +10930,7 @@
       </c>
       <c r="M165" s="6" t="inlineStr">
         <is>
-          <t>https://ae.linkedin.com/jobs/view/oliver-wyman-government-and-public-institutions-gpi-and-financial-services-fs-researcher-dubai-at-oliver-wyman-4460354191?position=14&amp;pageNum=0&amp;refId=umynRMWB8laV9lcrAC5yvg%3D%3D&amp;trackingId=ELxpmziWW%2B8sDM8xGhxmOA%3D%3D</t>
+          <t>https://ae.linkedin.com/jobs/view/hadoop-big-data-engineer-at-htc-global-services-4460123484?position=9&amp;pageNum=0&amp;refId=zJBbvwb5H0wsbJ5fs9ZTVw%3D%3D&amp;trackingId=SQM7VXeym81F4YKdSlXxkg%3D%3D</t>
         </is>
       </c>
     </row>
@@ -10940,12 +10940,12 @@
       </c>
       <c r="B166" s="3" t="inlineStr">
         <is>
-          <t>Oliver Wyman - Associate - Health and Life Sciences - Dubai</t>
+          <t>Business Analyst - Dubai (UAE Nationals only)</t>
         </is>
       </c>
       <c r="C166" s="3" t="inlineStr">
         <is>
-          <t>Oliver Wyman</t>
+          <t>Efficio</t>
         </is>
       </c>
       <c r="D166" s="3" t="inlineStr">
@@ -10968,7 +10968,7 @@
       </c>
       <c r="H166" s="3" t="inlineStr">
         <is>
-          <t>This is a management consulting role focused on Health and Life Sciences strategy at Oliver Wyman, requiring deep industry expertise in pharmaceuticals or MedTech and top-tier strategy consulting experience. It has zero alignment with the candidate's core GenAI, LLM, or Data Science specialization.</t>
+          <t>This role is a Business Analyst position focused on procurement and supply chain consulting, completely unrelated to data science, artificial intelligence, or the candidate's core GenAI/LLM specialization. Furthermore, the role explicitly requires being a UAE National.</t>
         </is>
       </c>
       <c r="I166" s="3" t="inlineStr">
@@ -10993,7 +10993,7 @@
       </c>
       <c r="M166" s="6" t="inlineStr">
         <is>
-          <t>https://ae.linkedin.com/jobs/view/oliver-wyman-associate-health-and-life-sciences-dubai-at-oliver-wyman-4460351294?position=8&amp;pageNum=0&amp;refId=umynRMWB8laV9lcrAC5yvg%3D%3D&amp;trackingId=GWJpOuiL92AZx2SkHg%2FfPg%3D%3D</t>
+          <t>https://ae.linkedin.com/jobs/view/business-analyst-dubai-uae-nationals-only-at-efficio-4291615037?position=11&amp;pageNum=0&amp;refId=umynRMWB8laV9lcrAC5yvg%3D%3D&amp;trackingId=97gwiNAcH3ASkR2fVgtg7A%3D%3D</t>
         </is>
       </c>
     </row>
@@ -11003,12 +11003,12 @@
       </c>
       <c r="B167" s="3" t="inlineStr">
         <is>
-          <t>F&amp;S Associate - UAE National</t>
+          <t>Oliver Wyman - Government and Public Institutions (GPI) and Financial Services (FS) Researcher - Dubai</t>
         </is>
       </c>
       <c r="C167" s="3" t="inlineStr">
         <is>
-          <t>Deliveroo</t>
+          <t>Oliver Wyman</t>
         </is>
       </c>
       <c r="D167" s="3" t="inlineStr">
@@ -11031,7 +11031,7 @@
       </c>
       <c r="H167" s="3" t="inlineStr">
         <is>
-          <t>This is a finance and strategy role focused on spreadsheets, variance analysis, and business reporting with no relation to Generative AI, machine learning, or data science. It is completely unrelated to the candidate's core technical specialization and profile.</t>
+          <t>This is a non-technical management consulting research role focusing on market data, databases like Factiva, and slide preparation in Excel/PowerPoint. It has no connection to the candidate's core specialization in Generative AI, LLMs, LangChain, or data science modeling.</t>
         </is>
       </c>
       <c r="I167" s="3" t="inlineStr">
@@ -11056,7 +11056,7 @@
       </c>
       <c r="M167" s="6" t="inlineStr">
         <is>
-          <t>https://ae.linkedin.com/jobs/view/f-s-associate-uae-national-at-deliveroo-4449749711?position=6&amp;pageNum=0&amp;refId=umynRMWB8laV9lcrAC5yvg%3D%3D&amp;trackingId=xir3IHLZTYXuoIlF3oUkeg%3D%3D</t>
+          <t>https://ae.linkedin.com/jobs/view/oliver-wyman-government-and-public-institutions-gpi-and-financial-services-fs-researcher-dubai-at-oliver-wyman-4460354191?position=14&amp;pageNum=0&amp;refId=umynRMWB8laV9lcrAC5yvg%3D%3D&amp;trackingId=ELxpmziWW%2B8sDM8xGhxmOA%3D%3D</t>
         </is>
       </c>
     </row>
@@ -11066,12 +11066,12 @@
       </c>
       <c r="B168" s="3" t="inlineStr">
         <is>
-          <t>BI Engineer</t>
+          <t>Oliver Wyman - Associate - Health and Life Sciences - Dubai</t>
         </is>
       </c>
       <c r="C168" s="3" t="inlineStr">
         <is>
-          <t>JD.COM</t>
+          <t>Oliver Wyman</t>
         </is>
       </c>
       <c r="D168" s="3" t="inlineStr">
@@ -11081,7 +11081,7 @@
       </c>
       <c r="E168" s="2" t="inlineStr">
         <is>
-          <t>2026-08-29</t>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="F168" s="7" t="n">
@@ -11094,12 +11094,12 @@
       </c>
       <c r="H168" s="3" t="inlineStr">
         <is>
-          <t>This role is a BI Engineer position focused on supply chain, logistics, and retail operations rather than data science, AI, or Generative AI. It is entirely unrelated to the candidate's core expertise in LLMs, RAG, and agentic systems.</t>
+          <t>This is a management consulting role focused on Health and Life Sciences strategy at Oliver Wyman, requiring deep industry expertise in pharmaceuticals or MedTech and top-tier strategy consulting experience. It has zero alignment with the candidate's core GenAI, LLM, or Data Science specialization.</t>
         </is>
       </c>
       <c r="I168" s="3" t="inlineStr">
         <is>
-          <t>Yes - German required (see JD for exact level)</t>
+          <t>Not stated in JD</t>
         </is>
       </c>
       <c r="J168" s="3" t="inlineStr">
@@ -11107,9 +11107,9 @@
           <t>Not stated in JD</t>
         </is>
       </c>
-      <c r="K168" s="9" t="inlineStr">
-        <is>
-          <t>New this run (2026-08-29 13:17 UTC)</t>
+      <c r="K168" s="2" t="inlineStr">
+        <is>
+          <t>From previous run</t>
         </is>
       </c>
       <c r="L168" s="2" t="inlineStr">
@@ -11119,7 +11119,7 @@
       </c>
       <c r="M168" s="6" t="inlineStr">
         <is>
-          <t>https://ae.linkedin.com/jobs/view/bi-engineer-at-jd-com-4414670937?position=6&amp;pageNum=0&amp;refId=WT017Qp%2F1VFpbzjZb903BA%3D%3D&amp;trackingId=uXRSjK39jDOlXpbtHq2yzQ%3D%3D</t>
+          <t>https://ae.linkedin.com/jobs/view/oliver-wyman-associate-health-and-life-sciences-dubai-at-oliver-wyman-4460351294?position=8&amp;pageNum=0&amp;refId=umynRMWB8laV9lcrAC5yvg%3D%3D&amp;trackingId=GWJpOuiL92AZx2SkHg%2FfPg%3D%3D</t>
         </is>
       </c>
     </row>
@@ -11129,22 +11129,22 @@
       </c>
       <c r="B169" s="3" t="inlineStr">
         <is>
-          <t>Power BI Developer</t>
+          <t>F&amp;S Associate - UAE National</t>
         </is>
       </c>
       <c r="C169" s="3" t="inlineStr">
         <is>
-          <t>Danube Group</t>
+          <t>Deliveroo</t>
         </is>
       </c>
       <c r="D169" s="3" t="inlineStr">
         <is>
-          <t>Dubai, United Arab Emirates</t>
+          <t>Dubai, Dubai, United Arab Emirates</t>
         </is>
       </c>
       <c r="E169" s="2" t="inlineStr">
         <is>
-          <t>2026-08-29</t>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="F169" s="7" t="n">
@@ -11157,7 +11157,7 @@
       </c>
       <c r="H169" s="3" t="inlineStr">
         <is>
-          <t>This is a Power BI Developer role focused on dashboards, data visualization, DAX, and SQL, which is completely unrelated to the candidate's core specialization in Generative AI, LLMs, and agentic workflows.</t>
+          <t>This is a finance and strategy role focused on spreadsheets, variance analysis, and business reporting with no relation to Generative AI, machine learning, or data science. It is completely unrelated to the candidate's core technical specialization and profile.</t>
         </is>
       </c>
       <c r="I169" s="3" t="inlineStr">
@@ -11170,9 +11170,9 @@
           <t>Not stated in JD</t>
         </is>
       </c>
-      <c r="K169" s="9" t="inlineStr">
-        <is>
-          <t>New this run (2026-08-29 13:17 UTC)</t>
+      <c r="K169" s="2" t="inlineStr">
+        <is>
+          <t>From previous run</t>
         </is>
       </c>
       <c r="L169" s="2" t="inlineStr">
@@ -11182,7 +11182,7 @@
       </c>
       <c r="M169" s="6" t="inlineStr">
         <is>
-          <t>https://ae.linkedin.com/jobs/view/power-bi-developer-at-danube-group-4459465901?position=5&amp;pageNum=0&amp;refId=WT017Qp%2F1VFpbzjZb903BA%3D%3D&amp;trackingId=2u7KtmoSLaInXvl%2FCAGPzw%3D%3D</t>
+          <t>https://ae.linkedin.com/jobs/view/f-s-associate-uae-national-at-deliveroo-4449749711?position=6&amp;pageNum=0&amp;refId=umynRMWB8laV9lcrAC5yvg%3D%3D&amp;trackingId=xir3IHLZTYXuoIlF3oUkeg%3D%3D</t>
         </is>
       </c>
     </row>
@@ -11192,12 +11192,12 @@
       </c>
       <c r="B170" s="3" t="inlineStr">
         <is>
-          <t>National Assistant Planner</t>
+          <t>BI Engineer</t>
         </is>
       </c>
       <c r="C170" s="3" t="inlineStr">
         <is>
-          <t>Al-Futtaim</t>
+          <t>JD.COM</t>
         </is>
       </c>
       <c r="D170" s="3" t="inlineStr">
@@ -11207,11 +11207,11 @@
       </c>
       <c r="E170" s="2" t="inlineStr">
         <is>
-          <t>2026-08-26</t>
+          <t>2026-08-29</t>
         </is>
       </c>
       <c r="F170" s="7" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="G170" s="8" t="inlineStr">
         <is>
@@ -11220,12 +11220,12 @@
       </c>
       <c r="H170" s="3" t="inlineStr">
         <is>
-          <t>This is a non-technical retail merchandise planning role focused on financial forecasting, inventory management, and sales planning, which is entirely unrelated to the candidate's GenAI, LLM, and data science specialization.</t>
+          <t>This role is a BI Engineer position focused on supply chain, logistics, and retail operations rather than data science, AI, or Generative AI. It is entirely unrelated to the candidate's core expertise in LLMs, RAG, and agentic systems.</t>
         </is>
       </c>
       <c r="I170" s="3" t="inlineStr">
         <is>
-          <t>Not stated in JD</t>
+          <t>Yes - German required (see JD for exact level)</t>
         </is>
       </c>
       <c r="J170" s="3" t="inlineStr">
@@ -11245,7 +11245,7 @@
       </c>
       <c r="M170" s="6" t="inlineStr">
         <is>
-          <t>https://ae.linkedin.com/jobs/view/national-assistant-planner-at-al-futtaim-4459335643?position=23&amp;pageNum=0&amp;refId=JBPPMgbgbAFzpV%2BDL5h2AA%3D%3D&amp;trackingId=udE1OmanEOJo5NqnDVVmsw%3D%3D</t>
+          <t>https://ae.linkedin.com/jobs/view/bi-engineer-at-jd-com-4414670937?position=6&amp;pageNum=0&amp;refId=WT017Qp%2F1VFpbzjZb903BA%3D%3D&amp;trackingId=uXRSjK39jDOlXpbtHq2yzQ%3D%3D</t>
         </is>
       </c>
     </row>
@@ -11255,26 +11255,26 @@
       </c>
       <c r="B171" s="3" t="inlineStr">
         <is>
-          <t>Forward Deployed AI Integrator (UAE National Only), Field Engineering</t>
+          <t>Power BI Developer</t>
         </is>
       </c>
       <c r="C171" s="3" t="inlineStr">
         <is>
-          <t>Amazon Web Services (AWS)</t>
+          <t>Danube Group</t>
         </is>
       </c>
       <c r="D171" s="3" t="inlineStr">
         <is>
-          <t>Dubai, Dubai, United Arab Emirates</t>
+          <t>Dubai, United Arab Emirates</t>
         </is>
       </c>
       <c r="E171" s="2" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-08-29</t>
         </is>
       </c>
       <c r="F171" s="7" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="G171" s="8" t="inlineStr">
         <is>
@@ -11283,7 +11283,7 @@
       </c>
       <c r="H171" s="3" t="inlineStr">
         <is>
-          <t>Although the role involves AI tooling and Python, it is restricted to UAE Nationals only, making it impossible for the candidate to qualify. Additionally, the position leans heavily toward technical program management rather than hands-on Generative AI and LLM engineering.</t>
+          <t>This is a Power BI Developer role focused on dashboards, data visualization, DAX, and SQL, which is completely unrelated to the candidate's core specialization in Generative AI, LLMs, and agentic workflows.</t>
         </is>
       </c>
       <c r="I171" s="3" t="inlineStr">
@@ -11308,7 +11308,7 @@
       </c>
       <c r="M171" s="6" t="inlineStr">
         <is>
-          <t>https://ae.linkedin.com/jobs/view/forward-deployed-ai-integrator-uae-national-only-field-engineering-at-amazon-web-services-aws-4459616402?position=14&amp;pageNum=0&amp;refId=JBPPMgbgbAFzpV%2BDL5h2AA%3D%3D&amp;trackingId=suYy8hgZkG37o3lG7FlDHQ%3D%3D</t>
+          <t>https://ae.linkedin.com/jobs/view/power-bi-developer-at-danube-group-4459465901?position=5&amp;pageNum=0&amp;refId=WT017Qp%2F1VFpbzjZb903BA%3D%3D&amp;trackingId=2u7KtmoSLaInXvl%2FCAGPzw%3D%3D</t>
         </is>
       </c>
     </row>
@@ -11318,12 +11318,12 @@
       </c>
       <c r="B172" s="3" t="inlineStr">
         <is>
-          <t>GIS Specialist / Developer</t>
+          <t>National Assistant Planner</t>
         </is>
       </c>
       <c r="C172" s="3" t="inlineStr">
         <is>
-          <t>AECOM</t>
+          <t>Al-Futtaim</t>
         </is>
       </c>
       <c r="D172" s="3" t="inlineStr">
@@ -11346,7 +11346,7 @@
       </c>
       <c r="H172" s="3" t="inlineStr">
         <is>
-          <t>This is a GIS Specialist role focused on ArcGIS Enterprise administration, spatial analysis, and Python/ArcPy automation, which is completely unrelated to the candidate's core specialization in Generative AI, LLMs, and agentic systems.</t>
+          <t>This is a non-technical retail merchandise planning role focused on financial forecasting, inventory management, and sales planning, which is entirely unrelated to the candidate's GenAI, LLM, and data science specialization.</t>
         </is>
       </c>
       <c r="I172" s="3" t="inlineStr">
@@ -11371,7 +11371,7 @@
       </c>
       <c r="M172" s="6" t="inlineStr">
         <is>
-          <t>https://ae.linkedin.com/jobs/view/gis-specialist-developer-at-aecom-4456869023?position=15&amp;pageNum=0&amp;refId=JBPPMgbgbAFzpV%2BDL5h2AA%3D%3D&amp;trackingId=lGxG6%2FYECt2YwYGWf5hEZA%3D%3D</t>
+          <t>https://ae.linkedin.com/jobs/view/national-assistant-planner-at-al-futtaim-4459335643?position=23&amp;pageNum=0&amp;refId=JBPPMgbgbAFzpV%2BDL5h2AA%3D%3D&amp;trackingId=udE1OmanEOJo5NqnDVVmsw%3D%3D</t>
         </is>
       </c>
     </row>
@@ -11381,12 +11381,12 @@
       </c>
       <c r="B173" s="3" t="inlineStr">
         <is>
-          <t>Quant Desk Lead and Portfolio Manager</t>
+          <t>Forward Deployed AI Integrator (UAE National Only), Field Engineering</t>
         </is>
       </c>
       <c r="C173" s="3" t="inlineStr">
         <is>
-          <t>EMCD</t>
+          <t>Amazon Web Services (AWS)</t>
         </is>
       </c>
       <c r="D173" s="3" t="inlineStr">
@@ -11396,7 +11396,7 @@
       </c>
       <c r="E173" s="2" t="inlineStr">
         <is>
-          <t>2026-08-26</t>
+          <t>2026-08-27</t>
         </is>
       </c>
       <c r="F173" s="7" t="n">
@@ -11409,7 +11409,7 @@
       </c>
       <c r="H173" s="3" t="inlineStr">
         <is>
-          <t>This is a finance and quantitative trading role focused on running a systematic trading desk, portfolio management, and P&amp;L ownership, which is entirely unrelated to the candidate's core specialization in Generative AI, LLMs, and agentic systems.</t>
+          <t>Although the role involves AI tooling and Python, it is restricted to UAE Nationals only, making it impossible for the candidate to qualify. Additionally, the position leans heavily toward technical program management rather than hands-on Generative AI and LLM engineering.</t>
         </is>
       </c>
       <c r="I173" s="3" t="inlineStr">
@@ -11434,7 +11434,7 @@
       </c>
       <c r="M173" s="6" t="inlineStr">
         <is>
-          <t>https://ae.linkedin.com/jobs/view/quant-desk-lead-and-portfolio-manager-at-emcd-4457949555?position=13&amp;pageNum=0&amp;refId=JBPPMgbgbAFzpV%2BDL5h2AA%3D%3D&amp;trackingId=drHtrw6uBtEz5S2i%2BjBT5A%3D%3D</t>
+          <t>https://ae.linkedin.com/jobs/view/forward-deployed-ai-integrator-uae-national-only-field-engineering-at-amazon-web-services-aws-4459616402?position=14&amp;pageNum=0&amp;refId=JBPPMgbgbAFzpV%2BDL5h2AA%3D%3D&amp;trackingId=suYy8hgZkG37o3lG7FlDHQ%3D%3D</t>
         </is>
       </c>
     </row>
@@ -11444,17 +11444,17 @@
       </c>
       <c r="B174" s="3" t="inlineStr">
         <is>
-          <t>Join Norlys Energy Trading</t>
+          <t>GIS Specialist / Developer</t>
         </is>
       </c>
       <c r="C174" s="3" t="inlineStr">
         <is>
-          <t>Norlys Energy Trading A/S</t>
+          <t>AECOM</t>
         </is>
       </c>
       <c r="D174" s="3" t="inlineStr">
         <is>
-          <t>Aalborg, North Denmark Region, Denmark</t>
+          <t>Dubai, Dubai, United Arab Emirates</t>
         </is>
       </c>
       <c r="E174" s="2" t="inlineStr">
@@ -11472,7 +11472,7 @@
       </c>
       <c r="H174" s="3" t="inlineStr">
         <is>
-          <t>This is an open, unsolicited job application for a general talent pool in energy trading, rather than a defined Data Science or Generative AI role. It completely lacks technical specifications, making it impossible to evaluate against the candidate's specialized GenAI and LLM expertise.</t>
+          <t>This is a GIS Specialist role focused on ArcGIS Enterprise administration, spatial analysis, and Python/ArcPy automation, which is completely unrelated to the candidate's core specialization in Generative AI, LLMs, and agentic systems.</t>
         </is>
       </c>
       <c r="I174" s="3" t="inlineStr">
@@ -11497,7 +11497,7 @@
       </c>
       <c r="M174" s="6" t="inlineStr">
         <is>
-          <t>https://dk.linkedin.com/jobs/view/join-norlys-energy-trading-at-norlys-energy-trading-a-s-4459158084?position=26&amp;pageNum=0&amp;refId=Pb2EWWHgR9a7i9BrLIIg7g%3D%3D&amp;trackingId=Z%2BOuDrbPap3omWro18MA2g%3D%3D</t>
+          <t>https://ae.linkedin.com/jobs/view/gis-specialist-developer-at-aecom-4456869023?position=15&amp;pageNum=0&amp;refId=JBPPMgbgbAFzpV%2BDL5h2AA%3D%3D&amp;trackingId=lGxG6%2FYECt2YwYGWf5hEZA%3D%3D</t>
         </is>
       </c>
     </row>
@@ -11507,17 +11507,17 @@
       </c>
       <c r="B175" s="3" t="inlineStr">
         <is>
-          <t>PhD scholarship in Modeling and Control of Parkinson’s Disease - DTU Electro</t>
+          <t>Quant Desk Lead and Portfolio Manager</t>
         </is>
       </c>
       <c r="C175" s="3" t="inlineStr">
         <is>
-          <t>DTU - Technical University of Denmark</t>
+          <t>EMCD</t>
         </is>
       </c>
       <c r="D175" s="3" t="inlineStr">
         <is>
-          <t>Kongens Lyngby, Capital Region of Denmark, Denmark</t>
+          <t>Dubai, Dubai, United Arab Emirates</t>
         </is>
       </c>
       <c r="E175" s="2" t="inlineStr">
@@ -11535,7 +11535,7 @@
       </c>
       <c r="H175" s="3" t="inlineStr">
         <is>
-          <t>This is a PhD scholarship position in neuroengineering, control systems, and healthcare technology at DTU, which is completely unrelated to the candidate's specialization in Generative AI, LLMs, and agentic systems.</t>
+          <t>This is a finance and quantitative trading role focused on running a systematic trading desk, portfolio management, and P&amp;L ownership, which is entirely unrelated to the candidate's core specialization in Generative AI, LLMs, and agentic systems.</t>
         </is>
       </c>
       <c r="I175" s="3" t="inlineStr">
@@ -11545,7 +11545,7 @@
       </c>
       <c r="J175" s="3" t="inlineStr">
         <is>
-          <t>Possible - relocation support mentioned, visa not explicit</t>
+          <t>Not stated in JD</t>
         </is>
       </c>
       <c r="K175" s="2" t="inlineStr">
@@ -11560,7 +11560,7 @@
       </c>
       <c r="M175" s="6" t="inlineStr">
         <is>
-          <t>https://dk.linkedin.com/jobs/view/phd-scholarship-in-modeling-and-control-of-parkinson%E2%80%99s-disease-dtu-electro-at-dtu-technical-university-of-denmark-4459145557?position=20&amp;pageNum=0&amp;refId=Pb2EWWHgR9a7i9BrLIIg7g%3D%3D&amp;trackingId=mStwcLkWBAvzmreGSwO4Hw%3D%3D</t>
+          <t>https://ae.linkedin.com/jobs/view/quant-desk-lead-and-portfolio-manager-at-emcd-4457949555?position=13&amp;pageNum=0&amp;refId=JBPPMgbgbAFzpV%2BDL5h2AA%3D%3D&amp;trackingId=drHtrw6uBtEz5S2i%2BjBT5A%3D%3D</t>
         </is>
       </c>
     </row>
@@ -11570,17 +11570,17 @@
       </c>
       <c r="B176" s="3" t="inlineStr">
         <is>
-          <t>Analytikere med flair for databehandling til PET's kontraspionageindsats mod Rusland</t>
+          <t>Join Norlys Energy Trading</t>
         </is>
       </c>
       <c r="C176" s="3" t="inlineStr">
         <is>
-          <t>Politi</t>
+          <t>Norlys Energy Trading A/S</t>
         </is>
       </c>
       <c r="D176" s="3" t="inlineStr">
         <is>
-          <t>Copenhagen, Capital Region of Denmark, Denmark</t>
+          <t>Aalborg, North Denmark Region, Denmark</t>
         </is>
       </c>
       <c r="E176" s="2" t="inlineStr">
@@ -11598,7 +11598,7 @@
       </c>
       <c r="H176" s="3" t="inlineStr">
         <is>
-          <t>This is a national security intelligence and counter-espionage analyst role at the Danish Security and Intelligence Service (PET), which is completely unrelated to data science, artificial intelligence, or the candidate's Generative AI and LLM specialization.</t>
+          <t>This is an open, unsolicited job application for a general talent pool in energy trading, rather than a defined Data Science or Generative AI role. It completely lacks technical specifications, making it impossible to evaluate against the candidate's specialized GenAI and LLM expertise.</t>
         </is>
       </c>
       <c r="I176" s="3" t="inlineStr">
@@ -11623,7 +11623,7 @@
       </c>
       <c r="M176" s="6" t="inlineStr">
         <is>
-          <t>https://dk.linkedin.com/jobs/view/analytikere-med-flair-for-databehandling-til-pet-s-kontraspionageindsats-mod-rusland-at-politi-4457943820?position=18&amp;pageNum=0&amp;refId=Pb2EWWHgR9a7i9BrLIIg7g%3D%3D&amp;trackingId=%2FGEw4KOC0oARqkQIDTGJ4Q%3D%3D</t>
+          <t>https://dk.linkedin.com/jobs/view/join-norlys-energy-trading-at-norlys-energy-trading-a-s-4459158084?position=26&amp;pageNum=0&amp;refId=Pb2EWWHgR9a7i9BrLIIg7g%3D%3D&amp;trackingId=Z%2BOuDrbPap3omWro18MA2g%3D%3D</t>
         </is>
       </c>
     </row>
@@ -11633,17 +11633,17 @@
       </c>
       <c r="B177" s="3" t="inlineStr">
         <is>
-          <t>PostDoc - Uncertainty-Aware Optimization in Inverse Problems for Next-Generation 3D Scanning</t>
+          <t>PhD scholarship in Modeling and Control of Parkinson’s Disease - DTU Electro</t>
         </is>
       </c>
       <c r="C177" s="3" t="inlineStr">
         <is>
-          <t>3Shape</t>
+          <t>DTU - Technical University of Denmark</t>
         </is>
       </c>
       <c r="D177" s="3" t="inlineStr">
         <is>
-          <t>Copenhagen, Capital Region of Denmark, Denmark</t>
+          <t>Kongens Lyngby, Capital Region of Denmark, Denmark</t>
         </is>
       </c>
       <c r="E177" s="2" t="inlineStr">
@@ -11661,7 +11661,7 @@
       </c>
       <c r="H177" s="3" t="inlineStr">
         <is>
-          <t>This is a PostDoc position focused on mathematical optimization, numerical linear algebra, and uncertainty quantification for 3D scanning, which requires a PhD. It has no overlap with the candidate's specialization in GenAI, LLMs, and agentic systems.</t>
+          <t>This is a PhD scholarship position in neuroengineering, control systems, and healthcare technology at DTU, which is completely unrelated to the candidate's specialization in Generative AI, LLMs, and agentic systems.</t>
         </is>
       </c>
       <c r="I177" s="3" t="inlineStr">
@@ -11671,7 +11671,7 @@
       </c>
       <c r="J177" s="3" t="inlineStr">
         <is>
-          <t>Not stated in JD</t>
+          <t>Possible - relocation support mentioned, visa not explicit</t>
         </is>
       </c>
       <c r="K177" s="2" t="inlineStr">
@@ -11686,7 +11686,7 @@
       </c>
       <c r="M177" s="6" t="inlineStr">
         <is>
-          <t>https://dk.linkedin.com/jobs/view/postdoc-uncertainty-aware-optimization-in-inverse-problems-for-next-generation-3d-scanning-at-3shape-4459171806?position=15&amp;pageNum=0&amp;refId=Pb2EWWHgR9a7i9BrLIIg7g%3D%3D&amp;trackingId=bO0aSGZ%2FUAxThXN9yvOERg%3D%3D</t>
+          <t>https://dk.linkedin.com/jobs/view/phd-scholarship-in-modeling-and-control-of-parkinson%E2%80%99s-disease-dtu-electro-at-dtu-technical-university-of-denmark-4459145557?position=20&amp;pageNum=0&amp;refId=Pb2EWWHgR9a7i9BrLIIg7g%3D%3D&amp;trackingId=mStwcLkWBAvzmreGSwO4Hw%3D%3D</t>
         </is>
       </c>
     </row>
@@ -11696,17 +11696,17 @@
       </c>
       <c r="B178" s="3" t="inlineStr">
         <is>
-          <t>Scientist, Quantitative Clinical Pharmacology (PK/PD Modeling &amp; Simulation)</t>
+          <t>Analytikere med flair for databehandling til PET's kontraspionageindsats mod Rusland</t>
         </is>
       </c>
       <c r="C178" s="3" t="inlineStr">
         <is>
-          <t>Hemab Therapeutics</t>
+          <t>Politi</t>
         </is>
       </c>
       <c r="D178" s="3" t="inlineStr">
         <is>
-          <t>Copenhagen Metropolitan Area</t>
+          <t>Copenhagen, Capital Region of Denmark, Denmark</t>
         </is>
       </c>
       <c r="E178" s="2" t="inlineStr">
@@ -11724,7 +11724,7 @@
       </c>
       <c r="H178" s="3" t="inlineStr">
         <is>
-          <t>This is a highly specialized biomedical role focusing on Pharmacokinetics/Pharmacodynamics (PK/PD) modeling and clinical pharmacology, requiring a Ph.D. and experience with tools like NONMEM or Monolix. It has zero overlap with the candidate's GenAI, LLM, and data science background.</t>
+          <t>This is a national security intelligence and counter-espionage analyst role at the Danish Security and Intelligence Service (PET), which is completely unrelated to data science, artificial intelligence, or the candidate's Generative AI and LLM specialization.</t>
         </is>
       </c>
       <c r="I178" s="3" t="inlineStr">
@@ -11749,7 +11749,7 @@
       </c>
       <c r="M178" s="6" t="inlineStr">
         <is>
-          <t>https://dk.linkedin.com/jobs/view/scientist-quantitative-clinical-pharmacology-pk-pd-modeling-simulation-at-hemab-therapeutics-4457218306?position=14&amp;pageNum=0&amp;refId=Pb2EWWHgR9a7i9BrLIIg7g%3D%3D&amp;trackingId=jhTyKvDAQ70R9PD5s0x2yA%3D%3D</t>
+          <t>https://dk.linkedin.com/jobs/view/analytikere-med-flair-for-databehandling-til-pet-s-kontraspionageindsats-mod-rusland-at-politi-4457943820?position=18&amp;pageNum=0&amp;refId=Pb2EWWHgR9a7i9BrLIIg7g%3D%3D&amp;trackingId=%2FGEw4KOC0oARqkQIDTGJ4Q%3D%3D</t>
         </is>
       </c>
     </row>
@@ -11759,17 +11759,17 @@
       </c>
       <c r="B179" s="3" t="inlineStr">
         <is>
-          <t>Senior Payload Data Operator</t>
+          <t>PostDoc - Uncertainty-Aware Optimization in Inverse Problems for Next-Generation 3D Scanning</t>
         </is>
       </c>
       <c r="C179" s="3" t="inlineStr">
         <is>
-          <t>FADA</t>
+          <t>3Shape</t>
         </is>
       </c>
       <c r="D179" s="3" t="inlineStr">
         <is>
-          <t>United Arab Emirates</t>
+          <t>Copenhagen, Capital Region of Denmark, Denmark</t>
         </is>
       </c>
       <c r="E179" s="2" t="inlineStr">
@@ -11787,7 +11787,7 @@
       </c>
       <c r="H179" s="3" t="inlineStr">
         <is>
-          <t>This is a satellite payload data engineering role focused on aerospace, remote sensing, and image processing (EO/SAR), which is completely unrelated to the candidate's specialization in GenAI, LLMs, and agentic systems.</t>
+          <t>This is a PostDoc position focused on mathematical optimization, numerical linear algebra, and uncertainty quantification for 3D scanning, which requires a PhD. It has no overlap with the candidate's specialization in GenAI, LLMs, and agentic systems.</t>
         </is>
       </c>
       <c r="I179" s="3" t="inlineStr">
@@ -11812,7 +11812,7 @@
       </c>
       <c r="M179" s="6" t="inlineStr">
         <is>
-          <t>https://ae.linkedin.com/jobs/view/senior-payload-data-operator-at-fada-4448986926?position=20&amp;pageNum=0&amp;refId=W92GFmCMxOQHlXfyvp17MQ%3D%3D&amp;trackingId=xdfP2za0I45WGIW%2FRJb%2BgA%3D%3D</t>
+          <t>https://dk.linkedin.com/jobs/view/postdoc-uncertainty-aware-optimization-in-inverse-problems-for-next-generation-3d-scanning-at-3shape-4459171806?position=15&amp;pageNum=0&amp;refId=Pb2EWWHgR9a7i9BrLIIg7g%3D%3D&amp;trackingId=bO0aSGZ%2FUAxThXN9yvOERg%3D%3D</t>
         </is>
       </c>
     </row>
@@ -11822,22 +11822,22 @@
       </c>
       <c r="B180" s="3" t="inlineStr">
         <is>
-          <t>Arabic Speech And Natural Language Processing Specialist</t>
+          <t>Scientist, Quantitative Clinical Pharmacology (PK/PD Modeling &amp; Simulation)</t>
         </is>
       </c>
       <c r="C180" s="3" t="inlineStr">
         <is>
-          <t>Birbal AI</t>
+          <t>Hemab Therapeutics</t>
         </is>
       </c>
       <c r="D180" s="3" t="inlineStr">
         <is>
-          <t>Abu Dhabi Emirate, United Arab Emirates</t>
+          <t>Copenhagen Metropolitan Area</t>
         </is>
       </c>
       <c r="E180" s="2" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-08-26</t>
         </is>
       </c>
       <c r="F180" s="7" t="n">
@@ -11850,7 +11850,7 @@
       </c>
       <c r="H180" s="3" t="inlineStr">
         <is>
-          <t>The role requires specialized expertise in Arabic speech technology (ASR, TTS, audio DSP) and native command of Gulf Arabic dialects, which does not match the candidate's core background in GenAI, LLMs, and RAG for English-language banking and HR use cases.</t>
+          <t>This is a highly specialized biomedical role focusing on Pharmacokinetics/Pharmacodynamics (PK/PD) modeling and clinical pharmacology, requiring a Ph.D. and experience with tools like NONMEM or Monolix. It has zero overlap with the candidate's GenAI, LLM, and data science background.</t>
         </is>
       </c>
       <c r="I180" s="3" t="inlineStr">
@@ -11875,7 +11875,7 @@
       </c>
       <c r="M180" s="6" t="inlineStr">
         <is>
-          <t>https://ae.linkedin.com/jobs/view/arabic-speech-and-natural-language-processing-specialist-at-birbal-ai-4457738899?position=14&amp;pageNum=0&amp;refId=W92GFmCMxOQHlXfyvp17MQ%3D%3D&amp;trackingId=ztG06Ly%2FIZ3fxm%2Fhvl626A%3D%3D</t>
+          <t>https://dk.linkedin.com/jobs/view/scientist-quantitative-clinical-pharmacology-pk-pd-modeling-simulation-at-hemab-therapeutics-4457218306?position=14&amp;pageNum=0&amp;refId=Pb2EWWHgR9a7i9BrLIIg7g%3D%3D&amp;trackingId=jhTyKvDAQ70R9PD5s0x2yA%3D%3D</t>
         </is>
       </c>
     </row>
@@ -11885,12 +11885,12 @@
       </c>
       <c r="B181" s="3" t="inlineStr">
         <is>
-          <t>Member of Technical Staff - Medical Research (Remote)</t>
+          <t>Senior Payload Data Operator</t>
         </is>
       </c>
       <c r="C181" s="3" t="inlineStr">
         <is>
-          <t>Hire Feed</t>
+          <t>FADA</t>
         </is>
       </c>
       <c r="D181" s="3" t="inlineStr">
@@ -11900,7 +11900,7 @@
       </c>
       <c r="E181" s="2" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-08-26</t>
         </is>
       </c>
       <c r="F181" s="7" t="n">
@@ -11913,7 +11913,7 @@
       </c>
       <c r="H181" s="3" t="inlineStr">
         <is>
-          <t>This role is completely unrelated to the candidate's specialization in Generative AI, LLMs, and agentic workflows, focusing instead on medical imaging, computational biology, and clinical research requiring a PhD.</t>
+          <t>This is a satellite payload data engineering role focused on aerospace, remote sensing, and image processing (EO/SAR), which is completely unrelated to the candidate's specialization in GenAI, LLMs, and agentic systems.</t>
         </is>
       </c>
       <c r="I181" s="3" t="inlineStr">
@@ -11938,7 +11938,7 @@
       </c>
       <c r="M181" s="6" t="inlineStr">
         <is>
-          <t>https://ae.linkedin.com/jobs/view/member-of-technical-staff-medical-research-remote-at-hire-feed-4459638503?position=3&amp;pageNum=0&amp;refId=W92GFmCMxOQHlXfyvp17MQ%3D%3D&amp;trackingId=b91zxKPZNgdFnMmW%2FlYbHA%3D%3D</t>
+          <t>https://ae.linkedin.com/jobs/view/senior-payload-data-operator-at-fada-4448986926?position=20&amp;pageNum=0&amp;refId=W92GFmCMxOQHlXfyvp17MQ%3D%3D&amp;trackingId=xdfP2za0I45WGIW%2FRJb%2BgA%3D%3D</t>
         </is>
       </c>
     </row>
@@ -11948,17 +11948,17 @@
       </c>
       <c r="B182" s="3" t="inlineStr">
         <is>
-          <t>AI Image Specialist</t>
+          <t>Arabic Speech And Natural Language Processing Specialist</t>
         </is>
       </c>
       <c r="C182" s="3" t="inlineStr">
         <is>
-          <t>Puffy</t>
+          <t>Birbal AI</t>
         </is>
       </c>
       <c r="D182" s="3" t="inlineStr">
         <is>
-          <t>Dubai, United Arab Emirates</t>
+          <t>Abu Dhabi Emirate, United Arab Emirates</t>
         </is>
       </c>
       <c r="E182" s="2" t="inlineStr">
@@ -11976,7 +11976,7 @@
       </c>
       <c r="H182" s="3" t="inlineStr">
         <is>
-          <t>This is an AI Image Specialist role focused on generative visual design and creative production (Midjourney, DALL-E, image synthesis), which is completely unrelated to the candidate's core specialization in LLMs, RAG, LangChain, and agentic AI pipelines for data science and enterprise applications.</t>
+          <t>The role requires specialized expertise in Arabic speech technology (ASR, TTS, audio DSP) and native command of Gulf Arabic dialects, which does not match the candidate's core background in GenAI, LLMs, and RAG for English-language banking and HR use cases.</t>
         </is>
       </c>
       <c r="I182" s="3" t="inlineStr">
@@ -11986,7 +11986,7 @@
       </c>
       <c r="J182" s="3" t="inlineStr">
         <is>
-          <t>Yes - explicitly stated in JD</t>
+          <t>Not stated in JD</t>
         </is>
       </c>
       <c r="K182" s="2" t="inlineStr">
@@ -12001,7 +12001,7 @@
       </c>
       <c r="M182" s="6" t="inlineStr">
         <is>
-          <t>https://ae.linkedin.com/jobs/view/ai-image-specialist-at-puffy-4457756193?position=10&amp;pageNum=0&amp;refId=50H6yCrEXIuhgr6eqEojNg%3D%3D&amp;trackingId=9EIvgvUNu%2BE37717JffiJA%3D%3D</t>
+          <t>https://ae.linkedin.com/jobs/view/arabic-speech-and-natural-language-processing-specialist-at-birbal-ai-4457738899?position=14&amp;pageNum=0&amp;refId=W92GFmCMxOQHlXfyvp17MQ%3D%3D&amp;trackingId=ztG06Ly%2FIZ3fxm%2Fhvl626A%3D%3D</t>
         </is>
       </c>
     </row>
@@ -12011,22 +12011,22 @@
       </c>
       <c r="B183" s="3" t="inlineStr">
         <is>
-          <t>Market Operations &amp; Analytics Specialist — Institutional</t>
+          <t>Member of Technical Staff - Medical Research (Remote)</t>
         </is>
       </c>
       <c r="C183" s="3" t="inlineStr">
         <is>
-          <t>Confidential</t>
+          <t>Hire Feed</t>
         </is>
       </c>
       <c r="D183" s="3" t="inlineStr">
         <is>
-          <t>Dubai, United Arab Emirates</t>
+          <t>United Arab Emirates</t>
         </is>
       </c>
       <c r="E183" s="2" t="inlineStr">
         <is>
-          <t>2026-08-28</t>
+          <t>2026-08-27</t>
         </is>
       </c>
       <c r="F183" s="7" t="n">
@@ -12039,7 +12039,7 @@
       </c>
       <c r="H183" s="3" t="inlineStr">
         <is>
-          <t>This role is completely unrelated to data science, artificial intelligence, LLMs, or generative AI, focusing entirely on cryptocurrency exchange operations, institutional client management, and trading analytics instead.</t>
+          <t>This role is completely unrelated to the candidate's specialization in Generative AI, LLMs, and agentic workflows, focusing instead on medical imaging, computational biology, and clinical research requiring a PhD.</t>
         </is>
       </c>
       <c r="I183" s="3" t="inlineStr">
@@ -12064,7 +12064,7 @@
       </c>
       <c r="M183" s="6" t="inlineStr">
         <is>
-          <t>https://ae.linkedin.com/jobs/view/market-operations-analytics-specialist-%E2%80%94-institutional-at-confidential-4453037100?position=10&amp;pageNum=0&amp;refId=zJBbvwb5H0wsbJ5fs9ZTVw%3D%3D&amp;trackingId=ENnWCvoEQXOg1fXKuxlBug%3D%3D</t>
+          <t>https://ae.linkedin.com/jobs/view/member-of-technical-staff-medical-research-remote-at-hire-feed-4459638503?position=3&amp;pageNum=0&amp;refId=W92GFmCMxOQHlXfyvp17MQ%3D%3D&amp;trackingId=b91zxKPZNgdFnMmW%2FlYbHA%3D%3D</t>
         </is>
       </c>
     </row>
@@ -12074,17 +12074,17 @@
       </c>
       <c r="B184" s="3" t="inlineStr">
         <is>
-          <t>Quantitative Developer, Systematic Equities</t>
+          <t>AI Image Specialist</t>
         </is>
       </c>
       <c r="C184" s="3" t="inlineStr">
         <is>
-          <t>Millennium</t>
+          <t>Puffy</t>
         </is>
       </c>
       <c r="D184" s="3" t="inlineStr">
         <is>
-          <t>Dubai, Dubai, United Arab Emirates</t>
+          <t>Dubai, United Arab Emirates</t>
         </is>
       </c>
       <c r="E184" s="2" t="inlineStr">
@@ -12102,7 +12102,7 @@
       </c>
       <c r="H184" s="3" t="inlineStr">
         <is>
-          <t>This role is a quantitative software engineering position focused on low-latency trading infrastructure, C++/C# development, and execution systems for a hedge fund, which is entirely unrelated to the candidate's specialization in GenAI, LLMs, and agentic architectures.</t>
+          <t>This is an AI Image Specialist role focused on generative visual design and creative production (Midjourney, DALL-E, image synthesis), which is completely unrelated to the candidate's core specialization in LLMs, RAG, LangChain, and agentic AI pipelines for data science and enterprise applications.</t>
         </is>
       </c>
       <c r="I184" s="3" t="inlineStr">
@@ -12112,7 +12112,7 @@
       </c>
       <c r="J184" s="3" t="inlineStr">
         <is>
-          <t>Not stated in JD</t>
+          <t>Yes - explicitly stated in JD</t>
         </is>
       </c>
       <c r="K184" s="2" t="inlineStr">
@@ -12127,7 +12127,7 @@
       </c>
       <c r="M184" s="6" t="inlineStr">
         <is>
-          <t>https://ae.linkedin.com/jobs/view/quantitative-developer-systematic-equities-at-millennium-4290849018?position=6&amp;pageNum=0&amp;refId=zJBbvwb5H0wsbJ5fs9ZTVw%3D%3D&amp;trackingId=8TTWkyG2j%2F7MELtLSQ5VCA%3D%3D</t>
+          <t>https://ae.linkedin.com/jobs/view/ai-image-specialist-at-puffy-4457756193?position=10&amp;pageNum=0&amp;refId=50H6yCrEXIuhgr6eqEojNg%3D%3D&amp;trackingId=9EIvgvUNu%2BE37717JffiJA%3D%3D</t>
         </is>
       </c>
     </row>
@@ -12137,17 +12137,17 @@
       </c>
       <c r="B185" s="3" t="inlineStr">
         <is>
-          <t>Senior Specialist - Portfolio Management</t>
+          <t>Market Operations &amp; Analytics Specialist — Institutional</t>
         </is>
       </c>
       <c r="C185" s="3" t="inlineStr">
         <is>
-          <t>MENA Careers</t>
+          <t>Confidential</t>
         </is>
       </c>
       <c r="D185" s="3" t="inlineStr">
         <is>
-          <t>Dubai, Dubai, United Arab Emirates</t>
+          <t>Dubai, United Arab Emirates</t>
         </is>
       </c>
       <c r="E185" s="2" t="inlineStr">
@@ -12165,7 +12165,7 @@
       </c>
       <c r="H185" s="3" t="inlineStr">
         <is>
-          <t>This is a non-AI banking role focused on portfolio management, loan optimization, and regulatory capital compliance in Dubai requiring UAE nationality, which completely misaligns with the candidate's GenAI, LLM, and data science specialization.</t>
+          <t>This role is completely unrelated to data science, artificial intelligence, LLMs, or generative AI, focusing entirely on cryptocurrency exchange operations, institutional client management, and trading analytics instead.</t>
         </is>
       </c>
       <c r="I185" s="3" t="inlineStr">
@@ -12190,7 +12190,7 @@
       </c>
       <c r="M185" s="6" t="inlineStr">
         <is>
-          <t>https://ae.linkedin.com/jobs/view/senior-specialist-portfolio-management-at-mena-careers-4458066015?position=12&amp;pageNum=0&amp;refId=umynRMWB8laV9lcrAC5yvg%3D%3D&amp;trackingId=kbnf5IoX2jxOWD9%2Fe1UaKg%3D%3D</t>
+          <t>https://ae.linkedin.com/jobs/view/market-operations-analytics-specialist-%E2%80%94-institutional-at-confidential-4453037100?position=10&amp;pageNum=0&amp;refId=zJBbvwb5H0wsbJ5fs9ZTVw%3D%3D&amp;trackingId=ENnWCvoEQXOg1fXKuxlBug%3D%3D</t>
         </is>
       </c>
     </row>
@@ -12200,12 +12200,12 @@
       </c>
       <c r="B186" s="3" t="inlineStr">
         <is>
-          <t>Manager Logistics Performance</t>
+          <t>Quantitative Developer, Systematic Equities</t>
         </is>
       </c>
       <c r="C186" s="3" t="inlineStr">
         <is>
-          <t>talabat</t>
+          <t>Millennium</t>
         </is>
       </c>
       <c r="D186" s="3" t="inlineStr">
@@ -12215,7 +12215,7 @@
       </c>
       <c r="E186" s="2" t="inlineStr">
         <is>
-          <t>2026-08-28</t>
+          <t>2026-08-27</t>
         </is>
       </c>
       <c r="F186" s="7" t="n">
@@ -12228,12 +12228,12 @@
       </c>
       <c r="H186" s="3" t="inlineStr">
         <is>
-          <t>This is a commercial operations, logistics, and P&amp;L management role completely unrelated to data science, artificial intelligence, or Large Language Models. It requires background in marketplace operations, logistics, or quick-commerce rather than GenAI engineering.</t>
+          <t>This role is a quantitative software engineering position focused on low-latency trading infrastructure, C++/C# development, and execution systems for a hedge fund, which is entirely unrelated to the candidate's specialization in GenAI, LLMs, and agentic architectures.</t>
         </is>
       </c>
       <c r="I186" s="3" t="inlineStr">
         <is>
-          <t>Yes - German required (see JD for exact level)</t>
+          <t>Not stated in JD</t>
         </is>
       </c>
       <c r="J186" s="3" t="inlineStr">
@@ -12253,7 +12253,7 @@
       </c>
       <c r="M186" s="6" t="inlineStr">
         <is>
-          <t>https://ae.linkedin.com/jobs/view/manager-logistics-performance-at-talabat-4440740657?position=7&amp;pageNum=0&amp;refId=umynRMWB8laV9lcrAC5yvg%3D%3D&amp;trackingId=lMQWp6LAUNLwXpGhMCpl2Q%3D%3D</t>
+          <t>https://ae.linkedin.com/jobs/view/quantitative-developer-systematic-equities-at-millennium-4290849018?position=6&amp;pageNum=0&amp;refId=zJBbvwb5H0wsbJ5fs9ZTVw%3D%3D&amp;trackingId=8TTWkyG2j%2F7MELtLSQ5VCA%3D%3D</t>
         </is>
       </c>
     </row>
@@ -12263,17 +12263,17 @@
       </c>
       <c r="B187" s="3" t="inlineStr">
         <is>
-          <t>Perception Engineer</t>
+          <t>Senior Specialist - Portfolio Management</t>
         </is>
       </c>
       <c r="C187" s="3" t="inlineStr">
         <is>
-          <t>Careernet</t>
+          <t>MENA Careers</t>
         </is>
       </c>
       <c r="D187" s="3" t="inlineStr">
         <is>
-          <t>Ajman, Ajman Emirate, United Arab Emirates</t>
+          <t>Dubai, Dubai, United Arab Emirates</t>
         </is>
       </c>
       <c r="E187" s="2" t="inlineStr">
@@ -12291,93 +12291,219 @@
       </c>
       <c r="H187" s="3" t="inlineStr">
         <is>
+          <t>This is a non-AI banking role focused on portfolio management, loan optimization, and regulatory capital compliance in Dubai requiring UAE nationality, which completely misaligns with the candidate's GenAI, LLM, and data science specialization.</t>
+        </is>
+      </c>
+      <c r="I187" s="3" t="inlineStr">
+        <is>
+          <t>Not stated in JD</t>
+        </is>
+      </c>
+      <c r="J187" s="3" t="inlineStr">
+        <is>
+          <t>Not stated in JD</t>
+        </is>
+      </c>
+      <c r="K187" s="2" t="inlineStr">
+        <is>
+          <t>From previous run</t>
+        </is>
+      </c>
+      <c r="L187" s="2" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="M187" s="6" t="inlineStr">
+        <is>
+          <t>https://ae.linkedin.com/jobs/view/senior-specialist-portfolio-management-at-mena-careers-4458066015?position=12&amp;pageNum=0&amp;refId=umynRMWB8laV9lcrAC5yvg%3D%3D&amp;trackingId=kbnf5IoX2jxOWD9%2Fe1UaKg%3D%3D</t>
+        </is>
+      </c>
+    </row>
+    <row r="188" ht="55" customHeight="1">
+      <c r="A188" s="2" t="n">
+        <v>187</v>
+      </c>
+      <c r="B188" s="3" t="inlineStr">
+        <is>
+          <t>Manager Logistics Performance</t>
+        </is>
+      </c>
+      <c r="C188" s="3" t="inlineStr">
+        <is>
+          <t>talabat</t>
+        </is>
+      </c>
+      <c r="D188" s="3" t="inlineStr">
+        <is>
+          <t>Dubai, Dubai, United Arab Emirates</t>
+        </is>
+      </c>
+      <c r="E188" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="F188" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="G188" s="8" t="inlineStr">
+        <is>
+          <t>Below threshold</t>
+        </is>
+      </c>
+      <c r="H188" s="3" t="inlineStr">
+        <is>
+          <t>This is a commercial operations, logistics, and P&amp;L management role completely unrelated to data science, artificial intelligence, or Large Language Models. It requires background in marketplace operations, logistics, or quick-commerce rather than GenAI engineering.</t>
+        </is>
+      </c>
+      <c r="I188" s="3" t="inlineStr">
+        <is>
+          <t>Yes - German required (see JD for exact level)</t>
+        </is>
+      </c>
+      <c r="J188" s="3" t="inlineStr">
+        <is>
+          <t>Not stated in JD</t>
+        </is>
+      </c>
+      <c r="K188" s="2" t="inlineStr">
+        <is>
+          <t>From previous run</t>
+        </is>
+      </c>
+      <c r="L188" s="2" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="M188" s="6" t="inlineStr">
+        <is>
+          <t>https://ae.linkedin.com/jobs/view/manager-logistics-performance-at-talabat-4440740657?position=7&amp;pageNum=0&amp;refId=umynRMWB8laV9lcrAC5yvg%3D%3D&amp;trackingId=lMQWp6LAUNLwXpGhMCpl2Q%3D%3D</t>
+        </is>
+      </c>
+    </row>
+    <row r="189" ht="55" customHeight="1">
+      <c r="A189" s="2" t="n">
+        <v>188</v>
+      </c>
+      <c r="B189" s="3" t="inlineStr">
+        <is>
+          <t>Perception Engineer</t>
+        </is>
+      </c>
+      <c r="C189" s="3" t="inlineStr">
+        <is>
+          <t>Careernet</t>
+        </is>
+      </c>
+      <c r="D189" s="3" t="inlineStr">
+        <is>
+          <t>Ajman, Ajman Emirate, United Arab Emirates</t>
+        </is>
+      </c>
+      <c r="E189" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="F189" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="G189" s="8" t="inlineStr">
+        <is>
+          <t>Below threshold</t>
+        </is>
+      </c>
+      <c r="H189" s="3" t="inlineStr">
+        <is>
           <t>This is a hardware-focused Perception Engineer role centering on 2D/3D computer vision, camera calibration, point clouds, and robotics. It is completely unrelated to the candidate's specialization in GenAI, LLMs, RAG, and agentic AI.</t>
         </is>
       </c>
-      <c r="I187" s="3" t="inlineStr">
-        <is>
-          <t>Not stated in JD</t>
-        </is>
-      </c>
-      <c r="J187" s="3" t="inlineStr">
-        <is>
-          <t>Not stated in JD</t>
-        </is>
-      </c>
-      <c r="K187" s="2" t="inlineStr">
-        <is>
-          <t>From previous run</t>
-        </is>
-      </c>
-      <c r="L187" s="2" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="M187" s="6" t="inlineStr">
+      <c r="I189" s="3" t="inlineStr">
+        <is>
+          <t>Not stated in JD</t>
+        </is>
+      </c>
+      <c r="J189" s="3" t="inlineStr">
+        <is>
+          <t>Not stated in JD</t>
+        </is>
+      </c>
+      <c r="K189" s="2" t="inlineStr">
+        <is>
+          <t>From previous run</t>
+        </is>
+      </c>
+      <c r="L189" s="2" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="M189" s="6" t="inlineStr">
         <is>
           <t>https://ae.linkedin.com/jobs/view/perception-engineer-at-careernet-4458403150?position=10&amp;pageNum=0&amp;refId=umynRMWB8laV9lcrAC5yvg%3D%3D&amp;trackingId=8I7i%2FeIdinpIC7lB70K7fg%3D%3D</t>
         </is>
       </c>
     </row>
-    <row r="188" ht="55" customHeight="1">
-      <c r="A188" s="10" t="n">
-        <v>187</v>
-      </c>
-      <c r="B188" s="11" t="inlineStr">
+    <row r="190" ht="55" customHeight="1">
+      <c r="A190" s="10" t="n">
+        <v>189</v>
+      </c>
+      <c r="B190" s="11" t="inlineStr">
         <is>
           <t>Data Scientist</t>
         </is>
       </c>
-      <c r="C188" s="11" t="inlineStr">
+      <c r="C190" s="11" t="inlineStr">
         <is>
           <t>Magno IT Recruitment</t>
         </is>
       </c>
-      <c r="D188" s="11" t="inlineStr">
+      <c r="D190" s="11" t="inlineStr">
         <is>
           <t>Amsterdam, North Holland, Netherlands</t>
         </is>
       </c>
-      <c r="E188" s="10" t="inlineStr">
+      <c r="E190" s="10" t="inlineStr">
         <is>
           <t>2026-08-26</t>
         </is>
       </c>
-      <c r="F188" s="10" t="n">
+      <c r="F190" s="10" t="n">
         <v>92</v>
       </c>
-      <c r="G188" s="12" t="inlineStr">
+      <c r="G190" s="12" t="inlineStr">
         <is>
           <t>APPLY</t>
         </is>
       </c>
-      <c r="H188" s="11" t="inlineStr">
+      <c r="H190" s="11" t="inlineStr">
         <is>
           <t>This Senior AI Engineer role is an exceptional technical match, focusing directly on LLMs, RAG, agentic AI applications, and semantic search which align precisely with the candidate's core specialization. The seniority level (Senior) fits the candidate's 10+ years of experience very well.</t>
         </is>
       </c>
-      <c r="I188" s="11" t="inlineStr">
-        <is>
-          <t>Not stated in JD</t>
-        </is>
-      </c>
-      <c r="J188" s="11" t="inlineStr">
-        <is>
-          <t>Not stated in JD</t>
-        </is>
-      </c>
-      <c r="K188" s="10" t="inlineStr">
-        <is>
-          <t>From previous run</t>
-        </is>
-      </c>
-      <c r="L188" s="10" t="inlineStr">
+      <c r="I190" s="11" t="inlineStr">
+        <is>
+          <t>Not stated in JD</t>
+        </is>
+      </c>
+      <c r="J190" s="11" t="inlineStr">
+        <is>
+          <t>Not stated in JD</t>
+        </is>
+      </c>
+      <c r="K190" s="10" t="inlineStr">
+        <is>
+          <t>From previous run</t>
+        </is>
+      </c>
+      <c r="L190" s="10" t="inlineStr">
         <is>
           <t>Closed</t>
         </is>
       </c>
-      <c r="M188" s="13" t="inlineStr">
+      <c r="M190" s="13" t="inlineStr">
         <is>
           <t>https://nl.linkedin.com/jobs/view/data-scientist-at-magno-it-recruitment-4448992517?position=9&amp;pageNum=0&amp;refId=AM27LUOGtvYOeETm648UMw%3D%3D&amp;trackingId=26%2BZzuSXNPWrglox%2BL4Wqg%3D%3D</t>
         </is>
@@ -12572,6 +12698,8 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M186" r:id="rId185"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M187" r:id="rId186"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M188" r:id="rId187"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M189" r:id="rId188"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M190" r:id="rId189"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>